<commit_message>
Update Round 2 tracker: first replies (Meredith yes; Christa & Kelly elementary; Walter bounced)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -49,7 +49,7 @@
       <color rgb="00666666"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F6FB0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFEFEF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,11 +89,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -460,10 +478,10 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="40" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,41 +552,57 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Aliso Viejo Christian School</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Aliso Viejo</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Meredith Arldt</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>marldt@avchristianschool.org</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>YES — happy to take part</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -830,41 +864,57 @@
       <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Ben Lippen School</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Columbia</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>SC</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Christa Agee</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>christa.agee@benlippen.com</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>No — elementary educator</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr"/>
+      <c r="L10" s="3" t="inlineStr"/>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-10: elementary educator, never taught middle school; declined.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1089,41 +1139,57 @@
       <c r="M16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Bethlehem Christian Academy - Elementary</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Bethlehem</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Kelly Vann</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>kvann@bcamail.org</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>No — works with K3–5th; referral</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr"/>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-10: works with K3-5th, suggested a better-fit contact (cc SJones@bcamail.org).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1225,7 +1291,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AshleyKim@crosspointacademy.org</t>
+          <t>ashleykim@crosspointacademy.org</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
@@ -1262,7 +1328,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CarolynNg@crosspointacademy.org</t>
+          <t>carolynng@crosspointacademy.org</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -1299,7 +1365,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>HelenYooLee@crosspointacademy.org</t>
+          <t>helenyoolee@crosspointacademy.org</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -1336,7 +1402,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>JennyLee@crosspointacademy.org</t>
+          <t>jennylee@crosspointacademy.org</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -1373,7 +1439,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>StephenLim@crosspointacademy.org</t>
+          <t>stephenlim@crosspointacademy.org</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1595,7 +1661,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>EvaK@CCAEagles.org</t>
+          <t>evak@ccaeagles.org</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -1669,7 +1735,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Kathya@ccaeagles.org</t>
+          <t>kathya@ccaeagles.org</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1706,7 +1772,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>LeaC@CCAEagles.org</t>
+          <t>leac@ccaeagles.org</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -3186,7 +3252,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Danielle.Williams@cypresschristian.org</t>
+          <t>danielle.williams@cypresschristian.org</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
@@ -3667,7 +3733,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Cathie.Kelly@eagleslanding.org</t>
+          <t>cathie.kelly@eagleslanding.org</t>
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
@@ -3753,41 +3819,45 @@
       <c r="M88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" t="n">
+      <c r="A89" s="4" t="n">
         <v>88</v>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>Eagle's Landing Christian Academy - Junior High</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="4" t="inlineStr">
         <is>
           <t>McDonough</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D89" s="4" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E89" s="4" t="inlineStr">
         <is>
           <t>Walter Shields</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>Walter.Shields@eagleslanding.org</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>walter.shields@eagleslanding.org</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr"/>
+      <c r="H89" s="4" t="inlineStr"/>
+      <c r="I89" s="4" t="inlineStr"/>
+      <c r="J89" s="4" t="inlineStr"/>
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+      <c r="M89" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: address not found at eagleslanding.org. Needs a corrected address or drop.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -5474,21 +5544,21 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Questions Preview Email (sent to educators who agree, before scheduling)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Subject: The questions ahead of our conversation — DeepRoots Middle School curriculum</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
@@ -5502,7 +5572,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Options: 5-8? / 6-8? / 7-8?</t>
         </is>
@@ -5516,7 +5586,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Options: Developmentally? / Spiritually? / Emotionally?</t>
         </is>
@@ -5558,7 +5628,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
@@ -5572,7 +5642,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Options: Teaching / Reading / Discussion time / Activities</t>
         </is>
@@ -5586,7 +5656,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
         </is>
@@ -5600,7 +5670,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Options: To project images and other teaching materials / To play educational videos / Other</t>
         </is>
@@ -5614,7 +5684,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
         </is>
@@ -5628,7 +5698,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -5649,14 +5719,14 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Options: 6th / 7th / 8th</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
@@ -5677,7 +5747,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Options: 30 seconds -1min / 1 min-2min / 2 min-3min / 3 minutes +</t>
         </is>
@@ -5691,7 +5761,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Options: Photography / Illustrations / Infographics/diagrams / Maps and timelines / Historical artwork / Charts and visual explanations / Short-form comics or graphic storytelling / Other</t>
         </is>
@@ -5712,7 +5782,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>Options: Mostly visual, with short amounts of text / A balanced mix of text and visuals / Mostly text, with visuals used to support key concepts / It depends on the lesson</t>
         </is>
@@ -5740,7 +5810,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>Additional Questions</t>
         </is>
@@ -5761,7 +5831,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -5789,7 +5859,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
         <is>
           <t>Options: In school with boys taught by a male teacher and girls taught by a female teacher, with advance permission from parents / Sent home to parents as a resource to use with their own child as they see fit / We would not use it at our school or send it home to parents.</t>
         </is>
@@ -5803,7 +5873,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -5817,7 +5887,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B51" s="8" t="inlineStr">
         <is>
           <t>Options: Discussions / Alternate in-depth videos / Journaling prompts / Further Bible reading / Other activities</t>
         </is>
@@ -5866,7 +5936,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B58" s="8" t="inlineStr">
         <is>
           <t>Options: Videos that tie the lesson into real world application / Videos that hit on the key idea of the lesson / Videos that introduce the subject matter before teaching</t>
         </is>
@@ -5911,88 +5981,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>DeepRoots — Middle School Curriculum Outreach: Round 2 Response Tracker</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Last updated: 2026-09-10 — 3 replied, 1 said yes, 1 bounced (of 133).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>WHO: 133 additional administrators at the same 51 schools from Round 1 (the 61 already contacted on 2026-09-04 are excluded).</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DRAFTS: All 133 personalized emails were created as drafts in tdwinkler@deeprootsbible.com on 2026-09-10, BCC to Salesforce, ready to send.</t>
+          <t>Green = wants to take part. Grey = replied (declined/referral). Red = bounced address.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EXCLUDED: Lilian Mogle (chskingsmen.org — no longer there) and Mark Persson (chskingsman.org — likely mistyped domain).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>HOW TO USE:</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> - Fill "Date Emailed" as you send each draft.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> - "Responded?" = Yes/No; add the date and whether they want to take part.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> - "Questions Sent?" = Yes once you send the questions-preview email (see Questions Email tab).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> - "Meeting Date/Time" once scheduled.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>MONITORING: Claude checks the Gmail account daily for replies from these 133 addresses and updates the "Responded?" columns.</t>
+          <t>Fill Date Emailed as you send; Questions Sent once you send the preview email (Questions Email tab).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flag 11 bounced addresses in Round 2 tracker
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,9 +38,6 @@
       <sz val="12"/>
     </font>
     <font>
-      <i val="1"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="001F6FB0"/>
     </font>
@@ -49,7 +46,7 @@
       <color rgb="00666666"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +73,11 @@
         <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -97,10 +99,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -481,7 +483,7 @@
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="64" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -580,7 +582,11 @@
           <t>marldt@avchristianschool.org</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -892,7 +898,11 @@
           <t>christa.agee@benlippen.com</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1065,78 +1075,94 @@
       <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Bethlehem Christian Academy - Elementary</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Bethlehem</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Chris Holland</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>cholland@bcamail.org</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: address not found at bcamail.org.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Bethlehem Christian Academy - Elementary</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Bethlehem</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Jen Prior</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>jprior@bcamail.org</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: address not found at bcamail.org.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1167,7 +1193,11 @@
           <t>kvann@bcamail.org</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2191,41 +2221,49 @@
       <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>Charlotte Christian School</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Charlotte</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
         <is>
           <t>NC</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>Jen Payne</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>jen.payne@charchrist.com</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="inlineStr"/>
-      <c r="M45" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr"/>
+      <c r="K45" s="4" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr"/>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: address not found (550 5.2.1).</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2265,41 +2303,49 @@
       <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Christian Academy of Indiana</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>New Albany</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>Krystal Morrow</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>kmorrow@caschools.us</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr"/>
+      <c r="K47" s="4" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr"/>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: rejected by caschools.us mail gateway (Paubox).</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2524,78 +2570,94 @@
       <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="n">
+      <c r="A54" s="4" t="n">
         <v>53</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>Christian Academy of Louisville - English Station Campus</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Louisville</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>KY</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="4" t="inlineStr">
         <is>
           <t>Jennifer Rehnberg</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>jrehnberg@caschools.us</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
-      <c r="L54" t="inlineStr"/>
-      <c r="M54" t="inlineStr"/>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr"/>
+      <c r="I54" s="4" t="inlineStr"/>
+      <c r="J54" s="4" t="inlineStr"/>
+      <c r="K54" s="4" t="inlineStr"/>
+      <c r="L54" s="4" t="inlineStr"/>
+      <c r="M54" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: rejected by caschools.us mail gateway (Paubox).</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" t="n">
+      <c r="A55" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Christian Academy of Louisville - English Station Campus</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Louisville</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>KY</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>Jennifer Watson</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>jwatson@caschools.us</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
-      <c r="L55" t="inlineStr"/>
-      <c r="M55" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr"/>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="inlineStr"/>
+      <c r="K55" s="4" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr"/>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: rejected by caschools.us mail gateway (Paubox).</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3671,152 +3733,180 @@
       <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" t="n">
+      <c r="A85" s="4" t="n">
         <v>84</v>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B85" s="4" t="inlineStr">
         <is>
           <t>Eagle's Landing Christian Academy - Junior High</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="4" t="inlineStr">
         <is>
           <t>McDonough</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" s="4" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E85" s="4" t="inlineStr">
         <is>
           <t>Andy Whitlock</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="F85" s="4" t="inlineStr">
         <is>
           <t>andy.whitlock@eagleslanding.org</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr"/>
+      <c r="I85" s="4" t="inlineStr"/>
+      <c r="J85" s="4" t="inlineStr"/>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+      <c r="M85" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: message blocked / not found at eagleslanding.org.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" t="n">
+      <c r="A86" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B86" s="5" t="inlineStr">
         <is>
           <t>Eagle's Landing Christian Academy - Junior High</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>McDonough</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" s="5" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E86" s="5" t="inlineStr">
         <is>
           <t>Cathie Kelly</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="F86" s="5" t="inlineStr">
         <is>
           <t>cathie.kelly@eagleslanding.org</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
+      <c r="G86" s="5" t="inlineStr"/>
+      <c r="H86" s="5" t="inlineStr"/>
+      <c r="I86" s="5" t="inlineStr"/>
+      <c r="J86" s="5" t="inlineStr"/>
+      <c r="K86" s="5" t="inlineStr"/>
+      <c r="L86" s="5" t="inlineStr"/>
+      <c r="M86" s="5" t="inlineStr">
+        <is>
+          <t>CAUTION: all other eagleslanding.org addresses bounced 2026-09-10; likely invalid.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" t="n">
+      <c r="A87" s="4" t="n">
         <v>86</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="4" t="inlineStr">
         <is>
           <t>Eagle's Landing Christian Academy - Junior High</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="4" t="inlineStr">
         <is>
           <t>McDonough</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" s="4" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E87" s="4" t="inlineStr">
         <is>
           <t>Douglas Campbell, Jr</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="F87" s="4" t="inlineStr">
         <is>
           <t>douglas.campbell@eagleslanding.org</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr"/>
+      <c r="J87" s="4" t="inlineStr"/>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+      <c r="M87" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: message blocked / not found at eagleslanding.org.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" t="n">
+      <c r="A88" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B88" s="4" t="inlineStr">
         <is>
           <t>Eagle's Landing Christian Academy - Junior High</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>McDonough</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" s="4" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="E88" s="4" t="inlineStr">
         <is>
           <t>Ivey Davis</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="F88" s="4" t="inlineStr">
         <is>
           <t>ivey.davis@eagleslanding.org</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr"/>
+      <c r="I88" s="4" t="inlineStr"/>
+      <c r="J88" s="4" t="inlineStr"/>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
+      <c r="M88" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: message blocked / not found at eagleslanding.org.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
@@ -3847,7 +3937,11 @@
           <t>walter.shields@eagleslanding.org</t>
         </is>
       </c>
-      <c r="G89" s="4" t="inlineStr"/>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
       <c r="H89" s="4" t="inlineStr"/>
       <c r="I89" s="4" t="inlineStr"/>
       <c r="J89" s="4" t="inlineStr"/>
@@ -3855,7 +3949,7 @@
       <c r="L89" s="4" t="inlineStr"/>
       <c r="M89" s="4" t="inlineStr">
         <is>
-          <t>BOUNCED 2026-09-10: address not found at eagleslanding.org. Needs a corrected address or drop.</t>
+          <t>BOUNCED 2026-09-10: recipient unknown at eagleslanding.org.</t>
         </is>
       </c>
     </row>
@@ -4193,41 +4287,49 @@
       <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" t="n">
+      <c r="A99" s="4" t="n">
         <v>98</v>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B99" s="4" t="inlineStr">
         <is>
           <t>Fellowship Christian School</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="4" t="inlineStr">
         <is>
           <t>Roswell</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D99" s="4" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr">
+      <c r="E99" s="4" t="inlineStr">
         <is>
           <t>Gina Tomberlin</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr">
+      <c r="F99" s="4" t="inlineStr">
         <is>
           <t>gina.tomberlin@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
-      <c r="H99" t="inlineStr"/>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr"/>
+      <c r="I99" s="4" t="inlineStr"/>
+      <c r="J99" s="4" t="inlineStr"/>
+      <c r="K99" s="4" t="inlineStr"/>
+      <c r="L99" s="4" t="inlineStr"/>
+      <c r="M99" s="4" t="inlineStr">
+        <is>
+          <t>BOUNCED 2026-09-10: message blocked by recipient server.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -5536,7 +5638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B62"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -5544,427 +5646,420 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Questions Preview Email (sent to educators who agree, before scheduling)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Subject: The questions ahead of our conversation — DeepRoots Middle School curriculum</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Questions Preview Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>Marketing &amp; Sales</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1. How does your school categorize Middle School or Junior High…</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1. How does your school categorize Middle School or Junior High…</t>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Options: 5-8? / 6-8? / 7-8?</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Options: 5-8? / 6-8? / 7-8?</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2. What are the primary differences between a 6th, 7th, and 8th grade student…</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2. What are the primary differences between a 6th, 7th, and 8th grade student…</t>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Options: Developmentally? / Spiritually? / Emotionally?</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Options: Developmentally? / Spiritually? / Emotionally?</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>3. How do you find it best to reach both churched and unchurched students in your class? Is this an issue for you? What have you seen work best?</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3. How do you find it best to reach both churched and unchurched students in your class? Is this an issue for you? What have you seen work best?</t>
+          <t>4. What do you like or dislike about what you are currently using for your Bible curriculum?</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4. What do you like or dislike about what you are currently using for your Bible curriculum?</t>
+          <t>5. What elements would you like to see in it each week?</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5. What elements would you like to see in it each week?</t>
+          <t>6. What are the core ideals that you wish each of your students left your class identifying with?</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6. What are the core ideals that you wish each of your students left your class identifying with?</t>
+          <t>7. What types of resources (videos, activities, etc.) are the most helpful for you as a teacher?</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>7. What types of resources (videos, activities, etc.) are the most helpful for you as a teacher?</t>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Editorial</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Editorial</t>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8. How many minutes can your students pay attention to the following?</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>8. How many minutes can your students pay attention to the following?</t>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Options: Teaching / Reading / Discussion time / Activities</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Options: Teaching / Reading / Discussion time / Activities</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9. What kind of engagements do your students enjoy the most…</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>9. What kind of engagements do your students enjoy the most…</t>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="8" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>10. How do you use screens and technology in your classroom?</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Options: To project images and other teaching materials / To play educational videos / Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>11. What questions/issues do you see your students wrestling with…</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>10. How do you use screens and technology in your classroom?</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Options: To project images and other teaching materials / To play educational videos / Other</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>11. What questions/issues do you see your students wrestling with…</t>
-        </is>
-      </c>
-    </row>
     <row r="22">
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>12. Would you use an end-of the-year project students prepare as a group?</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>12. Would you use an end-of the-year project students prepare as a group?</t>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Options: Yes / No / Maybe</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Options: Yes / No / Maybe</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>13. What tools have helped with parent engagement?</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>13. What tools have helped with parent engagement?</t>
+          <t>14. What is your school’s policy on homework?</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>14. What is your school’s policy on homework?</t>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Options: 6th / 7th / 8th</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Options: 6th / 7th / 8th</t>
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Production</t>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>15. What videos do you currently show in class? How do you currently use those videos in your classroom to support your teaching?</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>15. What videos do you currently show in class? How do you currently use those videos in your classroom to support your teaching?</t>
+          <t>16. What length of videos is most engaging for your students?</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>16. What length of videos is most engaging for your students?</t>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Options: 30 seconds -1min / 1 min-2min / 2 min-3min / 3 minutes +</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="8" t="inlineStr">
-        <is>
-          <t>Options: 30 seconds -1min / 1 min-2min / 2 min-3min / 3 minutes +</t>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>17. What types of visuals do you think are most effective at engaging Middle School students?</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>17. What types of visuals do you think are most effective at engaging Middle School students?</t>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Options: Photography / Illustrations / Infographics/diagrams / Maps and timelines / Historical artwork / Charts and visual explanations / Short-form comics or graphic storytelling / Other</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>Options: Photography / Illustrations / Infographics/diagrams / Maps and timelines / Historical artwork / Charts and visual explanations / Short-form comics or graphic storytelling / Other</t>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>18. Do you prefer digital assessments or printables?</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>18. Do you prefer digital assessments or printables?</t>
+          <t>19. What balance would you prefer between text and visuals on a typical student page?</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>19. What balance would you prefer between text and visuals on a typical student page?</t>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Options: Mostly visual, with short amounts of text / A balanced mix of text and visuals / Mostly text, with visuals used to support key concepts / It depends on the lesson</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>Options: Mostly visual, with short amounts of text / A balanced mix of text and visuals / Mostly text, with visuals used to support key concepts / It depends on the lesson</t>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>20. What would make a Middle School student want to pick up a curriculum book or open a digital lesson rather than seeing it as “just another textbook”?</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>20. What would make a Middle School student want to pick up a curriculum book or open a digital lesson rather than seeing it as “just another textbook”?</t>
+          <t>21. Are you limited by the amount of material you are allowed to print?</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>21. Are you limited by the amount of material you are allowed to print?</t>
+          <t>22. If an activity required supplies not typically found in the classroom, for example food items, would your school provide the funds or would you, as the teacher, have to provide supplemental materials?</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>22. If an activity required supplies not typically found in the classroom, for example food items, would your school provide the funds or would you, as the teacher, have to provide supplemental materials?</t>
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Additional Questions</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>Additional Questions</t>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>23. After 20 minutes of essential material, how much additional time would you like the optional material to fill?</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>23. After 20 minutes of essential material, how much additional time would you like the optional material to fill?</t>
+          <t>24. Would you be interested in a multi-subject Timeline that focused on Bible events but allowed you to choose to display other subjects, such as Empires, Literature, Music and Arts, People, Scientific Inventions, etc. which would allow you and students to click to read a short summary and access images, music, etc.?</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>24. Would you be interested in a multi-subject Timeline that focused on Bible events but allowed you to choose to display other subjects, such as Empires, Literature, Music and Arts, People, Scientific Inventions, etc. which would allow you and students to click to read a short summary and access images, music, etc.?</t>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Options: Yes / No / Maybe</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="8" t="inlineStr">
-        <is>
-          <t>Options: Yes / No / Maybe</t>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>25. Approximately how many minutes of screen time and technology would you permit in Bible class?</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>25. Approximately how many minutes of screen time and technology would you permit in Bible class?</t>
+          <t>26. What tools have you found most effective for encouraging Bible reading at home?</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>26. What tools have you found most effective for encouraging Bible reading at home?</t>
+          <t>27. If the DeepRoots Middle School curriculum offered an optional human sexuality Unit about what God’s Word says about identity, behavior, and purity, how would you use it?</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>27. If the DeepRoots Middle School curriculum offered an optional human sexuality Unit about what God’s Word says about identity, behavior, and purity, how would you use it?</t>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>Options: In school with boys taught by a male teacher and girls taught by a female teacher, with advance permission from parents / Sent home to parents as a resource to use with their own child as they see fit / We would not use it at our school or send it home to parents.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>Options: In school with boys taught by a male teacher and girls taught by a female teacher, with advance permission from parents / Sent home to parents as a resource to use with their own child as they see fit / We would not use it at our school or send it home to parents.</t>
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>28. Would you be interested in a separate Logic course, primarily taught through videos, and reinforced with worksheets?</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>28. Would you be interested in a separate Logic course, primarily taught through videos, and reinforced with worksheets?</t>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>Options: Yes / No / Maybe</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="8" t="inlineStr">
-        <is>
-          <t>Options: Yes / No / Maybe</t>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>29. If a curriculum offered 5 minutes of independent Bible reading and 15 minutes of Bible teaching, including an active engagement,would you utilize optional material to dig deeper into the subject? If so, what kinds of engagements would you use?</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>29. If a curriculum offered 5 minutes of independent Bible reading and 15 minutes of Bible teaching, including an active engagement,would you utilize optional material to dig deeper into the subject? If so, what kinds of engagements would you use?</t>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>Options: Discussions / Alternate in-depth videos / Journaling prompts / Further Bible reading / Other activities</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="8" t="inlineStr">
-        <is>
-          <t>Options: Discussions / Alternate in-depth videos / Journaling prompts / Further Bible reading / Other activities</t>
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>30. How important is it for your students to handle a printable reference book (DeepRoots’ Course Pack) versus using a reference book online?</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>30. How important is it for your students to handle a printable reference book (DeepRoots’ Course Pack) versus using a reference book online?</t>
+          <t>31. If you had a choice between individual quiet work or a group activity, which would you prefer? Which would your students prefer?</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>31. If you had a choice between individual quiet work or a group activity, which would you prefer? Which would your students prefer?</t>
+          <t>32. As a teacher, what does your ideal Bible lesson look like?</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>32. As a teacher, what does your ideal Bible lesson look like?</t>
+          <t>33. How do you measure the success of a curriculum?</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>33. How do you measure the success of a curriculum?</t>
+          <t>34. Are there any visual styles, trends, or design approaches you think would not work well with your Middle School students?</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>34. Are there any visual styles, trends, or design approaches you think would not work well with your Middle School students?</t>
+          <t>35. What short videos would be helpful to supplement your teaching?</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>35. What short videos would be helpful to supplement your teaching?</t>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>Options: Videos that tie the lesson into real world application / Videos that hit on the key idea of the lesson / Videos that introduce the subject matter before teaching</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="B58" s="8" t="inlineStr">
-        <is>
-          <t>Options: Videos that tie the lesson into real world application / Videos that hit on the key idea of the lesson / Videos that introduce the subject matter before teaching</t>
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>36. On a scale of 1-10 how would you rate role-play activities for engagement?</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>36. On a scale of 1-10 how would you rate role-play activities for engagement?</t>
+          <t>37. What elements of a Bible curriculum do you not prefer?</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>37. What elements of a Bible curriculum do you not prefer?</t>
+          <t>38. What gets and holds your students attention in Bible class?</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
-        <is>
-          <t>38. What gets and holds your students attention in Bible class?</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
         <is>
           <t>39. In your opinion, what would a middle school Bible curriculum look like that is easy to teach while also being impactful for students?</t>
         </is>
@@ -5988,16 +6083,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>DeepRoots — Middle School Curriculum Outreach: Round 2 Response Tracker</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>DeepRoots — Middle School Round 2 Response Tracker</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Last updated: 2026-09-10 — 3 replied, 1 said yes, 1 bounced (of 133).</t>
+          <t>Updated 2026-09-10: 3 replied, 1 want in, 11 bounced (of 133).</t>
         </is>
       </c>
     </row>
@@ -6007,14 +6102,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Green = wants to take part. Grey = replied (declined/referral). Red = bounced address.</t>
+          <t>Green=wants in. Grey=replied/declined. Red=bounced (bad address). Yellow=caution.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fill Date Emailed as you send; Questions Sent once you send the preview email (Questions Email tab).</t>
+          <t>All 4 sent eagleslanding.org addresses bounced — that school's addresses look invalid.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: Sarah Barlowe & Tanya Murphy replies (both decline; Tanya refers Diana Helton)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -480,10 +480,10 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="64" customWidth="1" min="13" max="13"/>
+    <col width="66" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2348,41 +2348,61 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="3" t="n">
         <v>47</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Christian Academy of Indiana</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>New Albany</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="3" t="inlineStr">
         <is>
           <t>Sarah Barlowe</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="3" t="inlineStr">
         <is>
           <t>sbarlowe@caschools.us</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
-      <c r="K48" t="inlineStr"/>
-      <c r="L48" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>No - K-12 ELL teacher, not a fit</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr"/>
+      <c r="L48" s="3" t="inlineStr"/>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-10: teaches ELL in small pull-out groups; does not think it is a good fit.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -4813,41 +4833,61 @@
       <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
-      <c r="A113" t="n">
+      <c r="A113" s="3" t="n">
         <v>112</v>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B113" s="3" t="inlineStr">
         <is>
           <t>Foundation Academy - Lakeside</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C113" s="3" t="inlineStr">
         <is>
           <t>Orlando</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D113" s="3" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
+      <c r="E113" s="3" t="inlineStr">
         <is>
           <t>Tanya Murphy</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr">
+      <c r="F113" s="3" t="inlineStr">
         <is>
           <t>tanya.murphy@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
-      <c r="M113" t="inlineStr"/>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>No - administrator; referral</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr"/>
+      <c r="L113" s="3" t="inlineStr"/>
+      <c r="M113" s="3" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-10: has not used the curriculum with students (administrator); refers Diana Helton, who has used DeepRoots.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -6076,7 +6116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -6092,7 +6132,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-10: 3 replied, 1 want in, 11 bounced (of 133).</t>
+          <t>Updated 2026-09-10: 5 replied, 1 want in, 11 bounced (of 133).</t>
         </is>
       </c>
     </row>
@@ -6102,14 +6142,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Green=wants in. Grey=replied/declined. Red=bounced (bad address). Yellow=caution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>All 4 sent eagleslanding.org addresses bounced — that school's addresses look invalid.</t>
+          <t>Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record new reply on Calvary Christian Academy - Ft Lauderdale thread
Julianne Rettig (n=30) replied on the auto-forwarded thread originally
sent to Kathy Agarth (n=31, now retired), offering to help personally
or connect us with the school's MS Bible teachers. Mark both records
responded, and flag Julianne for the questions-preview email next.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XFe7baNzGqeP2WJQxc1z2m
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$134</definedName>
@@ -46,7 +46,7 @@
       <color rgb="00666666"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +78,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+        <bgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFEFEF"/>
+        <bgColor rgb="00EFEFEF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -91,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -103,6 +115,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -639,13 +653,6 @@
           <t>alison.gioia@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -676,13 +683,6 @@
           <t>chris.zaccaro@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -713,13 +713,6 @@
           <t>kasey.murray@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -750,13 +743,6 @@
           <t>kate.lunberry@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -787,13 +773,6 @@
           <t>arudy@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -824,13 +803,6 @@
           <t>ghall@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -861,13 +833,6 @@
           <t>lreyes@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -955,13 +920,6 @@
           <t>kelli.larsen@benlippen.com</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -992,13 +950,6 @@
           <t>steve.maurelli@benlippen.com</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1029,13 +980,6 @@
           <t>sheri_fyke@bereanwpb.org</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1066,13 +1010,6 @@
           <t>apeavy@bcamail.org</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1250,13 +1187,6 @@
           <t>goode@bocachristian.org</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1287,13 +1217,6 @@
           <t>fryk@bocachristian.org</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1324,13 +1247,6 @@
           <t>ashleykim@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1361,13 +1277,6 @@
           <t>carolynng@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1398,13 +1307,6 @@
           <t>helenyoolee@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1435,13 +1337,6 @@
           <t>jennylee@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1472,13 +1367,6 @@
           <t>stephenlim@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1509,13 +1397,6 @@
           <t>jreyes@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1546,13 +1427,6 @@
           <t>jmcclintock@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1583,13 +1457,6 @@
           <t>mmarquez@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1620,13 +1487,6 @@
           <t>addyc@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1657,13 +1517,6 @@
           <t>davidd@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1694,87 +1547,120 @@
           <t>evak@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>Calvary Christian Academy - Ft Lauderdale</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="9" t="inlineStr">
         <is>
           <t>Fort Lauderdale</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="9" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E31" s="9" t="inlineStr">
         <is>
           <t>Julianne Rettig</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>julianner@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
-      <c r="L31" t="inlineStr"/>
-      <c r="M31" t="inlineStr"/>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I31" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="J31" s="9" t="inlineStr">
+        <is>
+          <t>YES — happy to help personally (or refer to MS Bible teachers)</t>
+        </is>
+      </c>
+      <c r="K31" s="9" t="inlineStr"/>
+      <c r="L31" s="9" t="inlineStr"/>
+      <c r="M31" s="9" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>Calvary Christian Academy - Ft Lauderdale</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>Fort Lauderdale</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>Kathy Agarth</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="10" t="inlineStr">
         <is>
           <t>kathya@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
-      <c r="L32" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="J32" s="10" t="inlineStr">
+        <is>
+          <t>N/A — retired; referred to Julianne Rettig (n=30, also on list)</t>
+        </is>
+      </c>
+      <c r="K32" s="10" t="inlineStr"/>
+      <c r="L32" s="10" t="inlineStr"/>
+      <c r="M32" s="10" t="inlineStr">
+        <is>
+          <t>Reply received 2026-09-11 from Julianne Rettig (Director of Upper School Academics), who now receives Kathy's auto-forwarded mail since Kathy has retired: Julianne offered to help personally or connect us with the MS Bible teachers. Treat Julianne (n=30) as the active contact for this thread; no action needed on Kathy's address.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1805,13 +1691,6 @@
           <t>leac@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1842,13 +1721,6 @@
           <t>nikkib@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1879,13 +1751,6 @@
           <t>darylb@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1916,13 +1781,6 @@
           <t>jperez@ccslancers.com</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1953,13 +1811,6 @@
           <t>sdiaz@ccslancers.com</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1990,13 +1841,6 @@
           <t>angelaguiton@cbckannapolis.com</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2027,13 +1871,6 @@
           <t>hornerb@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2064,13 +1901,6 @@
           <t>kassie@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2101,13 +1931,6 @@
           <t>freitask@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2138,13 +1961,6 @@
           <t>ashley.jenkins@charchrist.com</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2175,13 +1991,6 @@
           <t>brandon.henderson@charchrist.com</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2212,13 +2021,6 @@
           <t>christina.sachtleben@charchrist.com</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -2294,13 +2096,6 @@
           <t>katey.balikian@charchrist.com</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -2433,13 +2228,6 @@
           <t>sneal@caschools.us</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2470,13 +2258,6 @@
           <t>acarson@caschools.us</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2507,13 +2288,6 @@
           <t>bwiley@caschools.us</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2544,13 +2318,6 @@
           <t>ctroyer@caschools.us</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2581,13 +2348,6 @@
           <t>cwallace@caschools.us</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -2708,13 +2468,6 @@
           <t>jgutierrez@caschools.us</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2745,13 +2498,6 @@
           <t>lberg@caschools.us</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2782,13 +2528,6 @@
           <t>mchitty@caschools.us</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2819,13 +2558,6 @@
           <t>mcrawford@caschools.us</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2856,13 +2588,6 @@
           <t>svincentz@caschools.us</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2893,13 +2618,6 @@
           <t>aengle@cfsknights.org</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2930,13 +2648,6 @@
           <t>mclay@cfsknights.org</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2967,13 +2678,6 @@
           <t>shixon@cfsknights.org</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3004,13 +2708,6 @@
           <t>apetersen@chslions.com</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3041,13 +2738,6 @@
           <t>victoria.swing@concordchristian.org</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3078,13 +2768,6 @@
           <t>jstudt@concordchristianschool.org</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3115,13 +2798,6 @@
           <t>klittleton@concordchristianschool.org</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3152,13 +2828,6 @@
           <t>kmaddox@concordcs.org</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3189,13 +2858,6 @@
           <t>mark.clinton@cornerstonechristian.com</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3226,13 +2888,6 @@
           <t>ckronberger@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3263,13 +2918,6 @@
           <t>kmerina@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3300,13 +2948,6 @@
           <t>lkieling@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3337,13 +2978,6 @@
           <t>danielle.williams@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3374,13 +3008,6 @@
           <t>erin.wilhelm@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3411,13 +3038,6 @@
           <t>jessica.gates@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3448,13 +3068,6 @@
           <t>dhenry@dayspringchristian.com</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3485,13 +3098,6 @@
           <t>kjohnson@dayspringchristian.com</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3522,13 +3128,6 @@
           <t>shall@dhca.org</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3559,13 +3158,6 @@
           <t>emily.manuel@dmcs.org</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3596,13 +3188,6 @@
           <t>hnerem@dmcs.org</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3633,13 +3218,6 @@
           <t>ksteen@dmcs.org</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3670,13 +3248,6 @@
           <t>lsteele@dmcs.org</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3707,13 +3278,6 @@
           <t>slortz@dmcs.org</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3744,13 +3308,6 @@
           <t>wweaver@dmcs.org</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -4002,13 +3559,6 @@
           <t>j_kughn@ehcseagles.com</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4039,13 +3589,6 @@
           <t>tmm@elkhartchristian.org</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4076,13 +3619,6 @@
           <t>awilliams@faithlafayette.org</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4113,13 +3649,6 @@
           <t>kkelso@faithlafayette.org</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4150,13 +3679,6 @@
           <t>erik.harris@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4187,13 +3709,6 @@
           <t>jennifer.harris@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4224,13 +3739,6 @@
           <t>jeremy.jones@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4261,13 +3769,6 @@
           <t>will.lamb@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4298,13 +3799,6 @@
           <t>danielle.reeves@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -4380,13 +3874,6 @@
           <t>michelle.eastman@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4417,13 +3904,6 @@
           <t>sherri.mcleroy@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -4454,13 +3934,6 @@
           <t>cdavis@fbchighsprings.org</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
-      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -4491,13 +3964,6 @@
           <t>spotter@fbchighsprings.org</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
-      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -4528,13 +3994,6 @@
           <t>mrs.coleman@firstchristianacademy.com</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4565,13 +4024,6 @@
           <t>mrs.butler@firstchristianacademy.com</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
-      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4602,13 +4054,6 @@
           <t>lthompson@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
-      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4639,13 +4084,6 @@
           <t>lwilson@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
-      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -4676,13 +4114,6 @@
           <t>rgutzwiller@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
-      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4713,13 +4144,6 @@
           <t>brooke.newell@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
-      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -4750,13 +4174,6 @@
           <t>corey.cline@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
-      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4787,13 +4204,6 @@
           <t>jessica.meade@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
-      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4824,13 +4234,6 @@
           <t>julie.daniel@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
-      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n">
@@ -4918,13 +4321,6 @@
           <t>thomas.rodriguez@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
-      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -4955,13 +4351,6 @@
           <t>ajongko@gac.org</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
-      <c r="M115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -4992,13 +4381,6 @@
           <t>jbaker@gac.org</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
-      <c r="M116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5029,13 +4411,6 @@
           <t>rhelms@gac.org</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
-      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5066,13 +4441,6 @@
           <t>uricketts@gac.org</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
-      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5103,13 +4471,6 @@
           <t>c.williams@leechristian.org</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
-      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -5140,13 +4501,6 @@
           <t>g.dykes@leechristian.org</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5177,13 +4531,6 @@
           <t>dwillis@metroca.com</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -5214,13 +4561,6 @@
           <t>jfeamster@metroca.com</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
-      <c r="M122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -5251,13 +4591,6 @@
           <t>kchenoweth@metroca.com</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
-      <c r="M123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -5288,13 +4621,6 @@
           <t>mbuffington@metroca.com</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -5325,13 +4651,6 @@
           <t>ksabia@northhillschristian.com</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -5362,13 +4681,6 @@
           <t>rpierce@northhillschristian.com</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
-      <c r="M126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -5399,13 +4711,6 @@
           <t>cgrimmer@phoenixchristian.org</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
-      <c r="M127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -5436,13 +4741,6 @@
           <t>csianturi@phoenixchristian.org</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
-      <c r="M128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -5473,13 +4771,6 @@
           <t>michelle.wilson@ranchochristian.org</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
-      <c r="M129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -5510,13 +4801,6 @@
           <t>nate.porter@ranchochristian.org</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
-      <c r="M130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -5547,13 +4831,6 @@
           <t>bspeier@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
-      <c r="M131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -5584,13 +4861,6 @@
           <t>jgross@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr"/>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
-      <c r="M132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -5621,13 +4891,6 @@
           <t>scairo@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
-      <c r="H133" t="inlineStr"/>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
-      <c r="M133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -5658,13 +4921,6 @@
           <t>mimel@tlcs.tlc.org</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
-      <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
-      <c r="M134" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:M134"/>
@@ -6136,9 +5392,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Tracker: add Sharron Jones (referral from Kelly Vann)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +46,7 @@
       <color rgb="00666666"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -80,14 +80,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
-        <bgColor rgb="00D9EAD3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EFEFEF"/>
-        <bgColor rgb="00EFEFEF"/>
+        <fgColor rgb="00DEEAF6"/>
       </patternFill>
     </fill>
   </fills>
@@ -103,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -112,11 +105,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -482,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M134"/>
+  <dimension ref="A1:M135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -653,6 +645,13 @@
           <t>alison.gioia@ashevillechristian.org</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -683,6 +682,13 @@
           <t>chris.zaccaro@ashevillechristian.org</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -713,6 +719,13 @@
           <t>kasey.murray@ashevillechristian.org</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -743,6 +756,13 @@
           <t>kate.lunberry@ashevillechristian.org</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -773,6 +793,13 @@
           <t>arudy@shoreschristian.org</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -803,6 +830,13 @@
           <t>ghall@shoreschristian.org</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -833,6 +867,13 @@
           <t>lreyes@shoreschristian.org</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -920,6 +961,13 @@
           <t>kelli.larsen@benlippen.com</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -950,6 +998,13 @@
           <t>steve.maurelli@benlippen.com</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -980,6 +1035,13 @@
           <t>sheri_fyke@bereanwpb.org</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1010,6 +1072,13 @@
           <t>apeavy@bcamail.org</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1187,6 +1256,13 @@
           <t>goode@bocachristian.org</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1217,6 +1293,13 @@
           <t>fryk@bocachristian.org</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1247,6 +1330,13 @@
           <t>ashleykim@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1277,6 +1367,13 @@
           <t>carolynng@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1307,6 +1404,13 @@
           <t>helenyoolee@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1337,6 +1441,13 @@
           <t>jennylee@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1367,6 +1478,13 @@
           <t>stephenlim@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1397,6 +1515,13 @@
           <t>jreyes@calvarydowney.org</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1427,6 +1552,13 @@
           <t>jmcclintock@calvarydowney.org</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1457,6 +1589,13 @@
           <t>mmarquez@calvarydowney.org</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1487,6 +1626,13 @@
           <t>addyc@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1517,6 +1663,13 @@
           <t>davidd@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1547,116 +1700,123 @@
           <t>evak@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="n">
+      <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Calvary Christian Academy - Ft Lauderdale</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Fort Lauderdale</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Julianne Rettig</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>julianner@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H31" s="9" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I31" s="9" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="J31" s="9" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>YES — happy to help personally (or refer to MS Bible teachers)</t>
         </is>
       </c>
-      <c r="K31" s="9" t="inlineStr"/>
-      <c r="L31" s="9" t="inlineStr"/>
-      <c r="M31" s="9" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n">
+      <c r="A32" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Calvary Christian Academy - Ft Lauderdale</t>
         </is>
       </c>
-      <c r="C32" s="10" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Fort Lauderdale</t>
         </is>
       </c>
-      <c r="D32" s="10" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>Kathy Agarth</t>
         </is>
       </c>
-      <c r="F32" s="10" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>kathya@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G32" s="10" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H32" s="10" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I32" s="10" t="inlineStr">
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="J32" s="10" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>N/A — retired; referred to Julianne Rettig (n=30, also on list)</t>
         </is>
       </c>
-      <c r="K32" s="10" t="inlineStr"/>
-      <c r="L32" s="10" t="inlineStr"/>
-      <c r="M32" s="10" t="inlineStr">
+      <c r="K32" s="3" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr"/>
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>Reply received 2026-09-11 from Julianne Rettig (Director of Upper School Academics), who now receives Kathy's auto-forwarded mail since Kathy has retired: Julianne offered to help personally or connect us with the MS Bible teachers. Treat Julianne (n=30) as the active contact for this thread; no action needed on Kathy's address.</t>
         </is>
@@ -1691,6 +1851,13 @@
           <t>leac@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1721,6 +1888,13 @@
           <t>nikkib@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1751,6 +1925,13 @@
           <t>darylb@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1781,6 +1962,13 @@
           <t>jperez@ccslancers.com</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1811,6 +1999,13 @@
           <t>sdiaz@ccslancers.com</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1841,6 +2036,13 @@
           <t>angelaguiton@cbckannapolis.com</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1871,6 +2073,13 @@
           <t>hornerb@chapel-hill.org</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1901,6 +2110,13 @@
           <t>kassie@chapel-hill.org</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1931,6 +2147,13 @@
           <t>freitask@chapel-hill.org</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1961,6 +2184,13 @@
           <t>ashley.jenkins@charchrist.com</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1991,6 +2221,13 @@
           <t>brandon.henderson@charchrist.com</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2021,6 +2258,13 @@
           <t>christina.sachtleben@charchrist.com</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -2096,6 +2340,13 @@
           <t>katey.balikian@charchrist.com</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -2228,6 +2479,13 @@
           <t>sneal@caschools.us</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2258,6 +2516,13 @@
           <t>acarson@caschools.us</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2288,6 +2553,13 @@
           <t>bwiley@caschools.us</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2318,6 +2590,13 @@
           <t>ctroyer@caschools.us</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2348,6 +2627,13 @@
           <t>cwallace@caschools.us</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -2468,6 +2754,13 @@
           <t>jgutierrez@caschools.us</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2498,6 +2791,13 @@
           <t>lberg@caschools.us</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2528,6 +2828,13 @@
           <t>mchitty@caschools.us</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2558,6 +2865,13 @@
           <t>mcrawford@caschools.us</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2588,6 +2902,13 @@
           <t>svincentz@caschools.us</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2618,6 +2939,13 @@
           <t>aengle@cfsknights.org</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2648,6 +2976,13 @@
           <t>mclay@cfsknights.org</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2678,6 +3013,13 @@
           <t>shixon@cfsknights.org</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2708,6 +3050,13 @@
           <t>apetersen@chslions.com</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2738,6 +3087,13 @@
           <t>victoria.swing@concordchristian.org</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2768,6 +3124,13 @@
           <t>jstudt@concordchristianschool.org</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2798,6 +3161,13 @@
           <t>klittleton@concordchristianschool.org</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2828,6 +3198,13 @@
           <t>kmaddox@concordcs.org</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2858,6 +3235,13 @@
           <t>mark.clinton@cornerstonechristian.com</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2888,6 +3272,13 @@
           <t>ckronberger@crosshillchristian.com</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2918,6 +3309,13 @@
           <t>kmerina@crosshillchristian.com</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2948,6 +3346,13 @@
           <t>lkieling@crosshillchristian.com</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2978,6 +3383,13 @@
           <t>danielle.williams@cypresschristian.org</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3008,6 +3420,13 @@
           <t>erin.wilhelm@cypresschristian.org</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3038,6 +3457,13 @@
           <t>jessica.gates@cypresschristian.org</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3068,6 +3494,13 @@
           <t>dhenry@dayspringchristian.com</t>
         </is>
       </c>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3098,6 +3531,13 @@
           <t>kjohnson@dayspringchristian.com</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3128,6 +3568,13 @@
           <t>shall@dhca.org</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3158,6 +3605,13 @@
           <t>emily.manuel@dmcs.org</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3188,6 +3642,13 @@
           <t>hnerem@dmcs.org</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3218,6 +3679,13 @@
           <t>ksteen@dmcs.org</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3248,6 +3716,13 @@
           <t>lsteele@dmcs.org</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3278,6 +3753,13 @@
           <t>slortz@dmcs.org</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3308,6 +3790,13 @@
           <t>wweaver@dmcs.org</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -3559,6 +4048,13 @@
           <t>j_kughn@ehcseagles.com</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3589,6 +4085,13 @@
           <t>tmm@elkhartchristian.org</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3619,6 +4122,13 @@
           <t>awilliams@faithlafayette.org</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3649,6 +4159,13 @@
           <t>kkelso@faithlafayette.org</t>
         </is>
       </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3679,6 +4196,13 @@
           <t>erik.harris@fcspatriots.com</t>
         </is>
       </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3709,6 +4233,13 @@
           <t>jennifer.harris@fcspatriots.com</t>
         </is>
       </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3739,6 +4270,13 @@
           <t>jeremy.jones@fcspatriots.com</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3769,6 +4307,13 @@
           <t>will.lamb@fcspatriots.com</t>
         </is>
       </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3799,6 +4344,13 @@
           <t>danielle.reeves@fcspaladins.org</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -3874,6 +4426,13 @@
           <t>michelle.eastman@fcspaladins.org</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3904,6 +4463,13 @@
           <t>sherri.mcleroy@fcspaladins.org</t>
         </is>
       </c>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -3934,6 +4500,13 @@
           <t>cdavis@fbchighsprings.org</t>
         </is>
       </c>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -3964,6 +4537,13 @@
           <t>spotter@fbchighsprings.org</t>
         </is>
       </c>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -3994,6 +4574,13 @@
           <t>mrs.coleman@firstchristianacademy.com</t>
         </is>
       </c>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4024,6 +4611,13 @@
           <t>mrs.butler@firstchristianacademy.com</t>
         </is>
       </c>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4054,6 +4648,13 @@
           <t>lthompson@foothillchristian.org</t>
         </is>
       </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4084,6 +4685,13 @@
           <t>lwilson@foothillchristian.org</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -4114,6 +4722,13 @@
           <t>rgutzwiller@foothillchristian.org</t>
         </is>
       </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4144,6 +4759,13 @@
           <t>brooke.newell@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -4174,6 +4796,13 @@
           <t>corey.cline@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4204,6 +4833,13 @@
           <t>jessica.meade@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4234,6 +4870,13 @@
           <t>julie.daniel@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n">
@@ -4321,6 +4964,13 @@
           <t>thomas.rodriguez@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -4351,6 +5001,13 @@
           <t>ajongko@gac.org</t>
         </is>
       </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -4381,6 +5038,13 @@
           <t>jbaker@gac.org</t>
         </is>
       </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -4411,6 +5075,13 @@
           <t>rhelms@gac.org</t>
         </is>
       </c>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -4441,6 +5112,13 @@
           <t>uricketts@gac.org</t>
         </is>
       </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -4471,6 +5149,13 @@
           <t>c.williams@leechristian.org</t>
         </is>
       </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -4501,6 +5186,13 @@
           <t>g.dykes@leechristian.org</t>
         </is>
       </c>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -4531,6 +5223,13 @@
           <t>dwillis@metroca.com</t>
         </is>
       </c>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -4561,6 +5260,13 @@
           <t>jfeamster@metroca.com</t>
         </is>
       </c>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -4591,6 +5297,13 @@
           <t>kchenoweth@metroca.com</t>
         </is>
       </c>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -4621,6 +5334,13 @@
           <t>mbuffington@metroca.com</t>
         </is>
       </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -4651,6 +5371,13 @@
           <t>ksabia@northhillschristian.com</t>
         </is>
       </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -4681,6 +5408,13 @@
           <t>rpierce@northhillschristian.com</t>
         </is>
       </c>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -4711,6 +5445,13 @@
           <t>cgrimmer@phoenixchristian.org</t>
         </is>
       </c>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -4741,6 +5482,13 @@
           <t>csianturi@phoenixchristian.org</t>
         </is>
       </c>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -4771,6 +5519,13 @@
           <t>michelle.wilson@ranchochristian.org</t>
         </is>
       </c>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -4801,6 +5556,13 @@
           <t>nate.porter@ranchochristian.org</t>
         </is>
       </c>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -4831,6 +5593,13 @@
           <t>bspeier@southfieldchristian.org</t>
         </is>
       </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -4861,6 +5630,13 @@
           <t>jgross@southfieldchristian.org</t>
         </is>
       </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -4891,6 +5667,13 @@
           <t>scairo@southfieldchristian.org</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -4921,9 +5704,57 @@
           <t>mimel@tlcs.tlc.org</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="6" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="6" t="inlineStr">
+        <is>
+          <t>Bethlehem Christian Academy - Elementary</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="inlineStr">
+        <is>
+          <t>Bethlehem</t>
+        </is>
+      </c>
+      <c r="D135" s="6" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="E135" s="6" t="inlineStr">
+        <is>
+          <t>Sharron Jones</t>
+        </is>
+      </c>
+      <c r="F135" s="6" t="inlineStr">
+        <is>
+          <t>sjones@bcamail.org</t>
+        </is>
+      </c>
+      <c r="G135" s="6" t="inlineStr"/>
+      <c r="H135" s="6" t="inlineStr"/>
+      <c r="I135" s="6" t="inlineStr"/>
+      <c r="J135" s="6" t="inlineStr"/>
+      <c r="K135" s="6" t="inlineStr"/>
+      <c r="L135" s="6" t="inlineStr"/>
+      <c r="M135" s="6" t="inlineStr">
+        <is>
+          <t>REFERRAL from Kelly Vann (Bethlehem). Invitation drafted 2026-09-11.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M134"/>
+  <autoFilter ref="A1:M135"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4942,14 +5773,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Questions Preview Email</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
@@ -4963,7 +5794,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Options: 5-8? / 6-8? / 7-8?</t>
         </is>
@@ -4977,7 +5808,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Options: Developmentally? / Spiritually? / Emotionally?</t>
         </is>
@@ -5019,7 +5850,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
@@ -5033,7 +5864,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Options: Teaching / Reading / Discussion time / Activities</t>
         </is>
@@ -5047,7 +5878,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
         </is>
@@ -5061,7 +5892,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>Options: To project images and other teaching materials / To play educational videos / Other</t>
         </is>
@@ -5075,7 +5906,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
         </is>
@@ -5089,7 +5920,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -5110,14 +5941,14 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="9" t="inlineStr">
         <is>
           <t>Options: 6th / 7th / 8th</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
@@ -5138,7 +5969,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Options: 30 seconds -1min / 1 min-2min / 2 min-3min / 3 minutes +</t>
         </is>
@@ -5152,7 +5983,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>Options: Photography / Illustrations / Infographics/diagrams / Maps and timelines / Historical artwork / Charts and visual explanations / Short-form comics or graphic storytelling / Other</t>
         </is>
@@ -5173,7 +6004,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Options: Mostly visual, with short amounts of text / A balanced mix of text and visuals / Mostly text, with visuals used to support key concepts / It depends on the lesson</t>
         </is>
@@ -5201,7 +6032,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Additional Questions</t>
         </is>
@@ -5222,7 +6053,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -5250,7 +6081,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B46" s="9" t="inlineStr">
         <is>
           <t>Options: In school with boys taught by a male teacher and girls taught by a female teacher, with advance permission from parents / Sent home to parents as a resource to use with their own child as they see fit / We would not use it at our school or send it home to parents.</t>
         </is>
@@ -5264,7 +6095,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -5278,7 +6109,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>Options: Discussions / Alternate in-depth videos / Journaling prompts / Further Bible reading / Other activities</t>
         </is>
@@ -5327,7 +6158,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="B57" s="8" t="inlineStr">
+      <c r="B57" s="9" t="inlineStr">
         <is>
           <t>Options: Videos that tie the lesson into real world application / Videos that hit on the key idea of the lesson / Videos that introduce the subject matter before teaching</t>
         </is>
@@ -5379,7 +6210,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>DeepRoots — Middle School Round 2 Response Tracker</t>
         </is>
@@ -5388,15 +6219,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-10: 5 replied, 1 want in, 11 bounced (of 133).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Updated 2026-09-11: 134 contacts, 7 replied, 2 want in, 11 bounced, 1 referral added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution.</t>
+          <t>Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution. Blue=referral contact.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: correct referral name to Shannon Jones
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -5733,7 +5733,7 @@
       </c>
       <c r="E135" s="6" t="inlineStr">
         <is>
-          <t>Sharron Jones</t>
+          <t>Shannon Jones</t>
         </is>
       </c>
       <c r="F135" s="6" t="inlineStr">
@@ -5749,7 +5749,7 @@
       <c r="L135" s="6" t="inlineStr"/>
       <c r="M135" s="6" t="inlineStr">
         <is>
-          <t>REFERRAL from Kelly Vann (Bethlehem). Invitation drafted 2026-09-11.</t>
+          <t>REFERRAL from Kelly Vann (Bethlehem). Invitation sent 2026-09-10 (greeting "Shannon").</t>
         </is>
       </c>
     </row>
@@ -6219,7 +6219,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-11: 134 contacts, 7 replied, 2 want in, 11 bounced, 1 referral added.</t>
+          <t>Updated 2026-09-11: 134 contacts, 7 replied, 2 want in, 11 bounced, 1 referral.</t>
         </is>
       </c>
     </row>
@@ -6229,7 +6229,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution. Blue=referral contact.</t>
+          <t>Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution. Blue=referral.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker check 2026-09-15: add Donna Hurley (referral, yes) and Diana Helton (yes); Dee Henry referral
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$135</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$137</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M135"/>
+  <dimension ref="A1:M137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -486,7 +486,7 @@
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="66" customWidth="1" min="13" max="13"/>
@@ -1757,7 +1757,11 @@
           <t>YES — happy to help personally (or refer to MS Bible teachers)</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="L31" s="2" t="inlineStr"/>
       <c r="M31" s="2" t="inlineStr">
         <is>
@@ -3466,41 +3470,61 @@
       <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" t="n">
+      <c r="A76" s="3" t="n">
         <v>75</v>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>Dayspring Christian Academy</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>Mountville</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>Dee Henry</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F76" s="3" t="inlineStr">
         <is>
           <t>dhenry@dayspringchristian.com</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>Referral -&gt; Donna Hurley (Upper School curriculum director)</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr"/>
+      <c r="L76" s="3" t="inlineStr"/>
+      <c r="M76" s="3" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-14: referred Donna Hurley (dhurley@dayspringchristian.com), who would love to talk. Troy engaged both 2026-09-14.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -5753,8 +5777,126 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Mountville</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>Donna Hurley</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>dhurley@dayspringchristian.com</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>YES - Upper School curriculum director, wants to talk</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr"/>
+      <c r="L136" s="2" t="inlineStr"/>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Foundation Academy</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Winter Garden</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>Diana Helton</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>diana.helton@foundationacademy.net</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>YES - happy to help (elementary)</t>
+        </is>
+      </c>
+      <c r="K137" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L137" s="2" t="inlineStr"/>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>Round 1 contact; agreed 2026-09-11 and questions sent 2026-09-11. Also referred by Tanya Murphy.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M135"/>
+  <autoFilter ref="A1:M137"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6219,7 +6361,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-11: 134 contacts, 7 replied, 2 want in, 11 bounced, 1 referral.</t>
+          <t>Updated 2026-09-15: 136 contacts, 10 replied, 4 want in, 11 bounced.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker check 2026-09-16: add Wendy Wagoner (yes, questions sent)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$137</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$138</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M137"/>
+  <dimension ref="A1:M138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -5895,8 +5895,69 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Christian Academy of Indiana</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>New Albany</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>Wendy Wagoner</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>wwagoner@caschools.us</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>YES - happy to help</t>
+        </is>
+      </c>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L138" s="2" t="inlineStr"/>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M137"/>
+  <autoFilter ref="A1:M138"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6361,7 +6422,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-15: 136 contacts, 10 replied, 4 want in, 11 bounced.</t>
+          <t>Updated 2026-09-16: 137 contacts, 11 replied, 5 want in, 11 bounced.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: log scheduling nudges sent 2026-09-17 to the 5 participants
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -488,7 +488,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="12" max="12"/>
     <col width="66" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -609,10 +609,14 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Nudged 2026-09-17 for times</t>
+        </is>
+      </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule.</t>
+          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
         </is>
       </c>
     </row>
@@ -1762,10 +1766,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Nudged 2026-09-17 for times</t>
+        </is>
+      </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next.</t>
+          <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
         </is>
       </c>
     </row>
@@ -5827,10 +5835,14 @@
         </is>
       </c>
       <c r="K136" s="2" t="inlineStr"/>
-      <c r="L136" s="2" t="inlineStr"/>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>Nudged 2026-09-17 for times</t>
+        </is>
+      </c>
       <c r="M136" s="2" t="inlineStr">
         <is>
-          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14.</t>
+          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
         </is>
       </c>
     </row>
@@ -5888,10 +5900,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="L137" s="2" t="inlineStr"/>
+      <c r="L137" s="2" t="inlineStr">
+        <is>
+          <t>Nudged 2026-09-17 for times</t>
+        </is>
+      </c>
       <c r="M137" s="2" t="inlineStr">
         <is>
-          <t>Round 1 contact; agreed 2026-09-11 and questions sent 2026-09-11. Also referred by Tanya Murphy.</t>
+          <t>Round 1 contact; agreed 2026-09-11 and questions sent 2026-09-11. Also referred by Tanya Murphy. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
         </is>
       </c>
     </row>
@@ -5949,10 +5965,14 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="L138" s="2" t="inlineStr"/>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>Nudged 2026-09-17 for times</t>
+        </is>
+      </c>
       <c r="M138" s="2" t="inlineStr">
         <is>
-          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16.</t>
+          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
         </is>
       </c>
     </row>
@@ -6422,7 +6442,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-16: 137 contacts, 11 replied, 5 want in, 11 bounced.</t>
+          <t>Updated 2026-09-17: 137 contacts, 11 replied, 5 want in, 11 bounced. Scheduling nudges sent to the 5 who want in.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker: Meredith availability (Pacific); Julianne deferred a few weeks
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -488,7 +488,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
     <col width="66" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -611,12 +611,12 @@
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Nudged 2026-09-17 for times</t>
+          <t>Availability (Pacific): next wk Mon/Thu/Fri 10-12 PT; following wk Mon/Wed 9-11 PT</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
+          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule. | Scheduling nudge sent 2026-09-17 (asked for times). | Sent availability 2026-09-17 (Pacific). Propose a specific slot.</t>
         </is>
       </c>
     </row>
@@ -1768,12 +1768,12 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Nudged 2026-09-17 for times</t>
+          <t>Deferred - off campus ~a few weeks (as of 2026-09-17); will follow up</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
+          <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-17: off campus a few weeks; will follow up.</t>
         </is>
       </c>
     </row>
@@ -6426,7 +6426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -6442,7 +6442,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-17: 137 contacts, 11 replied, 5 want in, 11 bounced. Scheduling nudges sent to the 5 who want in.</t>
+          <t>Updated 2026-09-17: 137 contacts, 11 replied, 5 want in, 11 bounced.</t>
         </is>
       </c>
     </row>
@@ -6453,6 +6453,13 @@
       <c r="A4" t="inlineStr">
         <is>
           <t>Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution. Blue=referral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Meredith Arldt sent availability (Pacific); Julianne Rettig deferred a few weeks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: Donna Hurley (Dayspring) follow-up reply 2026-09-19
She apologized for the delay, is checking with Angela Adams (Bible
dept chair) on interest, and will respond soon. No times proposed yet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WkBcobkgTQhkez322wqovF
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$138</definedName>
@@ -649,13 +649,6 @@
           <t>alison.gioia@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -686,13 +679,6 @@
           <t>chris.zaccaro@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -723,13 +709,6 @@
           <t>kasey.murray@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -760,13 +739,6 @@
           <t>kate.lunberry@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -797,13 +769,6 @@
           <t>arudy@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -834,13 +799,6 @@
           <t>ghall@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -871,13 +829,6 @@
           <t>lreyes@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -965,13 +916,6 @@
           <t>kelli.larsen@benlippen.com</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1002,13 +946,6 @@
           <t>steve.maurelli@benlippen.com</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1039,13 +976,6 @@
           <t>sheri_fyke@bereanwpb.org</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1076,13 +1006,6 @@
           <t>apeavy@bcamail.org</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1260,13 +1183,6 @@
           <t>goode@bocachristian.org</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1297,13 +1213,6 @@
           <t>fryk@bocachristian.org</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1334,13 +1243,6 @@
           <t>ashleykim@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1371,13 +1273,6 @@
           <t>carolynng@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1408,13 +1303,6 @@
           <t>helenyoolee@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1445,13 +1333,6 @@
           <t>jennylee@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1482,13 +1363,6 @@
           <t>stephenlim@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1519,13 +1393,6 @@
           <t>jreyes@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1556,13 +1423,6 @@
           <t>jmcclintock@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1593,13 +1453,6 @@
           <t>mmarquez@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1630,13 +1483,6 @@
           <t>addyc@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1667,13 +1513,6 @@
           <t>davidd@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1704,13 +1543,6 @@
           <t>evak@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1863,13 +1695,6 @@
           <t>leac@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1900,13 +1725,6 @@
           <t>nikkib@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1937,13 +1755,6 @@
           <t>darylb@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1974,13 +1785,6 @@
           <t>jperez@ccslancers.com</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2011,13 +1815,6 @@
           <t>sdiaz@ccslancers.com</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2048,13 +1845,6 @@
           <t>angelaguiton@cbckannapolis.com</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2085,13 +1875,6 @@
           <t>hornerb@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2122,13 +1905,6 @@
           <t>kassie@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2159,13 +1935,6 @@
           <t>freitask@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2196,13 +1965,6 @@
           <t>ashley.jenkins@charchrist.com</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2233,13 +1995,6 @@
           <t>brandon.henderson@charchrist.com</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2270,13 +2025,6 @@
           <t>christina.sachtleben@charchrist.com</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -2352,13 +2100,6 @@
           <t>katey.balikian@charchrist.com</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -2491,13 +2232,6 @@
           <t>sneal@caschools.us</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2528,13 +2262,6 @@
           <t>acarson@caschools.us</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2565,13 +2292,6 @@
           <t>bwiley@caschools.us</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2602,13 +2322,6 @@
           <t>ctroyer@caschools.us</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2639,13 +2352,6 @@
           <t>cwallace@caschools.us</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -2766,13 +2472,6 @@
           <t>jgutierrez@caschools.us</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2803,13 +2502,6 @@
           <t>lberg@caschools.us</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2840,13 +2532,6 @@
           <t>mchitty@caschools.us</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2877,13 +2562,6 @@
           <t>mcrawford@caschools.us</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2914,13 +2592,6 @@
           <t>svincentz@caschools.us</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2951,13 +2622,6 @@
           <t>aengle@cfsknights.org</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2988,13 +2652,6 @@
           <t>mclay@cfsknights.org</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3025,13 +2682,6 @@
           <t>shixon@cfsknights.org</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3062,13 +2712,6 @@
           <t>apetersen@chslions.com</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3099,13 +2742,6 @@
           <t>victoria.swing@concordchristian.org</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3136,13 +2772,6 @@
           <t>jstudt@concordchristianschool.org</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3173,13 +2802,6 @@
           <t>klittleton@concordchristianschool.org</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3210,13 +2832,6 @@
           <t>kmaddox@concordcs.org</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3247,13 +2862,6 @@
           <t>mark.clinton@cornerstonechristian.com</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3284,13 +2892,6 @@
           <t>ckronberger@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3321,13 +2922,6 @@
           <t>kmerina@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3358,13 +2952,6 @@
           <t>lkieling@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3395,13 +2982,6 @@
           <t>danielle.williams@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3432,13 +3012,6 @@
           <t>erin.wilhelm@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3469,13 +3042,6 @@
           <t>jessica.gates@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -3563,13 +3129,6 @@
           <t>kjohnson@dayspringchristian.com</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3600,13 +3159,6 @@
           <t>shall@dhca.org</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3637,13 +3189,6 @@
           <t>emily.manuel@dmcs.org</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3674,13 +3219,6 @@
           <t>hnerem@dmcs.org</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3711,13 +3249,6 @@
           <t>ksteen@dmcs.org</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3748,13 +3279,6 @@
           <t>lsteele@dmcs.org</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3785,13 +3309,6 @@
           <t>slortz@dmcs.org</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3822,13 +3339,6 @@
           <t>wweaver@dmcs.org</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -4080,13 +3590,6 @@
           <t>j_kughn@ehcseagles.com</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4117,13 +3620,6 @@
           <t>tmm@elkhartchristian.org</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4154,13 +3650,6 @@
           <t>awilliams@faithlafayette.org</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4191,13 +3680,6 @@
           <t>kkelso@faithlafayette.org</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4228,13 +3710,6 @@
           <t>erik.harris@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4265,13 +3740,6 @@
           <t>jennifer.harris@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4302,13 +3770,6 @@
           <t>jeremy.jones@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4339,13 +3800,6 @@
           <t>will.lamb@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4376,13 +3830,6 @@
           <t>danielle.reeves@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -4458,13 +3905,6 @@
           <t>michelle.eastman@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4495,13 +3935,6 @@
           <t>sherri.mcleroy@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -4532,13 +3965,6 @@
           <t>cdavis@fbchighsprings.org</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
-      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -4569,13 +3995,6 @@
           <t>spotter@fbchighsprings.org</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
-      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -4606,13 +4025,6 @@
           <t>mrs.coleman@firstchristianacademy.com</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4643,13 +4055,6 @@
           <t>mrs.butler@firstchristianacademy.com</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
-      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4680,13 +4085,6 @@
           <t>lthompson@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
-      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4717,13 +4115,6 @@
           <t>lwilson@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
-      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -4754,13 +4145,6 @@
           <t>rgutzwiller@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
-      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4791,13 +4175,6 @@
           <t>brooke.newell@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
-      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -4828,13 +4205,6 @@
           <t>corey.cline@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
-      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4865,13 +4235,6 @@
           <t>jessica.meade@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
-      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4902,13 +4265,6 @@
           <t>julie.daniel@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
-      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n">
@@ -4996,13 +4352,6 @@
           <t>thomas.rodriguez@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
-      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -5033,13 +4382,6 @@
           <t>ajongko@gac.org</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
-      <c r="M115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -5070,13 +4412,6 @@
           <t>jbaker@gac.org</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
-      <c r="M116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5107,13 +4442,6 @@
           <t>rhelms@gac.org</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
-      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5144,13 +4472,6 @@
           <t>uricketts@gac.org</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
-      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5181,13 +4502,6 @@
           <t>c.williams@leechristian.org</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
-      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -5218,13 +4532,6 @@
           <t>g.dykes@leechristian.org</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5255,13 +4562,6 @@
           <t>dwillis@metroca.com</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -5292,13 +4592,6 @@
           <t>jfeamster@metroca.com</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
-      <c r="M122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -5329,13 +4622,6 @@
           <t>kchenoweth@metroca.com</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
-      <c r="M123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -5366,13 +4652,6 @@
           <t>mbuffington@metroca.com</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -5403,13 +4682,6 @@
           <t>ksabia@northhillschristian.com</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -5440,13 +4712,6 @@
           <t>rpierce@northhillschristian.com</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
-      <c r="M126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -5477,13 +4742,6 @@
           <t>cgrimmer@phoenixchristian.org</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
-      <c r="M127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -5514,13 +4772,6 @@
           <t>csianturi@phoenixchristian.org</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
-      <c r="M128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -5551,13 +4802,6 @@
           <t>michelle.wilson@ranchochristian.org</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
-      <c r="M129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -5588,13 +4832,6 @@
           <t>nate.porter@ranchochristian.org</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
-      <c r="M130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -5625,13 +4862,6 @@
           <t>bspeier@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
-      <c r="M131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -5662,13 +4892,6 @@
           <t>jgross@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr"/>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
-      <c r="M132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -5699,13 +4922,6 @@
           <t>scairo@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
-      <c r="H133" t="inlineStr"/>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
-      <c r="M133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -5736,13 +4952,6 @@
           <t>mimel@tlcs.tlc.org</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
-      <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
-      <c r="M134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="n">
@@ -5826,23 +5035,23 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t>YES - Upper School curriculum director, wants to talk</t>
+          <t>YES - Upper School curriculum director, wants to talk; checking with Angela Adams (Bible dept chair) on her interest too</t>
         </is>
       </c>
       <c r="K136" s="2" t="inlineStr"/>
       <c r="L136" s="2" t="inlineStr">
         <is>
-          <t>Nudged 2026-09-17 for times</t>
+          <t>No times yet - she's checking with Angela and will respond soon (as of 2026-09-19)</t>
         </is>
       </c>
       <c r="M136" s="2" t="inlineStr">
         <is>
-          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
+          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up.</t>
         </is>
       </c>
     </row>
@@ -6446,9 +5655,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Tracker 2026-09-19: Donna Hurley checking with Angela, will send times
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$138</definedName>
@@ -649,6 +649,13 @@
           <t>alison.gioia@ashevillechristian.org</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -679,6 +686,13 @@
           <t>chris.zaccaro@ashevillechristian.org</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -709,6 +723,13 @@
           <t>kasey.murray@ashevillechristian.org</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -739,6 +760,13 @@
           <t>kate.lunberry@ashevillechristian.org</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -769,6 +797,13 @@
           <t>arudy@shoreschristian.org</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -799,6 +834,13 @@
           <t>ghall@shoreschristian.org</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -829,6 +871,13 @@
           <t>lreyes@shoreschristian.org</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -916,6 +965,13 @@
           <t>kelli.larsen@benlippen.com</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -946,6 +1002,13 @@
           <t>steve.maurelli@benlippen.com</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -976,6 +1039,13 @@
           <t>sheri_fyke@bereanwpb.org</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1006,6 +1076,13 @@
           <t>apeavy@bcamail.org</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1183,6 +1260,13 @@
           <t>goode@bocachristian.org</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1213,6 +1297,13 @@
           <t>fryk@bocachristian.org</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1243,6 +1334,13 @@
           <t>ashleykim@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1273,6 +1371,13 @@
           <t>carolynng@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1303,6 +1408,13 @@
           <t>helenyoolee@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1333,6 +1445,13 @@
           <t>jennylee@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1363,6 +1482,13 @@
           <t>stephenlim@crosspointacademy.org</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1393,6 +1519,13 @@
           <t>jreyes@calvarydowney.org</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1423,6 +1556,13 @@
           <t>jmcclintock@calvarydowney.org</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1453,6 +1593,13 @@
           <t>mmarquez@calvarydowney.org</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1483,6 +1630,13 @@
           <t>addyc@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1513,6 +1667,13 @@
           <t>davidd@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1543,6 +1704,13 @@
           <t>evak@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1695,6 +1863,13 @@
           <t>leac@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1725,6 +1900,13 @@
           <t>nikkib@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1755,6 +1937,13 @@
           <t>darylb@ccaeagles.org</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1785,6 +1974,13 @@
           <t>jperez@ccslancers.com</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1815,6 +2011,13 @@
           <t>sdiaz@ccslancers.com</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1845,6 +2048,13 @@
           <t>angelaguiton@cbckannapolis.com</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1875,6 +2085,13 @@
           <t>hornerb@chapel-hill.org</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1905,6 +2122,13 @@
           <t>kassie@chapel-hill.org</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1935,6 +2159,13 @@
           <t>freitask@chapel-hill.org</t>
         </is>
       </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1965,6 +2196,13 @@
           <t>ashley.jenkins@charchrist.com</t>
         </is>
       </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1995,6 +2233,13 @@
           <t>brandon.henderson@charchrist.com</t>
         </is>
       </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2025,6 +2270,13 @@
           <t>christina.sachtleben@charchrist.com</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -2100,6 +2352,13 @@
           <t>katey.balikian@charchrist.com</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -2232,6 +2491,13 @@
           <t>sneal@caschools.us</t>
         </is>
       </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2262,6 +2528,13 @@
           <t>acarson@caschools.us</t>
         </is>
       </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2292,6 +2565,13 @@
           <t>bwiley@caschools.us</t>
         </is>
       </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2322,6 +2602,13 @@
           <t>ctroyer@caschools.us</t>
         </is>
       </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2352,6 +2639,13 @@
           <t>cwallace@caschools.us</t>
         </is>
       </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -2472,6 +2766,13 @@
           <t>jgutierrez@caschools.us</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="inlineStr"/>
+      <c r="L56" t="inlineStr"/>
+      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2502,6 +2803,13 @@
           <t>lberg@caschools.us</t>
         </is>
       </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+      <c r="L57" t="inlineStr"/>
+      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2532,6 +2840,13 @@
           <t>mchitty@caschools.us</t>
         </is>
       </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+      <c r="L58" t="inlineStr"/>
+      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2562,6 +2877,13 @@
           <t>mcrawford@caschools.us</t>
         </is>
       </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+      <c r="L59" t="inlineStr"/>
+      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2592,6 +2914,13 @@
           <t>svincentz@caschools.us</t>
         </is>
       </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
+      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2622,6 +2951,13 @@
           <t>aengle@cfsknights.org</t>
         </is>
       </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+      <c r="L61" t="inlineStr"/>
+      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2652,6 +2988,13 @@
           <t>mclay@cfsknights.org</t>
         </is>
       </c>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr"/>
+      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2682,6 +3025,13 @@
           <t>shixon@cfsknights.org</t>
         </is>
       </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2712,6 +3062,13 @@
           <t>apetersen@chslions.com</t>
         </is>
       </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2742,6 +3099,13 @@
           <t>victoria.swing@concordchristian.org</t>
         </is>
       </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2772,6 +3136,13 @@
           <t>jstudt@concordchristianschool.org</t>
         </is>
       </c>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2802,6 +3173,13 @@
           <t>klittleton@concordchristianschool.org</t>
         </is>
       </c>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2832,6 +3210,13 @@
           <t>kmaddox@concordcs.org</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2862,6 +3247,13 @@
           <t>mark.clinton@cornerstonechristian.com</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2892,6 +3284,13 @@
           <t>ckronberger@crosshillchristian.com</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2922,6 +3321,13 @@
           <t>kmerina@crosshillchristian.com</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2952,6 +3358,13 @@
           <t>lkieling@crosshillchristian.com</t>
         </is>
       </c>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2982,6 +3395,13 @@
           <t>danielle.williams@cypresschristian.org</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3012,6 +3432,13 @@
           <t>erin.wilhelm@cypresschristian.org</t>
         </is>
       </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3042,6 +3469,13 @@
           <t>jessica.gates@cypresschristian.org</t>
         </is>
       </c>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -3129,6 +3563,13 @@
           <t>kjohnson@dayspringchristian.com</t>
         </is>
       </c>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3159,6 +3600,13 @@
           <t>shall@dhca.org</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3189,6 +3637,13 @@
           <t>emily.manuel@dmcs.org</t>
         </is>
       </c>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3219,6 +3674,13 @@
           <t>hnerem@dmcs.org</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr"/>
+      <c r="H80" t="inlineStr"/>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
+      <c r="K80" t="inlineStr"/>
+      <c r="L80" t="inlineStr"/>
+      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3249,6 +3711,13 @@
           <t>ksteen@dmcs.org</t>
         </is>
       </c>
+      <c r="G81" t="inlineStr"/>
+      <c r="H81" t="inlineStr"/>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
+      <c r="K81" t="inlineStr"/>
+      <c r="L81" t="inlineStr"/>
+      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3279,6 +3748,13 @@
           <t>lsteele@dmcs.org</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr"/>
+      <c r="H82" t="inlineStr"/>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
+      <c r="K82" t="inlineStr"/>
+      <c r="L82" t="inlineStr"/>
+      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3309,6 +3785,13 @@
           <t>slortz@dmcs.org</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr"/>
+      <c r="H83" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
+      <c r="K83" t="inlineStr"/>
+      <c r="L83" t="inlineStr"/>
+      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3339,6 +3822,13 @@
           <t>wweaver@dmcs.org</t>
         </is>
       </c>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
+      <c r="K84" t="inlineStr"/>
+      <c r="L84" t="inlineStr"/>
+      <c r="M84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -3590,6 +4080,13 @@
           <t>j_kughn@ehcseagles.com</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr"/>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+      <c r="K90" t="inlineStr"/>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3620,6 +4117,13 @@
           <t>tmm@elkhartchristian.org</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr"/>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+      <c r="K91" t="inlineStr"/>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3650,6 +4154,13 @@
           <t>awilliams@faithlafayette.org</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr"/>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+      <c r="K92" t="inlineStr"/>
+      <c r="L92" t="inlineStr"/>
+      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3680,6 +4191,13 @@
           <t>kkelso@faithlafayette.org</t>
         </is>
       </c>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+      <c r="K93" t="inlineStr"/>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3710,6 +4228,13 @@
           <t>erik.harris@fcspatriots.com</t>
         </is>
       </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+      <c r="K94" t="inlineStr"/>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3740,6 +4265,13 @@
           <t>jennifer.harris@fcspatriots.com</t>
         </is>
       </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+      <c r="K95" t="inlineStr"/>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3770,6 +4302,13 @@
           <t>jeremy.jones@fcspatriots.com</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
+      <c r="K96" t="inlineStr"/>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3800,6 +4339,13 @@
           <t>will.lamb@fcspatriots.com</t>
         </is>
       </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
+      <c r="K97" t="inlineStr"/>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3830,6 +4376,13 @@
           <t>danielle.reeves@fcspaladins.org</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
+      <c r="K98" t="inlineStr"/>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -3905,6 +4458,13 @@
           <t>michelle.eastman@fcspaladins.org</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
+      <c r="K100" t="inlineStr"/>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3935,6 +4495,13 @@
           <t>sherri.mcleroy@fcspaladins.org</t>
         </is>
       </c>
+      <c r="G101" t="inlineStr"/>
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
+      <c r="K101" t="inlineStr"/>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -3965,6 +4532,13 @@
           <t>cdavis@fbchighsprings.org</t>
         </is>
       </c>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
+      <c r="K102" t="inlineStr"/>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -3995,6 +4569,13 @@
           <t>spotter@fbchighsprings.org</t>
         </is>
       </c>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
+      <c r="K103" t="inlineStr"/>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -4025,6 +4606,13 @@
           <t>mrs.coleman@firstchristianacademy.com</t>
         </is>
       </c>
+      <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
+      <c r="K104" t="inlineStr"/>
+      <c r="L104" t="inlineStr"/>
+      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4055,6 +4643,13 @@
           <t>mrs.butler@firstchristianacademy.com</t>
         </is>
       </c>
+      <c r="G105" t="inlineStr"/>
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
+      <c r="K105" t="inlineStr"/>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4085,6 +4680,13 @@
           <t>lthompson@foothillchristian.org</t>
         </is>
       </c>
+      <c r="G106" t="inlineStr"/>
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
+      <c r="K106" t="inlineStr"/>
+      <c r="L106" t="inlineStr"/>
+      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4115,6 +4717,13 @@
           <t>lwilson@foothillchristian.org</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr"/>
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
+      <c r="K107" t="inlineStr"/>
+      <c r="L107" t="inlineStr"/>
+      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -4145,6 +4754,13 @@
           <t>rgutzwiller@foothillchristian.org</t>
         </is>
       </c>
+      <c r="G108" t="inlineStr"/>
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="inlineStr"/>
+      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4175,6 +4791,13 @@
           <t>brooke.newell@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G109" t="inlineStr"/>
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="inlineStr"/>
+      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -4205,6 +4828,13 @@
           <t>corey.cline@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4235,6 +4865,13 @@
           <t>jessica.meade@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G111" t="inlineStr"/>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr"/>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4265,6 +4902,13 @@
           <t>julie.daniel@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G112" t="inlineStr"/>
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+      <c r="K112" t="inlineStr"/>
+      <c r="L112" t="inlineStr"/>
+      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n">
@@ -4352,6 +4996,13 @@
           <t>thomas.rodriguez@foundationacademy.net</t>
         </is>
       </c>
+      <c r="G114" t="inlineStr"/>
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+      <c r="K114" t="inlineStr"/>
+      <c r="L114" t="inlineStr"/>
+      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -4382,6 +5033,13 @@
           <t>ajongko@gac.org</t>
         </is>
       </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+      <c r="K115" t="inlineStr"/>
+      <c r="L115" t="inlineStr"/>
+      <c r="M115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -4412,6 +5070,13 @@
           <t>jbaker@gac.org</t>
         </is>
       </c>
+      <c r="G116" t="inlineStr"/>
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+      <c r="K116" t="inlineStr"/>
+      <c r="L116" t="inlineStr"/>
+      <c r="M116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -4442,6 +5107,13 @@
           <t>rhelms@gac.org</t>
         </is>
       </c>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+      <c r="K117" t="inlineStr"/>
+      <c r="L117" t="inlineStr"/>
+      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -4472,6 +5144,13 @@
           <t>uricketts@gac.org</t>
         </is>
       </c>
+      <c r="G118" t="inlineStr"/>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+      <c r="K118" t="inlineStr"/>
+      <c r="L118" t="inlineStr"/>
+      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -4502,6 +5181,13 @@
           <t>c.williams@leechristian.org</t>
         </is>
       </c>
+      <c r="G119" t="inlineStr"/>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+      <c r="K119" t="inlineStr"/>
+      <c r="L119" t="inlineStr"/>
+      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -4532,6 +5218,13 @@
           <t>g.dykes@leechristian.org</t>
         </is>
       </c>
+      <c r="G120" t="inlineStr"/>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+      <c r="K120" t="inlineStr"/>
+      <c r="L120" t="inlineStr"/>
+      <c r="M120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -4562,6 +5255,13 @@
           <t>dwillis@metroca.com</t>
         </is>
       </c>
+      <c r="G121" t="inlineStr"/>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+      <c r="K121" t="inlineStr"/>
+      <c r="L121" t="inlineStr"/>
+      <c r="M121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -4592,6 +5292,13 @@
           <t>jfeamster@metroca.com</t>
         </is>
       </c>
+      <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+      <c r="K122" t="inlineStr"/>
+      <c r="L122" t="inlineStr"/>
+      <c r="M122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -4622,6 +5329,13 @@
           <t>kchenoweth@metroca.com</t>
         </is>
       </c>
+      <c r="G123" t="inlineStr"/>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+      <c r="K123" t="inlineStr"/>
+      <c r="L123" t="inlineStr"/>
+      <c r="M123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -4652,6 +5366,13 @@
           <t>mbuffington@metroca.com</t>
         </is>
       </c>
+      <c r="G124" t="inlineStr"/>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+      <c r="K124" t="inlineStr"/>
+      <c r="L124" t="inlineStr"/>
+      <c r="M124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -4682,6 +5403,13 @@
           <t>ksabia@northhillschristian.com</t>
         </is>
       </c>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+      <c r="K125" t="inlineStr"/>
+      <c r="L125" t="inlineStr"/>
+      <c r="M125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -4712,6 +5440,13 @@
           <t>rpierce@northhillschristian.com</t>
         </is>
       </c>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+      <c r="K126" t="inlineStr"/>
+      <c r="L126" t="inlineStr"/>
+      <c r="M126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -4742,6 +5477,13 @@
           <t>cgrimmer@phoenixchristian.org</t>
         </is>
       </c>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -4772,6 +5514,13 @@
           <t>csianturi@phoenixchristian.org</t>
         </is>
       </c>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+      <c r="K128" t="inlineStr"/>
+      <c r="L128" t="inlineStr"/>
+      <c r="M128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -4802,6 +5551,13 @@
           <t>michelle.wilson@ranchochristian.org</t>
         </is>
       </c>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+      <c r="K129" t="inlineStr"/>
+      <c r="L129" t="inlineStr"/>
+      <c r="M129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -4832,6 +5588,13 @@
           <t>nate.porter@ranchochristian.org</t>
         </is>
       </c>
+      <c r="G130" t="inlineStr"/>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+      <c r="K130" t="inlineStr"/>
+      <c r="L130" t="inlineStr"/>
+      <c r="M130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -4862,6 +5625,13 @@
           <t>bspeier@southfieldchristian.org</t>
         </is>
       </c>
+      <c r="G131" t="inlineStr"/>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+      <c r="K131" t="inlineStr"/>
+      <c r="L131" t="inlineStr"/>
+      <c r="M131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -4892,6 +5662,13 @@
           <t>jgross@southfieldchristian.org</t>
         </is>
       </c>
+      <c r="G132" t="inlineStr"/>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+      <c r="K132" t="inlineStr"/>
+      <c r="L132" t="inlineStr"/>
+      <c r="M132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -4922,6 +5699,13 @@
           <t>scairo@southfieldchristian.org</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr"/>
+      <c r="H133" t="inlineStr"/>
+      <c r="I133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+      <c r="K133" t="inlineStr"/>
+      <c r="L133" t="inlineStr"/>
+      <c r="M133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -4952,6 +5736,13 @@
           <t>mimel@tlcs.tlc.org</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr"/>
+      <c r="H134" t="inlineStr"/>
+      <c r="I134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+      <c r="K134" t="inlineStr"/>
+      <c r="L134" t="inlineStr"/>
+      <c r="M134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="n">
@@ -5046,12 +5837,12 @@
       <c r="K136" s="2" t="inlineStr"/>
       <c r="L136" s="2" t="inlineStr">
         <is>
-          <t>No times yet - she's checking with Angela and will respond soon (as of 2026-09-19)</t>
+          <t>Awaiting times - checking with Angela (as of 2026-09-19)</t>
         </is>
       </c>
       <c r="M136" s="2" t="inlineStr">
         <is>
-          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up.</t>
+          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up. | 2026-09-19: out of school recently; will check with Angela and follow up with times.</t>
         </is>
       </c>
     </row>
@@ -5635,7 +6426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5651,22 +6442,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-17: 137 contacts, 11 replied, 5 want in, 11 bounced.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Updated 2026-09-19: 137 contacts, 11 replied, 5 want in, 11 bounced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
           <t>Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution. Blue=referral.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Meredith Arldt sent availability (Pacific); Julianne Rettig deferred a few weeks.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker 2026-09-21: Meredith booked Thu Sep 24 11:00 PT (Google Meet)
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -46,7 +46,7 @@
       <color rgb="00666666"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -60,7 +60,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9EAD3"/>
+        <fgColor rgb="00B7E1CD"/>
       </patternFill>
     </fill>
     <fill>
@@ -71,6 +71,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
     <fill>
@@ -96,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -106,6 +111,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -488,7 +494,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="52" customWidth="1" min="12" max="12"/>
     <col width="66" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -611,12 +617,12 @@
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Availability (Pacific): next wk Mon/Thu/Fri 10-12 PT; following wk Mon/Wed 9-11 PT</t>
+          <t>BOOKED: Thu Sep 24 2026, 11:00 AM PT (2:00 PM ET) - Google Meet meet.google.com/hho-kmbi-aha</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule. | Scheduling nudge sent 2026-09-17 (asked for times). | Sent availability 2026-09-17 (Pacific). Propose a specific slot.</t>
+          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule. | Scheduling nudge sent 2026-09-17 (asked for times). | Sent availability 2026-09-17 (Pacific). Propose a specific slot. | 2026-09-21: booked Thu Sep 24 11:00 AM PT; calendar invite + confirmation sent.</t>
         </is>
       </c>
     </row>
@@ -1713,65 +1719,65 @@
       <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
+      <c r="A31" s="5" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Calvary Christian Academy - Ft Lauderdale</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Fort Lauderdale</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Julianne Rettig</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>julianner@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>YES — happy to help personally (or refer to MS Bible teachers)</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K31" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="L31" s="5" t="inlineStr">
         <is>
           <t>Deferred - off campus ~a few weeks (as of 2026-09-17); will follow up</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr">
+      <c r="M31" s="5" t="inlineStr">
         <is>
           <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-17: off campus a few weeks; will follow up.</t>
         </is>
@@ -3876,41 +3882,41 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="5" t="n">
+      <c r="A86" s="6" t="n">
         <v>85</v>
       </c>
-      <c r="B86" s="5" t="inlineStr">
+      <c r="B86" s="6" t="inlineStr">
         <is>
           <t>Eagle's Landing Christian Academy - Junior High</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr">
+      <c r="C86" s="6" t="inlineStr">
         <is>
           <t>McDonough</t>
         </is>
       </c>
-      <c r="D86" s="5" t="inlineStr">
+      <c r="D86" s="6" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E86" s="5" t="inlineStr">
+      <c r="E86" s="6" t="inlineStr">
         <is>
           <t>Cathie Kelly</t>
         </is>
       </c>
-      <c r="F86" s="5" t="inlineStr">
+      <c r="F86" s="6" t="inlineStr">
         <is>
           <t>cathie.kelly@eagleslanding.org</t>
         </is>
       </c>
-      <c r="G86" s="5" t="inlineStr"/>
-      <c r="H86" s="5" t="inlineStr"/>
-      <c r="I86" s="5" t="inlineStr"/>
-      <c r="J86" s="5" t="inlineStr"/>
-      <c r="K86" s="5" t="inlineStr"/>
-      <c r="L86" s="5" t="inlineStr"/>
-      <c r="M86" s="5" t="inlineStr">
+      <c r="G86" s="6" t="inlineStr"/>
+      <c r="H86" s="6" t="inlineStr"/>
+      <c r="I86" s="6" t="inlineStr"/>
+      <c r="J86" s="6" t="inlineStr"/>
+      <c r="K86" s="6" t="inlineStr"/>
+      <c r="L86" s="6" t="inlineStr"/>
+      <c r="M86" s="6" t="inlineStr">
         <is>
           <t>CAUTION: all other eagleslanding.org addresses bounced 2026-09-10; likely invalid.</t>
         </is>
@@ -5745,232 +5751,232 @@
       <c r="M134" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" s="6" t="n">
+      <c r="A135" s="7" t="n">
         <v>134</v>
       </c>
-      <c r="B135" s="6" t="inlineStr">
+      <c r="B135" s="7" t="inlineStr">
         <is>
           <t>Bethlehem Christian Academy - Elementary</t>
         </is>
       </c>
-      <c r="C135" s="6" t="inlineStr">
+      <c r="C135" s="7" t="inlineStr">
         <is>
           <t>Bethlehem</t>
         </is>
       </c>
-      <c r="D135" s="6" t="inlineStr">
+      <c r="D135" s="7" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E135" s="6" t="inlineStr">
+      <c r="E135" s="7" t="inlineStr">
         <is>
           <t>Shannon Jones</t>
         </is>
       </c>
-      <c r="F135" s="6" t="inlineStr">
+      <c r="F135" s="7" t="inlineStr">
         <is>
           <t>sjones@bcamail.org</t>
         </is>
       </c>
-      <c r="G135" s="6" t="inlineStr"/>
-      <c r="H135" s="6" t="inlineStr"/>
-      <c r="I135" s="6" t="inlineStr"/>
-      <c r="J135" s="6" t="inlineStr"/>
-      <c r="K135" s="6" t="inlineStr"/>
-      <c r="L135" s="6" t="inlineStr"/>
-      <c r="M135" s="6" t="inlineStr">
+      <c r="G135" s="7" t="inlineStr"/>
+      <c r="H135" s="7" t="inlineStr"/>
+      <c r="I135" s="7" t="inlineStr"/>
+      <c r="J135" s="7" t="inlineStr"/>
+      <c r="K135" s="7" t="inlineStr"/>
+      <c r="L135" s="7" t="inlineStr"/>
+      <c r="M135" s="7" t="inlineStr">
         <is>
           <t>REFERRAL from Kelly Vann (Bethlehem). Invitation sent 2026-09-10 (greeting "Shannon").</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n">
+      <c r="A136" s="5" t="n">
         <v>135</v>
       </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="B136" s="5" t="inlineStr">
         <is>
           <t>Dayspring Christian Academy</t>
         </is>
       </c>
-      <c r="C136" s="2" t="inlineStr">
+      <c r="C136" s="5" t="inlineStr">
         <is>
           <t>Mountville</t>
         </is>
       </c>
-      <c r="D136" s="2" t="inlineStr">
+      <c r="D136" s="5" t="inlineStr">
         <is>
           <t>PA</t>
         </is>
       </c>
-      <c r="E136" s="2" t="inlineStr">
+      <c r="E136" s="5" t="inlineStr">
         <is>
           <t>Donna Hurley</t>
         </is>
       </c>
-      <c r="F136" s="2" t="inlineStr">
+      <c r="F136" s="5" t="inlineStr">
         <is>
           <t>dhurley@dayspringchristian.com</t>
         </is>
       </c>
-      <c r="G136" s="2" t="inlineStr">
+      <c r="G136" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H136" s="2" t="inlineStr">
+      <c r="H136" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I136" s="2" t="inlineStr">
+      <c r="I136" s="5" t="inlineStr">
         <is>
           <t>2026-09-19</t>
         </is>
       </c>
-      <c r="J136" s="2" t="inlineStr">
+      <c r="J136" s="5" t="inlineStr">
         <is>
           <t>YES - Upper School curriculum director, wants to talk; checking with Angela Adams (Bible dept chair) on her interest too</t>
         </is>
       </c>
-      <c r="K136" s="2" t="inlineStr"/>
-      <c r="L136" s="2" t="inlineStr">
+      <c r="K136" s="5" t="inlineStr"/>
+      <c r="L136" s="5" t="inlineStr">
         <is>
           <t>Awaiting times - checking with Angela (as of 2026-09-19)</t>
         </is>
       </c>
-      <c r="M136" s="2" t="inlineStr">
+      <c r="M136" s="5" t="inlineStr">
         <is>
           <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up. | 2026-09-19: out of school recently; will check with Angela and follow up with times.</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n">
+      <c r="A137" s="5" t="n">
         <v>136</v>
       </c>
-      <c r="B137" s="2" t="inlineStr">
+      <c r="B137" s="5" t="inlineStr">
         <is>
           <t>Foundation Academy</t>
         </is>
       </c>
-      <c r="C137" s="2" t="inlineStr">
+      <c r="C137" s="5" t="inlineStr">
         <is>
           <t>Winter Garden</t>
         </is>
       </c>
-      <c r="D137" s="2" t="inlineStr">
+      <c r="D137" s="5" t="inlineStr">
         <is>
           <t>FL</t>
         </is>
       </c>
-      <c r="E137" s="2" t="inlineStr">
+      <c r="E137" s="5" t="inlineStr">
         <is>
           <t>Diana Helton</t>
         </is>
       </c>
-      <c r="F137" s="2" t="inlineStr">
+      <c r="F137" s="5" t="inlineStr">
         <is>
           <t>diana.helton@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G137" s="2" t="inlineStr">
+      <c r="G137" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H137" s="2" t="inlineStr">
+      <c r="H137" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I137" s="2" t="inlineStr">
+      <c r="I137" s="5" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="J137" s="2" t="inlineStr">
+      <c r="J137" s="5" t="inlineStr">
         <is>
           <t>YES - happy to help (elementary)</t>
         </is>
       </c>
-      <c r="K137" s="2" t="inlineStr">
+      <c r="K137" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L137" s="2" t="inlineStr">
+      <c r="L137" s="5" t="inlineStr">
         <is>
           <t>Nudged 2026-09-17 for times</t>
         </is>
       </c>
-      <c r="M137" s="2" t="inlineStr">
+      <c r="M137" s="5" t="inlineStr">
         <is>
           <t>Round 1 contact; agreed 2026-09-11 and questions sent 2026-09-11. Also referred by Tanya Murphy. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
         </is>
       </c>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n">
+      <c r="A138" s="5" t="n">
         <v>137</v>
       </c>
-      <c r="B138" s="2" t="inlineStr">
+      <c r="B138" s="5" t="inlineStr">
         <is>
           <t>Christian Academy of Indiana</t>
         </is>
       </c>
-      <c r="C138" s="2" t="inlineStr">
+      <c r="C138" s="5" t="inlineStr">
         <is>
           <t>New Albany</t>
         </is>
       </c>
-      <c r="D138" s="2" t="inlineStr">
+      <c r="D138" s="5" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="E138" s="2" t="inlineStr">
+      <c r="E138" s="5" t="inlineStr">
         <is>
           <t>Wendy Wagoner</t>
         </is>
       </c>
-      <c r="F138" s="2" t="inlineStr">
+      <c r="F138" s="5" t="inlineStr">
         <is>
           <t>wwagoner@caschools.us</t>
         </is>
       </c>
-      <c r="G138" s="2" t="inlineStr">
+      <c r="G138" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H138" s="2" t="inlineStr">
+      <c r="H138" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I138" s="2" t="inlineStr">
+      <c r="I138" s="5" t="inlineStr">
         <is>
           <t>2026-09-16</t>
         </is>
       </c>
-      <c r="J138" s="2" t="inlineStr">
+      <c r="J138" s="5" t="inlineStr">
         <is>
           <t>YES - happy to help</t>
         </is>
       </c>
-      <c r="K138" s="2" t="inlineStr">
+      <c r="K138" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L138" s="2" t="inlineStr">
+      <c r="L138" s="5" t="inlineStr">
         <is>
           <t>Nudged 2026-09-17 for times</t>
         </is>
       </c>
-      <c r="M138" s="2" t="inlineStr">
+      <c r="M138" s="5" t="inlineStr">
         <is>
           <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
         </is>
@@ -5996,14 +6002,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Questions Preview Email</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Marketing &amp; Sales</t>
         </is>
@@ -6017,7 +6023,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Options: 5-8? / 6-8? / 7-8?</t>
         </is>
@@ -6031,7 +6037,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Options: Developmentally? / Spiritually? / Emotionally?</t>
         </is>
@@ -6073,7 +6079,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>Editorial</t>
         </is>
@@ -6087,7 +6093,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Options: Teaching / Reading / Discussion time / Activities</t>
         </is>
@@ -6101,7 +6107,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
         </is>
@@ -6115,7 +6121,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Options: To project images and other teaching materials / To play educational videos / Other</t>
         </is>
@@ -6129,7 +6135,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Options: in 6th grade? / in 7th grade? / in 8th grade?</t>
         </is>
@@ -6143,7 +6149,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -6164,14 +6170,14 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Options: 6th / 7th / 8th</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>Production</t>
         </is>
@@ -6192,7 +6198,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Options: 30 seconds -1min / 1 min-2min / 2 min-3min / 3 minutes +</t>
         </is>
@@ -6206,7 +6212,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>Options: Photography / Illustrations / Infographics/diagrams / Maps and timelines / Historical artwork / Charts and visual explanations / Short-form comics or graphic storytelling / Other</t>
         </is>
@@ -6227,7 +6233,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="10" t="inlineStr">
         <is>
           <t>Options: Mostly visual, with short amounts of text / A balanced mix of text and visuals / Mostly text, with visuals used to support key concepts / It depends on the lesson</t>
         </is>
@@ -6255,7 +6261,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>Additional Questions</t>
         </is>
@@ -6276,7 +6282,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -6304,7 +6310,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="9" t="inlineStr">
+      <c r="B46" s="10" t="inlineStr">
         <is>
           <t>Options: In school with boys taught by a male teacher and girls taught by a female teacher, with advance permission from parents / Sent home to parents as a resource to use with their own child as they see fit / We would not use it at our school or send it home to parents.</t>
         </is>
@@ -6318,7 +6324,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B48" s="10" t="inlineStr">
         <is>
           <t>Options: Yes / No / Maybe</t>
         </is>
@@ -6332,7 +6338,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="9" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>Options: Discussions / Alternate in-depth videos / Journaling prompts / Further Bible reading / Other activities</t>
         </is>
@@ -6381,7 +6387,7 @@
       </c>
     </row>
     <row r="57">
-      <c r="B57" s="9" t="inlineStr">
+      <c r="B57" s="10" t="inlineStr">
         <is>
           <t>Options: Videos that tie the lesson into real world application / Videos that hit on the key idea of the lesson / Videos that introduce the subject matter before teaching</t>
         </is>
@@ -6433,7 +6439,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>DeepRoots — Middle School Round 2 Response Tracker</t>
         </is>
@@ -6442,7 +6448,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-19: 137 contacts, 11 replied, 5 want in, 11 bounced.</t>
+          <t>Updated 2026-09-21: 137 contacts, 11 replied, 5 want in, 1 booked, 11 bounced.</t>
         </is>
       </c>
     </row>
@@ -6452,7 +6458,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution. Blue=referral.</t>
+          <t>Teal=call booked. Green=wants in. Grey=replied/declined. Red=bounced. Yellow=caution. Blue=referral.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tracker check 2026-09-24: Will Weaver (DMCS) replied, proposed times
Will Weaver (Head of Spiritual Formation, Des Moines Christian School)
replied wanting to take part and offered 2:30 PM Mon/Tue/Wed next week.
Flagged to confirm a day and send the questions-preview email.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MT7SzDEasnvgyeSqBQh4RV
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$138</definedName>
@@ -46,7 +46,7 @@
       <color rgb="00666666"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +88,12 @@
         <fgColor rgb="00DEEAF6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+        <bgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -101,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -115,6 +121,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -655,13 +662,6 @@
           <t>alison.gioia@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -692,13 +692,6 @@
           <t>chris.zaccaro@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -729,13 +722,6 @@
           <t>kasey.murray@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -766,13 +752,6 @@
           <t>kate.lunberry@ashevillechristian.org</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -803,13 +782,6 @@
           <t>arudy@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -840,13 +812,6 @@
           <t>ghall@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -877,13 +842,6 @@
           <t>lreyes@shoreschristian.org</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -971,13 +929,6 @@
           <t>kelli.larsen@benlippen.com</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1008,13 +959,6 @@
           <t>steve.maurelli@benlippen.com</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1045,13 +989,6 @@
           <t>sheri_fyke@bereanwpb.org</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1082,13 +1019,6 @@
           <t>apeavy@bcamail.org</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -1266,13 +1196,6 @@
           <t>goode@bocachristian.org</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1303,13 +1226,6 @@
           <t>fryk@bocachristian.org</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1340,13 +1256,6 @@
           <t>ashleykim@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1377,13 +1286,6 @@
           <t>carolynng@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1414,13 +1316,6 @@
           <t>helenyoolee@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1451,13 +1346,6 @@
           <t>jennylee@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
-      <c r="M23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1488,13 +1376,6 @@
           <t>stephenlim@crosspointacademy.org</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
-      <c r="L24" t="inlineStr"/>
-      <c r="M24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1525,13 +1406,6 @@
           <t>jreyes@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1562,13 +1436,6 @@
           <t>jmcclintock@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
-      <c r="L26" t="inlineStr"/>
-      <c r="M26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1599,13 +1466,6 @@
           <t>mmarquez@calvarydowney.org</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
-      <c r="L27" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1636,13 +1496,6 @@
           <t>addyc@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1673,13 +1526,6 @@
           <t>davidd@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr"/>
-      <c r="M29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1710,13 +1556,6 @@
           <t>evak@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
-      <c r="L30" t="inlineStr"/>
-      <c r="M30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
@@ -1869,13 +1708,6 @@
           <t>leac@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1906,13 +1738,6 @@
           <t>nikkib@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
-      <c r="L34" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1943,13 +1768,6 @@
           <t>darylb@ccaeagles.org</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1980,13 +1798,6 @@
           <t>jperez@ccslancers.com</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
-      <c r="L36" t="inlineStr"/>
-      <c r="M36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2017,13 +1828,6 @@
           <t>sdiaz@ccslancers.com</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
-      <c r="L37" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2054,13 +1858,6 @@
           <t>angelaguiton@cbckannapolis.com</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
-      <c r="L38" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2091,13 +1888,6 @@
           <t>hornerb@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2128,13 +1918,6 @@
           <t>kassie@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
-      <c r="L40" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2165,13 +1948,6 @@
           <t>freitask@chapel-hill.org</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2202,13 +1978,6 @@
           <t>ashley.jenkins@charchrist.com</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2239,13 +2008,6 @@
           <t>brandon.henderson@charchrist.com</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2276,13 +2038,6 @@
           <t>christina.sachtleben@charchrist.com</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -2358,13 +2113,6 @@
           <t>katey.balikian@charchrist.com</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
-      <c r="L46" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -2497,13 +2245,6 @@
           <t>sneal@caschools.us</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2534,13 +2275,6 @@
           <t>acarson@caschools.us</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2571,13 +2305,6 @@
           <t>bwiley@caschools.us</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2608,13 +2335,6 @@
           <t>ctroyer@caschools.us</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2645,13 +2365,6 @@
           <t>cwallace@caschools.us</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n">
@@ -2772,13 +2485,6 @@
           <t>jgutierrez@caschools.us</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2809,13 +2515,6 @@
           <t>lberg@caschools.us</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2846,13 +2545,6 @@
           <t>mchitty@caschools.us</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr"/>
-      <c r="M58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2883,13 +2575,6 @@
           <t>mcrawford@caschools.us</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr"/>
-      <c r="M59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2920,13 +2605,6 @@
           <t>svincentz@caschools.us</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr"/>
-      <c r="M60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2957,13 +2635,6 @@
           <t>aengle@cfsknights.org</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr"/>
-      <c r="M61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2994,13 +2665,6 @@
           <t>mclay@cfsknights.org</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
-      <c r="K62" t="inlineStr"/>
-      <c r="L62" t="inlineStr"/>
-      <c r="M62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3031,13 +2695,6 @@
           <t>shixon@cfsknights.org</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3068,13 +2725,6 @@
           <t>apetersen@chslions.com</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3105,13 +2755,6 @@
           <t>victoria.swing@concordchristian.org</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
-      <c r="K65" t="inlineStr"/>
-      <c r="L65" t="inlineStr"/>
-      <c r="M65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3142,13 +2785,6 @@
           <t>jstudt@concordchristianschool.org</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
-      <c r="K66" t="inlineStr"/>
-      <c r="L66" t="inlineStr"/>
-      <c r="M66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3179,13 +2815,6 @@
           <t>klittleton@concordchristianschool.org</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
-      <c r="K67" t="inlineStr"/>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3216,13 +2845,6 @@
           <t>kmaddox@concordcs.org</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr"/>
-      <c r="M68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3253,13 +2875,6 @@
           <t>mark.clinton@cornerstonechristian.com</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr"/>
-      <c r="M69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3290,13 +2905,6 @@
           <t>ckronberger@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3327,13 +2935,6 @@
           <t>kmerina@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
-      <c r="K71" t="inlineStr"/>
-      <c r="L71" t="inlineStr"/>
-      <c r="M71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3364,13 +2965,6 @@
           <t>lkieling@crosshillchristian.com</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -3401,13 +2995,6 @@
           <t>danielle.williams@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3438,13 +3025,6 @@
           <t>erin.wilhelm@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3475,13 +3055,6 @@
           <t>jessica.gates@cypresschristian.org</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -3569,13 +3142,6 @@
           <t>kjohnson@dayspringchristian.com</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3606,13 +3172,6 @@
           <t>shall@dhca.org</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3643,13 +3202,6 @@
           <t>emily.manuel@dmcs.org</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3680,13 +3232,6 @@
           <t>hnerem@dmcs.org</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3717,13 +3262,6 @@
           <t>ksteen@dmcs.org</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
-      <c r="H81" t="inlineStr"/>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3754,13 +3292,6 @@
           <t>lsteele@dmcs.org</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
-      <c r="H82" t="inlineStr"/>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3791,50 +3322,67 @@
           <t>slortz@dmcs.org</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
-      <c r="H83" t="inlineStr"/>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" t="n">
+      <c r="A84" s="11" t="n">
         <v>83</v>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B84" s="11" t="inlineStr">
         <is>
           <t>Des Moines Christian School</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="11" t="inlineStr">
         <is>
           <t>Urbandale</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D84" s="11" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E84" s="11" t="inlineStr">
         <is>
           <t>Will Weaver</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F84" s="11" t="inlineStr">
         <is>
           <t>wweaver@dmcs.org</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
+      <c r="G84" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="H84" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I84" s="11" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="J84" s="11" t="inlineStr">
+        <is>
+          <t>YES - proposed times, awaiting confirmation</t>
+        </is>
+      </c>
+      <c r="K84" s="11" t="n"/>
+      <c r="L84" s="11" t="inlineStr">
+        <is>
+          <t>Proposed: 2:30 PM each day next Mon/Tue/Wed (Sep 28-30 2026, his local = Urbandale IA / Central). Awaiting our confirmation of a specific day.</t>
+        </is>
+      </c>
+      <c r="M84" s="11" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-24 (title: Head of Spiritual Formation): "If you're still looking for feedback, I have availability at 2:30pm each day next Monday, Tuesday, and Wednesday. Let me know if one of those works for you." FLAG: pick a day, confirm time (convert 2:30 PM CT), and send questions-preview email + calendar invite.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
@@ -4086,13 +3634,6 @@
           <t>j_kughn@ehcseagles.com</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -4123,13 +3664,6 @@
           <t>tmm@elkhartchristian.org</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4160,13 +3694,6 @@
           <t>awilliams@faithlafayette.org</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -4197,13 +3724,6 @@
           <t>kkelso@faithlafayette.org</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -4234,13 +3754,6 @@
           <t>erik.harris@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -4271,13 +3784,6 @@
           <t>jennifer.harris@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr"/>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -4308,13 +3814,6 @@
           <t>jeremy.jones@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -4345,13 +3844,6 @@
           <t>will.lamb@fcspatriots.com</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -4382,13 +3874,6 @@
           <t>danielle.reeves@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n">
@@ -4464,13 +3949,6 @@
           <t>michelle.eastman@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -4501,13 +3979,6 @@
           <t>sherri.mcleroy@fcspaladins.org</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -4538,13 +4009,6 @@
           <t>cdavis@fbchighsprings.org</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
-      <c r="M102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -4575,13 +4039,6 @@
           <t>spotter@fbchighsprings.org</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
-      <c r="M103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -4612,13 +4069,6 @@
           <t>mrs.coleman@firstchristianacademy.com</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4649,13 +4099,6 @@
           <t>mrs.butler@firstchristianacademy.com</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
-      <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
-      <c r="M105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4686,13 +4129,6 @@
           <t>lthompson@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
-      <c r="M106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4723,13 +4159,6 @@
           <t>lwilson@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
-      <c r="M107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -4760,13 +4189,6 @@
           <t>rgutzwiller@foothillchristian.org</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr"/>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
-      <c r="M108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4797,13 +4219,6 @@
           <t>brooke.newell@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr"/>
-      <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
-      <c r="M109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -4834,13 +4249,6 @@
           <t>corey.cline@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr"/>
-      <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
-      <c r="M110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4871,13 +4279,6 @@
           <t>jessica.meade@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr"/>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
-      <c r="M111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4908,13 +4309,6 @@
           <t>julie.daniel@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr"/>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
-      <c r="M112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n">
@@ -5002,13 +4396,6 @@
           <t>thomas.rodriguez@foundationacademy.net</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
-      <c r="M114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -5039,13 +4426,6 @@
           <t>ajongko@gac.org</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
-      <c r="M115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -5076,13 +4456,6 @@
           <t>jbaker@gac.org</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
-      <c r="M116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -5113,13 +4486,6 @@
           <t>rhelms@gac.org</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
-      <c r="M117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -5150,13 +4516,6 @@
           <t>uricketts@gac.org</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
-      <c r="M118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -5187,13 +4546,6 @@
           <t>c.williams@leechristian.org</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
-      <c r="M119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -5224,13 +4576,6 @@
           <t>g.dykes@leechristian.org</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
-      <c r="H120" t="inlineStr"/>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
-      <c r="M120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -5261,13 +4606,6 @@
           <t>dwillis@metroca.com</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
-      <c r="H121" t="inlineStr"/>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
-      <c r="M121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -5298,13 +4636,6 @@
           <t>jfeamster@metroca.com</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
-      <c r="H122" t="inlineStr"/>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
-      <c r="M122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -5335,13 +4666,6 @@
           <t>kchenoweth@metroca.com</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
-      <c r="H123" t="inlineStr"/>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
-      <c r="M123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -5372,13 +4696,6 @@
           <t>mbuffington@metroca.com</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr"/>
-      <c r="H124" t="inlineStr"/>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
-      <c r="M124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -5409,13 +4726,6 @@
           <t>ksabia@northhillschristian.com</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
-      <c r="H125" t="inlineStr"/>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
-      <c r="M125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -5446,13 +4756,6 @@
           <t>rpierce@northhillschristian.com</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
-      <c r="H126" t="inlineStr"/>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
-      <c r="M126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -5483,13 +4786,6 @@
           <t>cgrimmer@phoenixchristian.org</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr"/>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
-      <c r="M127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -5520,13 +4816,6 @@
           <t>csianturi@phoenixchristian.org</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr"/>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
-      <c r="M128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -5557,13 +4846,6 @@
           <t>michelle.wilson@ranchochristian.org</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr"/>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
-      <c r="M129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -5594,13 +4876,6 @@
           <t>nate.porter@ranchochristian.org</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr"/>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
-      <c r="M130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -5631,13 +4906,6 @@
           <t>bspeier@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr"/>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
-      <c r="M131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -5668,13 +4936,6 @@
           <t>jgross@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr"/>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
-      <c r="M132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -5705,13 +4966,6 @@
           <t>scairo@southfieldchristian.org</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
-      <c r="H133" t="inlineStr"/>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
-      <c r="M133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -5742,13 +4996,6 @@
           <t>mimel@tlcs.tlc.org</t>
         </is>
       </c>
-      <c r="G134" t="inlineStr"/>
-      <c r="H134" t="inlineStr"/>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
-      <c r="L134" t="inlineStr"/>
-      <c r="M134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="7" t="n">
@@ -6452,9 +5699,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Daily reply check: log Meredith Arldt's post-interview thank-you, sync tracker files
Gmail search (in:inbox newer_than:8d) matched senders against the 138
tracked addresses. All matches were from already-tracked contacts; the
only genuinely new correspondence was Meredith Arldt's post-interview
thank-you note (2026-09-24), added to her notes in tracker_state.json.

Also regenerated response_tracker.csv and the xlsx from tracker_state.json,
which had drifted out of sync with several already-logged updates
(Julianne Rettig, Will Weaver, Donna Hurley, Diana Helton, Wendy Wagoner
meeting/notes fields, and the missing Carrie Feitl row).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TtozSZr3EiQV3RXxT13b9Y
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$139</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -487,7 +487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M138"/>
+  <dimension ref="A1:M139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -573,63 +573,63 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Aliso Viejo Christian School</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Aliso Viejo</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>Meredith Arldt</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>marldt@avchristianschool.org</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>YES — happy to take part</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>BOOKED: Thu Sep 24 2026, 11:00 AM PT (2:00 PM ET) - Google Meet meet.google.com/hho-kmbi-aha</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule. | Scheduling nudge sent 2026-09-17 (asked for times). | Sent availability 2026-09-17 (Pacific). Propose a specific slot. | 2026-09-21: booked Thu Sep 24 11:00 AM PT; calendar invite + confirmation sent.</t>
+      <c r="K2" s="5" t="n"/>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>BOOKED: Thu Sep 24 2026, 11:00 AM PT (2:00 PM ET) - Google Meet meet.google.com/vzx-fphv-kga - on work calendar (tdwinkler@deeprootsbible.com); Pat Williamson added as attendee</t>
+        </is>
+      </c>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule. | Scheduling nudge sent 2026-09-17 (asked for times). | Sent availability 2026-09-17 (Pacific). Propose a specific slot. | 2026-09-21: booked Thu Sep 24 11:00 AM PT; calendar invite + confirmation sent. | 2026-09-21: moved event to work calendar (tdwinkler@deeprootsbible.com), added Pat Williamson; new Meet link vzx-fphv-kga. | 2026-09-24: Interview held. Meredith replied same day with a thank-you note, apologizing for the call running long (past the planned 30 min) and offering to be available for any future follow-up questions. No action needed.</t>
         </is>
       </c>
     </row>
@@ -892,8 +892,8 @@
           <t>No — elementary educator</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="n"/>
+      <c r="L10" s="3" t="n"/>
       <c r="M10" s="3" t="inlineStr">
         <is>
           <t>Replied 2026-09-10: elementary educator, never taught middle school; declined.</t>
@@ -1054,11 +1054,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr"/>
-      <c r="I15" s="4" t="inlineStr"/>
-      <c r="J15" s="4" t="inlineStr"/>
-      <c r="K15" s="4" t="inlineStr"/>
-      <c r="L15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="4" t="n"/>
+      <c r="L15" s="4" t="n"/>
       <c r="M15" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: address not found at bcamail.org.</t>
@@ -1099,11 +1099,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
+      <c r="K16" s="4" t="n"/>
+      <c r="L16" s="4" t="n"/>
       <c r="M16" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: address not found at bcamail.org.</t>
@@ -1159,8 +1159,8 @@
           <t>No — works with K3–5th; referral</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="inlineStr">
         <is>
           <t>Replied 2026-09-10: works with K3-5th, suggested a better-fit contact (cc SJones@bcamail.org).</t>
@@ -1613,12 +1613,12 @@
       </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
-          <t>Deferred - off campus ~a few weeks (as of 2026-09-17); will follow up</t>
+          <t>Deferred (off campus a few weeks per 2026-09-17); patient follow-up drafted 2026-09-21, HOLD to send ~early Oct</t>
         </is>
       </c>
       <c r="M31" s="5" t="inlineStr">
         <is>
-          <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-17: off campus a few weeks; will follow up.</t>
+          <t>Replied 2026-09-11 (on the forwarded Kathy Agarth thread, since Kathy has retired and her mail auto-forwards to Julianne): "I would be happy to help personally or direct you to our MS Bible teachers." No specific times proposed yet. FLAG: send questions-preview email + ask for times next. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-17: off campus a few weeks; will follow up. | 2026-09-21: drafted patient no-rush follow-up (ready in Drafts); recommend holding until ~early October since she said she would follow up when back.</t>
         </is>
       </c>
     </row>
@@ -1671,8 +1671,8 @@
           <t>N/A — retired; referred to Julianne Rettig (n=30, also on list)</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr"/>
-      <c r="L32" s="3" t="inlineStr"/>
+      <c r="K32" s="3" t="n"/>
+      <c r="L32" s="3" t="n"/>
       <c r="M32" s="3" t="inlineStr">
         <is>
           <t>Reply received 2026-09-11 from Julianne Rettig (Director of Upper School Academics), who now receives Kathy's auto-forwarded mail since Kathy has retired: Julianne offered to help personally or connect us with the MS Bible teachers. Treat Julianne (n=30) as the active contact for this thread; no action needed on Kathy's address.</t>
@@ -2073,11 +2073,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H45" s="4" t="inlineStr"/>
-      <c r="I45" s="4" t="inlineStr"/>
-      <c r="J45" s="4" t="inlineStr"/>
-      <c r="K45" s="4" t="inlineStr"/>
-      <c r="L45" s="4" t="inlineStr"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="n"/>
+      <c r="K45" s="4" t="n"/>
+      <c r="L45" s="4" t="n"/>
       <c r="M45" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: address not found (550 5.2.1).</t>
@@ -2148,11 +2148,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr"/>
-      <c r="J47" s="4" t="inlineStr"/>
-      <c r="K47" s="4" t="inlineStr"/>
-      <c r="L47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="n"/>
+      <c r="I47" s="4" t="n"/>
+      <c r="J47" s="4" t="n"/>
+      <c r="K47" s="4" t="n"/>
+      <c r="L47" s="4" t="n"/>
       <c r="M47" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: rejected by caschools.us mail gateway (Paubox).</t>
@@ -2208,8 +2208,8 @@
           <t>No - K-12 ELL teacher, not a fit</t>
         </is>
       </c>
-      <c r="K48" s="3" t="inlineStr"/>
-      <c r="L48" s="3" t="inlineStr"/>
+      <c r="K48" s="3" t="n"/>
+      <c r="L48" s="3" t="n"/>
       <c r="M48" s="3" t="inlineStr">
         <is>
           <t>Replied 2026-09-10: teaches ELL in small pull-out groups; does not think it is a good fit.</t>
@@ -2400,11 +2400,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H54" s="4" t="inlineStr"/>
-      <c r="I54" s="4" t="inlineStr"/>
-      <c r="J54" s="4" t="inlineStr"/>
-      <c r="K54" s="4" t="inlineStr"/>
-      <c r="L54" s="4" t="inlineStr"/>
+      <c r="H54" s="4" t="n"/>
+      <c r="I54" s="4" t="n"/>
+      <c r="J54" s="4" t="n"/>
+      <c r="K54" s="4" t="n"/>
+      <c r="L54" s="4" t="n"/>
       <c r="M54" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: rejected by caschools.us mail gateway (Paubox).</t>
@@ -2445,11 +2445,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H55" s="4" t="inlineStr"/>
-      <c r="I55" s="4" t="inlineStr"/>
-      <c r="J55" s="4" t="inlineStr"/>
-      <c r="K55" s="4" t="inlineStr"/>
-      <c r="L55" s="4" t="inlineStr"/>
+      <c r="H55" s="4" t="n"/>
+      <c r="I55" s="4" t="n"/>
+      <c r="J55" s="4" t="n"/>
+      <c r="K55" s="4" t="n"/>
+      <c r="L55" s="4" t="n"/>
       <c r="M55" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: rejected by caschools.us mail gateway (Paubox).</t>
@@ -3105,8 +3105,8 @@
           <t>Referral -&gt; Donna Hurley (Upper School curriculum director)</t>
         </is>
       </c>
-      <c r="K76" s="3" t="inlineStr"/>
-      <c r="L76" s="3" t="inlineStr"/>
+      <c r="K76" s="3" t="n"/>
+      <c r="L76" s="3" t="n"/>
       <c r="M76" s="3" t="inlineStr">
         <is>
           <t>Replied 2026-09-14: referred Donna Hurley (dhurley@dayspringchristian.com), who would love to talk. Troy engaged both 2026-09-14.</t>
@@ -3324,63 +3324,63 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="11" t="n">
+      <c r="A84" s="5" t="n">
         <v>83</v>
       </c>
-      <c r="B84" s="11" t="inlineStr">
+      <c r="B84" s="5" t="inlineStr">
         <is>
           <t>Des Moines Christian School</t>
         </is>
       </c>
-      <c r="C84" s="11" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>Urbandale</t>
         </is>
       </c>
-      <c r="D84" s="11" t="inlineStr">
+      <c r="D84" s="5" t="inlineStr">
         <is>
           <t>IA</t>
         </is>
       </c>
-      <c r="E84" s="11" t="inlineStr">
+      <c r="E84" s="5" t="inlineStr">
         <is>
           <t>Will Weaver</t>
         </is>
       </c>
-      <c r="F84" s="11" t="inlineStr">
+      <c r="F84" s="5" t="inlineStr">
         <is>
           <t>wweaver@dmcs.org</t>
         </is>
       </c>
-      <c r="G84" s="11" t="inlineStr">
+      <c r="G84" s="5" t="inlineStr">
         <is>
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H84" s="11" t="inlineStr">
+      <c r="H84" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I84" s="11" t="inlineStr">
+      <c r="I84" s="5" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="J84" s="11" t="inlineStr">
-        <is>
-          <t>YES - proposed times, awaiting confirmation</t>
-        </is>
-      </c>
-      <c r="K84" s="11" t="n"/>
-      <c r="L84" s="11" t="inlineStr">
-        <is>
-          <t>Proposed: 2:30 PM each day next Mon/Tue/Wed (Sep 28-30 2026, his local = Urbandale IA / Central). Awaiting our confirmation of a specific day.</t>
-        </is>
-      </c>
-      <c r="M84" s="11" t="inlineStr">
-        <is>
-          <t>Replied 2026-09-24 (title: Head of Spiritual Formation): "If you're still looking for feedback, I have availability at 2:30pm each day next Monday, Tuesday, and Wednesday. Let me know if one of those works for you." FLAG: pick a day, confirm time (convert 2:30 PM CT), and send questions-preview email + calendar invite.</t>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>YES — proposed times, awaiting confirmation</t>
+        </is>
+      </c>
+      <c r="K84" s="5" t="n"/>
+      <c r="L84" s="5" t="inlineStr">
+        <is>
+          <t>BOOKED: Wed Sep 30 2026, 2:30 PM CT (3:30 PM ET) - Google Meet meet.google.com/fph-jmfv-gjt - work calendar; Pat Williamson attendee</t>
+        </is>
+      </c>
+      <c r="M84" s="5" t="inlineStr">
+        <is>
+          <t>Replied 2026-09-24 (title: Head of Spiritual Formation): "If you're still looking for feedback, I have availability at 2:30pm each day next Monday, Tuesday, and Wednesday. Let me know if one of those works for you." FLAG: pick a day, confirm time (convert 2:30 PM CT), and send questions-preview email + calendar invite. | 2026-09-24: Troy confirmed Wed Sep 30 2:30 PM CT (cc Pat); booked on work calendar w/ Meet link + Pat.</t>
         </is>
       </c>
     </row>
@@ -3418,11 +3418,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H85" s="4" t="inlineStr"/>
-      <c r="I85" s="4" t="inlineStr"/>
-      <c r="J85" s="4" t="inlineStr"/>
-      <c r="K85" s="4" t="inlineStr"/>
-      <c r="L85" s="4" t="inlineStr"/>
+      <c r="H85" s="4" t="n"/>
+      <c r="I85" s="4" t="n"/>
+      <c r="J85" s="4" t="n"/>
+      <c r="K85" s="4" t="n"/>
+      <c r="L85" s="4" t="n"/>
       <c r="M85" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: message blocked / not found at eagleslanding.org.</t>
@@ -3430,41 +3430,35 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="6" t="n">
+      <c r="A86" t="n">
         <v>85</v>
       </c>
-      <c r="B86" s="6" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>Eagle's Landing Christian Academy - Junior High</t>
         </is>
       </c>
-      <c r="C86" s="6" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>McDonough</t>
         </is>
       </c>
-      <c r="D86" s="6" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E86" s="6" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>Cathie Kelly</t>
         </is>
       </c>
-      <c r="F86" s="6" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>cathie.kelly@eagleslanding.org</t>
         </is>
       </c>
-      <c r="G86" s="6" t="inlineStr"/>
-      <c r="H86" s="6" t="inlineStr"/>
-      <c r="I86" s="6" t="inlineStr"/>
-      <c r="J86" s="6" t="inlineStr"/>
-      <c r="K86" s="6" t="inlineStr"/>
-      <c r="L86" s="6" t="inlineStr"/>
-      <c r="M86" s="6" t="inlineStr">
+      <c r="M86" t="inlineStr">
         <is>
           <t>CAUTION: all other eagleslanding.org addresses bounced 2026-09-10; likely invalid.</t>
         </is>
@@ -3504,11 +3498,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H87" s="4" t="inlineStr"/>
-      <c r="I87" s="4" t="inlineStr"/>
-      <c r="J87" s="4" t="inlineStr"/>
-      <c r="K87" s="4" t="inlineStr"/>
-      <c r="L87" s="4" t="inlineStr"/>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="4" t="n"/>
+      <c r="J87" s="4" t="n"/>
+      <c r="K87" s="4" t="n"/>
+      <c r="L87" s="4" t="n"/>
       <c r="M87" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: message blocked / not found at eagleslanding.org.</t>
@@ -3549,11 +3543,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H88" s="4" t="inlineStr"/>
-      <c r="I88" s="4" t="inlineStr"/>
-      <c r="J88" s="4" t="inlineStr"/>
-      <c r="K88" s="4" t="inlineStr"/>
-      <c r="L88" s="4" t="inlineStr"/>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
+      <c r="J88" s="4" t="n"/>
+      <c r="K88" s="4" t="n"/>
+      <c r="L88" s="4" t="n"/>
       <c r="M88" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: message blocked / not found at eagleslanding.org.</t>
@@ -3594,11 +3588,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H89" s="4" t="inlineStr"/>
-      <c r="I89" s="4" t="inlineStr"/>
-      <c r="J89" s="4" t="inlineStr"/>
-      <c r="K89" s="4" t="inlineStr"/>
-      <c r="L89" s="4" t="inlineStr"/>
+      <c r="H89" s="4" t="n"/>
+      <c r="I89" s="4" t="n"/>
+      <c r="J89" s="4" t="n"/>
+      <c r="K89" s="4" t="n"/>
+      <c r="L89" s="4" t="n"/>
       <c r="M89" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: recipient unknown at eagleslanding.org.</t>
@@ -3909,11 +3903,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="H99" s="4" t="inlineStr"/>
-      <c r="I99" s="4" t="inlineStr"/>
-      <c r="J99" s="4" t="inlineStr"/>
-      <c r="K99" s="4" t="inlineStr"/>
-      <c r="L99" s="4" t="inlineStr"/>
+      <c r="H99" s="4" t="n"/>
+      <c r="I99" s="4" t="n"/>
+      <c r="J99" s="4" t="n"/>
+      <c r="K99" s="4" t="n"/>
+      <c r="L99" s="4" t="n"/>
       <c r="M99" s="4" t="inlineStr">
         <is>
           <t>BOUNCED 2026-09-10: message blocked by recipient server.</t>
@@ -4359,8 +4353,8 @@
           <t>No - administrator; referral</t>
         </is>
       </c>
-      <c r="K113" s="3" t="inlineStr"/>
-      <c r="L113" s="3" t="inlineStr"/>
+      <c r="K113" s="3" t="n"/>
+      <c r="L113" s="3" t="n"/>
       <c r="M113" s="3" t="inlineStr">
         <is>
           <t>Replied 2026-09-10: has not used the curriculum with students (administrator); refers Diana Helton, who has used DeepRoots.</t>
@@ -4998,41 +4992,35 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="7" t="n">
+      <c r="A135" t="n">
         <v>134</v>
       </c>
-      <c r="B135" s="7" t="inlineStr">
+      <c r="B135" t="inlineStr">
         <is>
           <t>Bethlehem Christian Academy - Elementary</t>
         </is>
       </c>
-      <c r="C135" s="7" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>Bethlehem</t>
         </is>
       </c>
-      <c r="D135" s="7" t="inlineStr">
+      <c r="D135" t="inlineStr">
         <is>
           <t>GA</t>
         </is>
       </c>
-      <c r="E135" s="7" t="inlineStr">
+      <c r="E135" t="inlineStr">
         <is>
           <t>Shannon Jones</t>
         </is>
       </c>
-      <c r="F135" s="7" t="inlineStr">
+      <c r="F135" t="inlineStr">
         <is>
           <t>sjones@bcamail.org</t>
         </is>
       </c>
-      <c r="G135" s="7" t="inlineStr"/>
-      <c r="H135" s="7" t="inlineStr"/>
-      <c r="I135" s="7" t="inlineStr"/>
-      <c r="J135" s="7" t="inlineStr"/>
-      <c r="K135" s="7" t="inlineStr"/>
-      <c r="L135" s="7" t="inlineStr"/>
-      <c r="M135" s="7" t="inlineStr">
+      <c r="M135" t="inlineStr">
         <is>
           <t>REFERRAL from Kelly Vann (Bethlehem). Invitation sent 2026-09-10 (greeting "Shannon").</t>
         </is>
@@ -5087,15 +5075,15 @@
           <t>YES - Upper School curriculum director, wants to talk; checking with Angela Adams (Bible dept chair) on her interest too</t>
         </is>
       </c>
-      <c r="K136" s="5" t="inlineStr"/>
+      <c r="K136" s="5" t="n"/>
       <c r="L136" s="5" t="inlineStr">
         <is>
-          <t>Awaiting times - checking with Angela (as of 2026-09-19)</t>
+          <t>In progress: Donna asked to schedule (Sep 21); Troy proposed Thu Sep 24 3PM ET. Awaiting her confirm. CONFLICT WATCH: same slot as Diana Helton proposal (Thu Sep 24 3PM ET).</t>
         </is>
       </c>
       <c r="M136" s="5" t="inlineStr">
         <is>
-          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up. | 2026-09-19: out of school recently; will check with Angela and follow up with times.</t>
+          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up. | 2026-09-19: out of school recently; will check with Angela and follow up with times. | 2026-09-21: Donna replied "When would you like to schedule the call?" Troy proposed Thu Sep 24 3PM ET. Title confirmed: Director of Curriculum and Instruction, Dayspring. Awaiting confirm. | 2026-09-21: Sep 24 re-check reminder cancelled (Donna already scheduling).</t>
         </is>
       </c>
     </row>
@@ -5155,12 +5143,12 @@
       </c>
       <c r="L137" s="5" t="inlineStr">
         <is>
-          <t>Nudged 2026-09-17 for times</t>
+          <t>Proposed Thu Sep 24 2026, 4:00 PM ET (draft ready 2026-09-21); awaiting confirm. Moved off 3PM to avoid clash with Donna Hurley.</t>
         </is>
       </c>
       <c r="M137" s="5" t="inlineStr">
         <is>
-          <t>Round 1 contact; agreed 2026-09-11 and questions sent 2026-09-11. Also referred by Tanya Murphy. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
+          <t>Round 1 contact; agreed 2026-09-11 and questions sent 2026-09-11. Also referred by Tanya Murphy. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-21: drafted second nudge proposing a specific slot: Thu Sep 24 3:00 PM ET (her local, Winter Garden FL). Awaiting confirmation. | 2026-09-21: prior 3PM draft was never sent; recreated draft proposing Thu Sep 24 4:00 PM ET (moved off 3PM to avoid conflict with Donna). Awaiting confirm.</t>
         </is>
       </c>
     </row>
@@ -5220,17 +5208,78 @@
       </c>
       <c r="L138" s="5" t="inlineStr">
         <is>
-          <t>Nudged 2026-09-17 for times</t>
+          <t>In progress: Troy proposed Wed/Thu Sep 25 3PM ET (Sep 21); Wendy swamped this week (classroom + special events), open to NEXT week. Troy offered 3PM ET any day next week. Awaiting her day pick.</t>
         </is>
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
-          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times).</t>
+          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-21: drafted second nudge proposing a specific slot: Fri Sep 25 3:00 PM ET (her local, New Albany IN = Eastern). Grade level unconfirmed. Awaiting confirmation. | 2026-09-21: Troy handled live in Gmail. Wendy: received questions, cannot this week, might do next week. Troy: 3PM ET any day next week. Awaiting Wendy to name a day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Christian Academy School System (Louisville KY campus)</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>Louisville</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>Carrie Feitl</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr">
+        <is>
+          <t>cfeitl@caschools.us</t>
+        </is>
+      </c>
+      <c r="G139" s="5" t="n"/>
+      <c r="H139" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I139" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="J139" s="5" t="inlineStr">
+        <is>
+          <t>YES - willing to talk (K-5 Instructional Coach + K-12 system Data Coach; not middle school, longtime DeepRoots user)</t>
+        </is>
+      </c>
+      <c r="K139" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L139" s="5" t="inlineStr">
+        <is>
+          <t>Awaiting times - questions sent 2026-09-10, no reply since</t>
+        </is>
+      </c>
+      <c r="M139" s="5" t="inlineStr">
+        <is>
+          <t>From an earlier call/round (not in the round-2 list of 133). Spoke with Troy by phone ~Sep 3. Replied 2026-09-04 clarifying role (K-5 coach/K-12 data coach, Louisville KY = same caschools.us system as Wendy Wagoner). Troy replied 2026-09-10, sent questions, asked for times. No reply since (as of 2026-09-21). Eastern time. Nudge candidate.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M138"/>
+  <autoFilter ref="A1:M139"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5695,11 +5744,10 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-21: 137 contacts, 11 replied, 5 want in, 1 booked, 11 bounced.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Updated 2026-09-25: 138 contacts, 13 replied, 7 want in, 2 booked, 11 bounced.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Round 2 tracker: Wagoner booked Oct 2, Feitl note
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0161c8Yzk8sqQsFb97wP8NVi
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -5208,12 +5208,12 @@
       </c>
       <c r="L138" s="5" t="inlineStr">
         <is>
-          <t>In progress: Troy proposed Wed/Thu Sep 25 3PM ET (Sep 21); Wendy swamped this week (classroom + special events), open to NEXT week. Troy offered 3PM ET any day next week. Awaiting her day pick.</t>
+          <t>BOOKED: Fri Oct 2 2026, 3:00 PM ET (15-20 min) - Pat Williamson sending calendar invite/Meet link</t>
         </is>
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
-          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-21: drafted second nudge proposing a specific slot: Fri Sep 25 3:00 PM ET (her local, New Albany IN = Eastern). Grade level unconfirmed. Awaiting confirmation. | 2026-09-21: Troy handled live in Gmail. Wendy: received questions, cannot this week, might do next week. Troy: 3PM ET any day next week. Awaiting Wendy to name a day.</t>
+          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-21: drafted second nudge proposing a specific slot: Fri Sep 25 3:00 PM ET (her local, New Albany IN = Eastern). Grade level unconfirmed. Awaiting confirmation. | 2026-09-21: Troy handled live in Gmail. Wendy: received questions, cannot this week, might do next week. Troy: 3PM ET any day next week. Awaiting Wendy to name a day. | 2026-09-28: Wendy proposed Fri 3PM; Troy confirmed (cc Pat). 2026-09-29: Wendy confirmed she received the questions and is preparing for Friday. No action needed except confirm Pat's invite went out.</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="M139" s="5" t="inlineStr">
         <is>
-          <t>From an earlier call/round (not in the round-2 list of 133). Spoke with Troy by phone ~Sep 3. Replied 2026-09-04 clarifying role (K-5 coach/K-12 data coach, Louisville KY = same caschools.us system as Wendy Wagoner). Troy replied 2026-09-10, sent questions, asked for times. No reply since (as of 2026-09-21). Eastern time. Nudge candidate.</t>
+          <t>From an earlier call/round (not in the round-2 list of 133). Spoke with Troy by phone ~Sep 3. Replied 2026-09-04 clarifying role (K-5 coach/K-12 data coach, Louisville KY = same caschools.us system as Wendy Wagoner). Troy replied 2026-09-10, sent questions, asked for times. No reply since (as of 2026-09-21). Eastern time. Nudge candidate. | 2026-09-28: Carrie emailed asking for the pre-assessment printables (unrelated to interview); Troy sent them. Still no reply about interview times. Nudge candidate.</t>
         </is>
       </c>
     </row>
@@ -5744,7 +5744,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Updated 2026-09-25: 138 contacts, 13 replied, 7 want in, 2 booked, 11 bounced.</t>
+          <t>Updated 2026-09-29: 138 contacts, 13 replied, 7 want in, 3 booked, 11 bounced.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire Meredith interview into tracker: links + Interview Q&A tab
Added interview Doc + Q&A Sheet links to Meredith's row (all three tracker
formats) and an Interview Q&A tab (Q&A matrix + DeepRoots team-takeaways
block). Rebased on top of the Wagoner/Feitl tracker updates.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview Q&amp;A" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$139</definedName>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +46,23 @@
       <i val="1"/>
       <color rgb="00666666"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="000563C1"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -94,6 +110,16 @@
         <bgColor rgb="00D9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -107,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -122,6 +148,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -487,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M139"/>
+  <dimension ref="A1:O139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -503,6 +544,8 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="52" customWidth="1" min="12" max="12"/>
     <col width="66" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -571,6 +614,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="N1" s="12" t="inlineStr">
+        <is>
+          <t>Interview Notes (Doc)</t>
+        </is>
+      </c>
+      <c r="O1" s="12" t="inlineStr">
+        <is>
+          <t>Interview Q&amp;A (Sheet)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
@@ -624,12 +677,22 @@
       <c r="K2" s="5" t="n"/>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>BOOKED: Thu Sep 24 2026, 11:00 AM PT (2:00 PM ET) - Google Meet meet.google.com/vzx-fphv-kga - on work calendar (tdwinkler@deeprootsbible.com); Pat Williamson added as attendee</t>
+          <t>COMPLETED interview Sep 24 2026 (Gemini notes + transcript). Answers: see Interview Doc / Q&amp;A links.</t>
         </is>
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Replied 2026-09-10: "I would be happy to be a part of this development!" → SEND questions-preview email + schedule. | Scheduling nudge sent 2026-09-17 (asked for times). | Sent availability 2026-09-17 (Pacific). Propose a specific slot. | 2026-09-21: booked Thu Sep 24 11:00 AM PT; calendar invite + confirmation sent. | 2026-09-21: moved event to work calendar (tdwinkler@deeprootsbible.com), added Pat Williamson; new Meet link vzx-fphv-kga. | 2026-09-24: Interview held. Meredith replied same day with a thank-you note, apologizing for the call running long (past the planned 30 min) and offering to be available for any future follow-up questions. No action needed.</t>
+        </is>
+      </c>
+      <c r="N2" s="13" t="inlineStr">
+        <is>
+          <t>Interview with Meredith Arldt</t>
+        </is>
+      </c>
+      <c r="O2" s="13" t="inlineStr">
+        <is>
+          <t>DeepRoots Interview Q&amp;A</t>
         </is>
       </c>
     </row>
@@ -5280,6 +5343,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:M139"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5758,4 +5825,923 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Interview Q&amp;A (also lives in Google Sheets — team-editable): https://docs.google.com/spreadsheets/d/1l05g_q15y2aV9FaNr8ABGPQdbd-yyJ0NLf2xXKy8uc4/edit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="15" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Q#</t>
+        </is>
+      </c>
+      <c r="C2" s="15" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — 2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>How does your school categorize Middle School / Junior High (5-8, 6-8, 7-8)?</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Middle school is 6th, 7th, and 8th grade (6-8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>What are the primary differences between a 6th, 7th, and 8th grade student (developmentally, spiritually, emotionally)?</t>
+        </is>
+      </c>
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Students begin actively questioning their own faith and searching for personal identity ('why do I believe what I believe?') amid outside influences like social media. 6th graders want independence but still want the safety net of mom and dad, going back and forth. 7th graders like to push and challenge ('their own little beast'). 8th graders can get 'a little too big for their own.' Spirituality is hard at this age because it is not always tangible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>How do you best reach both churched and unchurched students? Is this an issue for you? What works best?</t>
+        </is>
+      </c>
+      <c r="D5" s="16" t="inlineStr">
+        <is>
+          <t>About 60% of the school population identifies with a church home; 40% do not. They are intentional about corporate worship (for some students it is their only weekly worship) and adopted the Teaching for Transformation framework (from CASE) two years ago, with flex projects that put faith into action. They are also rebuilding the historically broken bridge with their associated church to connect unchurched families with pastoral staff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>What do you like or dislike about your current Bible curriculum?</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>Currently workbook-based: Purposeful Design (Daring Deliverers), and Positive Action (Character Counts for 6th, Wise Up for 8th). All workbook-based and 'pretty dry and boring.' The goal is to keep Bible from feeling like just another academic class and to focus on students' hearts, not grade their faith.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>What elements would you like to see in it each week?</t>
+        </is>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>More reflection and personal application ('how does this resonate with you today? what do we do with this?'). Historical and cultural context so students understand the significance of events. Treat biblical figures and events as real history, not 'stories' or fairy tales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>What core ideals do you wish each student left your class identifying with?</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Moving from head knowledge to heart knowledge; a real identity in Christ; applying scripture to their own lives; striving to be the best version of who God created them to be.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Marketing &amp; Sales</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>What types of resources (videos, activities, etc.) are most helpful for you as a teacher?</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Short videos (about 1.5-5 minutes), historical family trees, Bible timelines, primary documents, original-language (Greek/Hebrew) references, and cultural/archaeological references (e.g., an archaeological Bible). Note: curating and vetting these is the most time-consuming part for teachers, so ready-made, vetted resources would help most.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Editorial</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>How many minutes can students pay attention to teaching, reading, discussion, activities?</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Lecture/teaching is kept to 15-20 minutes max before moving into discussion. A typical rhythm is a ~5-minute intro/review, a 10-15 minute lesson, then discussion. Class is mostly discussion-based; some reading.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Editorial</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>What kind of engagements do students enjoy most (by grade)?</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Discussion-based work and things they can relate to (real-world video, relatable visuals), partner work, and interactive questions. Discussion is the biggest draw across middle school.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Editorial</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>How do you use screens and technology in your classroom?</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Google Classroom is the platform; laptops are provided but screen time is intentionally limited (parents appreciate this). Currently projection-based; installing BenQ interactive smartboards by January (grant-funded), with teacher training.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Editorial</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>What questions/issues do you see students wrestling with (by grade)?</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Reconciling 'what my parents taught me' with 'what do I actually believe'; identity in Christ versus societal pressure and peer acceptance; influence of social media; and nominal Christianity ('Christian in name only') where students know the Sunday-school answers but haven't moved it from head to heart.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Editorial</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Would you use an end-of-year project students prepare as a group? (Yes/No/Maybe)</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Maybe / planning to: no big end-of-year project currently (some project element in the final exam), but she wants to add an 8th-grade capstone project tied to Teaching for Transformation as students move into high school.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Editorial</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>What tools have helped with parent engagement?</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>A required number of service hours per semester draws families in (parents help get middle schoolers to service projects and often serve together around a shared passion). Also communicating the grading approach clearly at tours, and rebuilding the church connection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Editorial</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>What is your school's homework policy (by grade)?</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>What videos do you currently show, and how do you use them?</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Right Now Media and YouTube clips; one recurring activity has students take a Christian song and build a Bible-study object lesson around it. All videos are vetted by the teacher/administrator before showing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>What length of video is most engaging? (30s-1m / 1-2m / 2-3m / 3m+)</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Short: generally no more than ~5 minutes, with song-based clips around 1.5-2 minutes, to match attention spans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" s="16" t="inlineStr">
+        <is>
+          <t>What types of visuals are most effective for middle schoolers?</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Real-life, relatable people (not cartoons); charts and graphs, family trees, timelines, historical artwork/renderings, primary documents, archaeological images, and maps. She favors visuals students can see themselves in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="C20" s="16" t="inlineStr">
+        <is>
+          <t>Do you prefer digital assessments or printables?</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Leaning digital: with the move to Google Classroom (year two), they are less tied to printables; students interact with lessons and submit work electronically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="C21" s="16" t="inlineStr">
+        <is>
+          <t>What balance between text and visuals on a typical student page?</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>A balanced mix of text and visuals (stated explicitly). As a former English teacher she values the written word and dissecting scripture, and also sees strong value in relatable visuals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>What would make a middle schooler pick up the curriculum rather than see it as 'just another textbook'?</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Relatable, real-world visuals plus the teacher's presentation and enthusiasm. Avoiding dry, workbook-feeling material; keeping it discussion-driven and engaging. The teacher's delivery makes a big difference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>Are you limited by the amount of material you can print?</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Not really limited. Teachers are asked to reduce paper where possible, but the school is well-resourced (budget, laptops, Google Classroom) and prints less in middle school than in elementary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>If an activity required non-standard supplies (e.g., food), would the school provide funds or would the teacher?</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>The school provides funds. Teachers have money set aside each year for curriculum and supplies; she orders what they need and tracks spending. In nine years she has never told a teacher 'no' to a resource request.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>After 20 minutes of essential material, how much additional time would you like optional material to fill?</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Since class is mostly discussion-based, if the core lesson runs about 20 minutes, guided discussion can take the majority of the remaining class time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="C26" s="16" t="inlineStr">
+        <is>
+          <t>Would you be interested in a multi-subject Timeline centered on Bible events (with optional Empires, Literature, Music/Arts, People, Inventions, clickable summaries and media)?</t>
+        </is>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Not asked verbatim, but very likely yes: she strongly values timelines (built family trees and displayed a Bible timeline so students could see how events were organized) and finds chronology a real challenge for students.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>Approximately how many minutes of screen time/technology would you permit in Bible class?</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>No specific number given; screen time is intentionally limited and balanced across the day rather than used continuously.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="C28" s="16" t="inlineStr">
+        <is>
+          <t>What tools have you found most effective for encouraging Bible reading at home?</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B29" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>If the curriculum offered an optional human sexuality unit, how would you use it?</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>They would not teach it at school; human sexuality is treated as a parent matter and left entirely to parents. They already skip such lessons (e.g., a unit 10 in the 8th-grade book) and coordinate with teachers to do so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Would you be interested in a separate Logic course, primarily taught through videos and reinforced with worksheets?</t>
+        </is>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Yes / interested, but video-based delivery matters: teachers would likely need videos of someone presenting the material to feel comfortable, rather than lecture- or worksheet-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B31" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>With 5 minutes of independent reading + 15 minutes of teaching/engagement, would you use optional deeper material? What engagements?</t>
+        </is>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>Yes. She likes a ~5-minute reflection/journaling opening, then a lesson (~20 minutes total), then discussion. Engagements: discussion, journaling/reflection, returning to scripture, and partner work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="C32" s="16" t="inlineStr">
+        <is>
+          <t>How important is handling a printable reference book (Course Pack) vs. an online reference?</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>Mixed, leaning digital with the Google Classroom move, but she still values the written word and dissecting scripture, so there is real value in a text reference for some students.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B33" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="C33" s="16" t="inlineStr">
+        <is>
+          <t>Individual quiet work vs. group activity: which do you prefer? Which do students prefer?</t>
+        </is>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>Group/discussion for both. Independent Bible study is hard for middle schoolers because they are not yet fluent in scripture, so guided, discussion-heavy classes are essential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B34" s="16" t="n">
+        <v>32</v>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>As a teacher, what does your ideal Bible lesson look like?</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>A short intro/review (~5 min), a focused lesson (~15-20 min), then discussion and partner work, woven with historical/cultural context and personal reflection/application, kept moving so students stay engaged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>How do you measure the success of a curriculum?</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Students being able to apply scripture to their own lives. Her tests always ended with an open-ended prompt: 'write an example of how this applies to your life,' which showed movement from head knowledge to heart knowledge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>Are there visual styles/trends/design approaches that would NOT work well?</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Younger, cartoon-style depictions of people. Middle schoolers are moving away from cartoons and want to see real people they can relate to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>What short videos would be helpful to supplement your teaching?</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Real-world application videos most of all, plus videos that hit the key idea and introduce/give context to the subject; relatable real-world visuals resonate most.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>On a scale of 1-10, how would you rate role-play activities for engagement?</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Low. Middle schoolers often dislike being put on the spot, especially about personal faith. Fine as an optional tool if a class is open to it, but not something to use consistently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>What elements of a Bible curriculum do you NOT prefer?</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Dry, boring material; 'just words on a page' or 'the next lesson in the workbook,' which brings the wrong attitude into class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>What gets and holds your students' attention in Bible class?</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Engaging discussion and debate, relatable real-world visuals and video, the teacher's enthusiasm and presentation, and variety that keeps the lesson moving.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>Additional (Extra Time)</t>
+        </is>
+      </c>
+      <c r="B41" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>What would a middle school Bible curriculum look like that is easy to teach and impactful?</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>The same depth and teacher resources DeepRoots provides for elementary, but with a different presentation model for middle school: not dry, relatable visuals, discussion-driven, rich in reflection/application and historical/cultural context, with enough ready-made resources that teachers are not building and vetting everything themselves. (They currently use DeepRoots for grades 3-5.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr"/>
+      <c r="B42" s="16" t="inlineStr"/>
+      <c r="C42" s="16" t="inlineStr"/>
+      <c r="D42" s="16" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>DEEPROOTS TEAM TAKEAWAYS — what we got out of this interview (said or unsaid)</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr"/>
+      <c r="C43" s="17" t="inlineStr"/>
+      <c r="D43" s="17" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="inlineStr"/>
+      <c r="B44" s="18" t="inlineStr"/>
+      <c r="C44" s="18" t="inlineStr">
+        <is>
+          <t>Team member</t>
+        </is>
+      </c>
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>Your takeaways / observations</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr"/>
+      <c r="B45" s="16" t="inlineStr"/>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Troy Winkler</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr"/>
+      <c r="B46" s="16" t="inlineStr"/>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>Pat Williamson</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr"/>
+      <c r="B47" s="16" t="inlineStr"/>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Nancy Wood</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="16" t="inlineStr"/>
+      <c r="B48" s="16" t="inlineStr"/>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>Tammy Plett</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="16" t="inlineStr"/>
+      <c r="B49" s="16" t="inlineStr"/>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Lisa Van Vlear</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="16" t="inlineStr"/>
+      <c r="B50" s="16" t="inlineStr"/>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>Overall / key takeaways for the curriculum</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Daily reply check: Donna Hurley booked Oct 6 3:20 PM ET (Angela joining)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QkTgFvQcj5zTHPKcY5dkwT
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interview Q&amp;A" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Atlantic Shores (VA) Feedback" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Response Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Questions Email" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Read Me" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Interview Q&amp;A" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Atlantic Shores (VA) Feedback" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Response Tracker'!$A$1:$M$139</definedName>
@@ -5170,12 +5170,12 @@
       <c r="K136" s="5" t="n"/>
       <c r="L136" s="5" t="inlineStr">
         <is>
-          <t>In progress: Donna asked to schedule (Sep 21); Troy proposed Thu Sep 24 3PM ET. Awaiting her confirm. CONFLICT WATCH: same slot as Diana Helton proposal (Thu Sep 24 3PM ET).</t>
+          <t>BOOKED: Tue Oct 6 2026, 3:20 PM ET (30 min) - Google Meet invite sent; Angela Adams (Bible dept chair, aadams@dayspringchristian.com) joining - Donna asked Troy to send Angela her own invite (Troy said he would, 2026-09-30)</t>
         </is>
       </c>
       <c r="M136" s="5" t="inlineStr">
         <is>
-          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up. | 2026-09-19: out of school recently; will check with Angela and follow up with times. | 2026-09-21: Donna replied "When would you like to schedule the call?" Troy proposed Thu Sep 24 3PM ET. Title confirmed: Director of Curriculum and Instruction, Dayspring. Awaiting confirm. | 2026-09-21: Sep 24 re-check reminder cancelled (Donna already scheduling).</t>
+          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up. | 2026-09-19: out of school recently; will check with Angela and follow up with times. | 2026-09-21: Donna replied "When would you like to schedule the call?" Troy proposed Thu Sep 24 3PM ET. Title confirmed: Director of Curriculum and Instruction, Dayspring. Awaiting confirm. | 2026-09-21: Sep 24 re-check reminder cancelled (Donna already scheduling). | 2026-09-29: Donna proposed Tue Oct 6 3:20 PM ET (Angela can join); Troy confirmed. Donna did not receive first invite; resent. | 2026-09-30: Donna found invite and responded; asked Troy to send Angela a separate invite - Troy replied he'd do so. Verify Angela's invite went out. Questions-preview email not yet sent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Wendy Wagoner (Christian Academy of Indiana) interview
Oct 2 interview run by Pat Williamson (attendees: Pat Williamson,
Megan Van Vlear, Lisa Van Vlear, Erin Eggertsen, Jacob Waller).
Mapped her answers to the 39-question set and added a Wendy Wagoner
column on the All Interviews master (teal) plus a dedicated Wendy
Wagoner interview tab in the Q&A workbook. She covered ~18 questions
in the call and will send written answers for the rest.

Tracker row #137 marked completed with interview doc + Q&A sheet
links; tracker_state.json, response_tracker.csv, and the Response
Tracker workbook tab updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -5312,12 +5312,22 @@
       </c>
       <c r="L138" s="5" t="inlineStr">
         <is>
-          <t>BOOKED: Fri Oct 2 2026, 3:00 PM ET (15-20 min) - Pat Williamson sending calendar invite/Meet link</t>
+          <t>COMPLETED interview Fri Oct 2 2026, 3:00 PM ET (Pat Williamson ran it; Gemini notes + transcript). Answers: Interview Doc + Q&amp;A Sheet (Wendy Wagoner tab/column).</t>
         </is>
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
           <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-21: drafted second nudge proposing a specific slot: Fri Sep 25 3:00 PM ET (her local, New Albany IN = Eastern). Grade level unconfirmed. Awaiting confirmation. | 2026-09-21: Troy handled live in Gmail. Wendy: received questions, cannot this week, might do next week. Troy: 3PM ET any day next week. Awaiting Wendy to name a day. | 2026-09-28: Wendy proposed Fri 3PM; Troy confirmed (cc Pat). 2026-09-29: Wendy confirmed she received the questions and is preparing for Friday. No action needed except confirm Pat's invite went out.</t>
+        </is>
+      </c>
+      <c r="N138" s="13" t="inlineStr">
+        <is>
+          <t>Interview with Wendy Wagoner</t>
+        </is>
+      </c>
+      <c r="O138" s="13" t="inlineStr">
+        <is>
+          <t>DeepRoots Interview Q&amp;A</t>
         </is>
       </c>
     </row>
@@ -5389,6 +5399,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N84" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O84" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N138" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O138" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5876,7 +5888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5886,6 +5898,7 @@
     <col width="58" customWidth="1" min="5" max="5"/>
     <col width="58" customWidth="1" min="6" max="6"/>
     <col width="58" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5931,6 +5944,11 @@
           <t>Horizon Christian Elementary (OR) — current K-5 use — 9/28/26</t>
         </is>
       </c>
+      <c r="H2" s="15" t="inlineStr">
+        <is>
+          <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -5958,6 +5976,11 @@
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr"/>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>They call it middle school (not junior high) and it is grades 5 through 8, a configuration that is new this year following a new building. Grades 5-6 function as an 'intermediate middle school' block, while grades 7-8 merge to serve as building blocks preparing students to roll into high school.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -5985,6 +6008,11 @@
         </is>
       </c>
       <c r="G4" s="16" t="inlineStr"/>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>She framed the key divide as between 5th-6th graders and 7th-8th graders, driven largely by faith development (spiritual and emotional). Elementary students are 'little sponges' with a stable DeepRoots foundation; middle schoolers hit a 'crossroads' of taking personal ownership of their faith, wrestling internally with who they are and with 'wonder questions,' and need relational, safe environments where their questions aren't met with shock. She called question 2 'complex'—'you probably could spend the whole time on that one.'</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -6020,6 +6048,11 @@
           <t>Many unchurched students (G4): confused by unfamiliar terms like 'Sanhedrin' and by using multiple Bible translations (their students use NIV). Asked for a single translation. 'Intro to Jesus' is the key unit for unchurched kids.</t>
         </is>
       </c>
+      <c r="H5" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -6055,6 +6088,11 @@
           <t>Overall going well K-5. Kids love the songs (G1) and the discussions; K praises the variety of activities for different learners ('variety is key'). Clunky to get used to at first (G1). Projecting the visuals is clunky across ALL grades.</t>
         </is>
       </c>
+      <c r="H6" s="16" t="inlineStr">
+        <is>
+          <t>In elementary, homeroom teachers teach DeepRoots directly and she praised it as a reliable, sound-doctrine 'great tool' and framework teachers can trust and make their own. The middle-school side is patched together: 5th grade moved away from DeepRoots to a hands-on apologetics track (The Case for Christ Junior), 6th grade teachers (led by Becky Wy) had to 'morph something to work' for the new 5-6 track, and 7-8 use cobbled-together tracks after being pulled from high school scheduling—largely because 'there just wasn't a lot to use' for middle school.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -6082,6 +6120,11 @@
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr"/>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>She favors thematic weekly outlines with flexible starting activities rather than rigid daily scripts: a 'theme for the week' plus ideas for how students can 'start your day with Jesus' (e.g., a song), then the core lesson/content, woven with discussion questions and spiritual-discipline experiences. Resources should let teachers adapt to the students in front of them.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -6109,6 +6152,11 @@
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr"/>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>A 'heart for God'—their school's central aim—with students taking personal ownership of their faith, where 'faith becomes sight,' and cultivating a desire to serve and 'spread the love of Jesus' at home, on campus, and worldwide.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -6144,6 +6192,11 @@
           <t>Wants Teaching Essentials split out by unit (not one long doc) with the key elements listed inline (Bible reading passage, memory verse) so teachers aren't juggling multiple sources; printed TNs are too long.</t>
         </is>
       </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>User-friendly, easy-to-implement resources with sound doctrine that teachers can 'trust and count on' and adapt; specifically discussion questions tied to passages or topics, and 'spiritual discipline toolboxes' with experiences teachers can run. She stressed many capable teachers simply need the tools put 'in their hands' and that ready-made, trustworthy material saves them time.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -6171,6 +6224,11 @@
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr"/>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>It depends heavily on the activity. She half-joked she can get kindergarteners to do imaginative prayer for 40 minutes and cited the 'a minute for however old you are' rule of thumb, but said if discussion is challenging, on the 'forefront of what they want to know,' and sparks curiosity, engagement goes well beyond that—and experiential, participatory activities with buy-in can last even longer. Bible classes run 30-40 minutes, typically ~20 minutes high-content teaching and ~20 minutes discussion.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -6202,6 +6260,11 @@
           <t>Kids love the songs and the discussions (K/G1); variety of activities valued (K).</t>
         </is>
       </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Speaking of middle school broadly rather than by grade, she pointed to discussion (especially curiosity-driven, 'wonder question' discussion), experiential and service opportunities, spiritual disciplines, and end-of-year/capstone projects as most powerful and engaging.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -6237,6 +6300,11 @@
           <t>Projecting the visuals/script is clunky for all grades; no student devices at school. A slideshow version (with show/hide slides) is the top ask.</t>
         </is>
       </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -6264,6 +6332,11 @@
         </is>
       </c>
       <c r="G13" s="16" t="inlineStr"/>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Taking ownership of their faith and figuring out 'who they are'; 'wonder questions' about God and a world that is 'groaning' and hard; and sensitive personal 'triggers'—family and real-life situations that surface during stories/lessons—that students are wrestling with.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -6291,6 +6364,11 @@
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr"/>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>Yes. Classes work together to lead chapel through the year, and 5th graders write an apologetics 'defend your faith' essay they share with each other. She described a 'spiritual portfolio' of 'relics' of spiritual fruit collected over time that transitions with students to the next grade/school, letting them 'see their faith development along the way'; such capstone projects give students pride and visible growth.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -6318,6 +6396,11 @@
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr"/>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -6345,6 +6428,11 @@
         </is>
       </c>
       <c r="G16" s="16" t="inlineStr"/>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -6372,6 +6460,11 @@
         </is>
       </c>
       <c r="G17" s="16" t="inlineStr"/>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -6407,6 +6500,11 @@
           <t>G5 uses some of our videos and supplements with others she finds herself.</t>
         </is>
       </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -6442,6 +6540,11 @@
           <t>G5 initially felt visuals were too young (kindergartener photos) — traced to starting with the 'Intro to Jesus' unit; the rest of the G5 visuals are age-appropriate. Need a differentiated 'Intro to Jesus' (upper vs lower elementary).</t>
         </is>
       </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
@@ -6477,6 +6580,11 @@
           <t>No student devices at school; want PRINTABLE pre- and post-assessments for all grade levels.</t>
         </is>
       </c>
+      <c r="H20" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -6504,6 +6612,11 @@
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr"/>
+      <c r="H21" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -6531,6 +6644,11 @@
         </is>
       </c>
       <c r="G22" s="16" t="inlineStr"/>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
@@ -6558,6 +6676,11 @@
         </is>
       </c>
       <c r="G23" s="16" t="inlineStr"/>
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
@@ -6585,6 +6708,11 @@
         </is>
       </c>
       <c r="G24" s="16" t="inlineStr"/>
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -6612,6 +6740,11 @@
         </is>
       </c>
       <c r="G25" s="16" t="inlineStr"/>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Classes run 30-40 minutes, so with ~20 minutes of core content there is roughly another ~20 minutes for discussion or alternative/experiential activities. She affirmed a 'digging deeper' section for schools with longer periods would be helpful, and noted resources can also be 'sprinkled in other moments' of the day (start-of-day activities, houses/projects) rather than all in one block.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -6639,6 +6772,11 @@
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr"/>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
@@ -6666,6 +6804,11 @@
         </is>
       </c>
       <c r="G27" s="16" t="inlineStr"/>
+      <c r="H27" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
@@ -6701,6 +6844,11 @@
           <t>G1 can't cover all unit material, so prefers ONE memory verse per unit instead of two (use the week-2 tested verse). One G1 teacher is improvising ASL hand motions to aid memory.</t>
         </is>
       </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -6728,6 +6876,11 @@
         </is>
       </c>
       <c r="G29" s="16" t="inlineStr"/>
+      <c r="H29" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
@@ -6755,6 +6908,11 @@
         </is>
       </c>
       <c r="G30" s="16" t="inlineStr"/>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -6782,6 +6940,11 @@
         </is>
       </c>
       <c r="G31" s="16" t="inlineStr"/>
+      <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Yes. She confirmed a 'digging deeper'/extra section would be useful and suggested it hold spiritual-discipline 'toolbox' ideas tied to what the story is highlighting, 'start your day / end your day' activities, brain-break style items, and topical 'if this arises' guidance with tidbits and resources for sensitive triggers students bring up.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -6809,6 +6972,11 @@
         </is>
       </c>
       <c r="G32" s="16" t="inlineStr"/>
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -6836,6 +7004,11 @@
         </is>
       </c>
       <c r="G33" s="16" t="inlineStr"/>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>She didn't directly rank the two, but leaned strongly toward relational, discussion-based and group/experiential learning as most powerful for middle school, while also valuing individual contemplative disciplines she teaches (e.g., meditation, 'take a minute' to pause and pray without words) where 'the Lord is going to meet each of you differently.'</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
@@ -6863,6 +7036,11 @@
         </is>
       </c>
       <c r="G34" s="16" t="inlineStr"/>
+      <c r="H34" s="16" t="inlineStr">
+        <is>
+          <t>A thematic weekly outline with a flexible start-of-day activity, then focused content (~20 min) and discussion (~20 min within a 30-40 min period), woven with an experiential spiritual-discipline element and good discussion questions, framed so teachers understand 'why we do it,' with room to evolve the lesson and adapt to immediate student needs.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
@@ -6898,6 +7076,11 @@
           <t>G4 test questions too verbose / over some students' heads (esp. unchurched); matching &amp; fill-in-the-blank easier than short answer. Want printable pre/post assessments for all grades.</t>
         </is>
       </c>
+      <c r="H35" s="16" t="inlineStr">
+        <is>
+          <t>Success shows up as students taking personal ownership of their faith and growing a 'heart for God'—movement she sees made visible through things like the spiritual portfolio of 'relics' of spiritual fruit that tracks a student's faith development over time, and through genuine worshipful, fruitful response rather than just completing content.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -6933,6 +7116,11 @@
           <t>Photos of kindergarteners don't relate for older grades; need age-appropriate visuals (and a differentiated 'Intro to Jesus' unit).</t>
         </is>
       </c>
+      <c r="H36" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -6960,6 +7148,11 @@
         </is>
       </c>
       <c r="G37" s="16" t="inlineStr"/>
+      <c r="H37" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -6991,6 +7184,11 @@
         </is>
       </c>
       <c r="G38" s="16" t="inlineStr"/>
+      <c r="H38" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
@@ -7018,6 +7216,11 @@
         </is>
       </c>
       <c r="G39" s="16" t="inlineStr"/>
+      <c r="H39" s="16" t="inlineStr">
+        <is>
+          <t>She cautioned against faith learning becoming 'just boxes that we're checking' and against overly rigid, minute-by-minute daily scripts, preferring flexible weekly thematic outlines teachers can adapt; she did not otherwise enumerate disliked curriculum elements.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
@@ -7045,6 +7248,11 @@
         </is>
       </c>
       <c r="G40" s="16" t="inlineStr"/>
+      <c r="H40" s="16" t="inlineStr">
+        <is>
+          <t>Challenging discussion on the 'forefront of what they want to know' that inspires curiosity, experiential activities where students have buy-in and participate, service and 'wonder question' conversations met safely and with God's truth, and opportunities to take ownership of their faith.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
@@ -7074,6 +7282,11 @@
       <c r="G41" s="16" t="inlineStr">
         <is>
           <t>A slideshow version where teachers choose which slides to show/hide; a single Bible translation (moving to all ESV); Teaching Essentials organized by unit with elements inline; printable pre/post assessments; age-appropriate visuals.</t>
+        </is>
+      </c>
+      <c r="H41" s="16" t="inlineStr">
+        <is>
+          <t>A reliable, sound-doctrine DeepRoots framework that is user-friendly and 'easy to implement'—flexible weekly thematic outlines rather than rigid scripts, discussion questions, spiritual-discipline 'toolboxes' and experiential opportunities with the 'why' explained so teachers aren't hesitant, a 'digging deeper' section for extra time, and topical 'if this arises' guidance for sensitive triggers—tools teachers can trust and 'make their own' for the students in front of them.</t>
         </is>
       </c>
     </row>
@@ -7085,6 +7298,7 @@
       <c r="E42" s="16" t="inlineStr"/>
       <c r="F42" s="16" t="inlineStr"/>
       <c r="G42" s="16" t="inlineStr"/>
+      <c r="H42" s="16" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
@@ -7098,6 +7312,7 @@
       <c r="E43" s="17" t="inlineStr"/>
       <c r="F43" s="17" t="inlineStr"/>
       <c r="G43" s="17" t="inlineStr"/>
+      <c r="H43" s="17" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="22" t="inlineStr"/>
@@ -7111,6 +7326,7 @@
       <c r="E44" s="22" t="inlineStr"/>
       <c r="F44" s="22" t="inlineStr"/>
       <c r="G44" s="22" t="inlineStr"/>
+      <c r="H44" s="22" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="18" t="inlineStr"/>
@@ -7140,6 +7356,11 @@
           <t>Horizon Christian Elementary (OR) — current K-5 use — 9/28/26</t>
         </is>
       </c>
+      <c r="H45" s="18" t="inlineStr">
+        <is>
+          <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr"/>
@@ -7157,6 +7378,7 @@
       <c r="E46" s="16" t="inlineStr"/>
       <c r="F46" s="16" t="inlineStr"/>
       <c r="G46" s="16" t="inlineStr"/>
+      <c r="H46" s="16" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr"/>
@@ -7174,6 +7396,7 @@
       <c r="E47" s="16" t="inlineStr"/>
       <c r="F47" s="16" t="inlineStr"/>
       <c r="G47" s="16" t="inlineStr"/>
+      <c r="H47" s="16" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr"/>
@@ -7191,6 +7414,7 @@
       <c r="E48" s="16" t="inlineStr"/>
       <c r="F48" s="16" t="inlineStr"/>
       <c r="G48" s="16" t="inlineStr"/>
+      <c r="H48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr"/>
@@ -7208,6 +7432,7 @@
       <c r="E49" s="16" t="inlineStr"/>
       <c r="F49" s="16" t="inlineStr"/>
       <c r="G49" s="16" t="inlineStr"/>
+      <c r="H49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr"/>
@@ -7225,6 +7450,7 @@
       <c r="E50" s="16" t="inlineStr"/>
       <c r="F50" s="16" t="inlineStr"/>
       <c r="G50" s="16" t="inlineStr"/>
+      <c r="H50" s="16" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr"/>
@@ -7238,6 +7464,7 @@
       <c r="E51" s="16" t="inlineStr"/>
       <c r="F51" s="16" t="inlineStr"/>
       <c r="G51" s="16" t="inlineStr"/>
+      <c r="H51" s="16" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr"/>
@@ -7247,6 +7474,7 @@
       <c r="E52" s="16" t="inlineStr"/>
       <c r="F52" s="16" t="inlineStr"/>
       <c r="G52" s="16" t="inlineStr"/>
+      <c r="H52" s="16" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="22" t="inlineStr"/>
@@ -7260,6 +7488,7 @@
       <c r="E53" s="22" t="inlineStr"/>
       <c r="F53" s="22" t="inlineStr"/>
       <c r="G53" s="22" t="inlineStr"/>
+      <c r="H53" s="22" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr"/>
@@ -7289,6 +7518,11 @@
           <t>Horizon Christian Elementary (OR) — current K-5 use — 9/28/26</t>
         </is>
       </c>
+      <c r="H54" s="18" t="inlineStr">
+        <is>
+          <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="16" t="inlineStr"/>
@@ -7302,6 +7536,7 @@
       <c r="E55" s="16" t="inlineStr"/>
       <c r="F55" s="16" t="inlineStr"/>
       <c r="G55" s="16" t="inlineStr"/>
+      <c r="H55" s="16" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr"/>
@@ -7315,6 +7550,7 @@
       <c r="E56" s="16" t="inlineStr"/>
       <c r="F56" s="16" t="inlineStr"/>
       <c r="G56" s="16" t="inlineStr"/>
+      <c r="H56" s="16" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr"/>
@@ -7328,6 +7564,7 @@
       <c r="E57" s="16" t="inlineStr"/>
       <c r="F57" s="16" t="inlineStr"/>
       <c r="G57" s="16" t="inlineStr"/>
+      <c r="H57" s="16" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr"/>
@@ -7341,6 +7578,7 @@
       <c r="E58" s="16" t="inlineStr"/>
       <c r="F58" s="16" t="inlineStr"/>
       <c r="G58" s="16" t="inlineStr"/>
+      <c r="H58" s="16" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr"/>
@@ -7354,6 +7592,7 @@
       <c r="E59" s="16" t="inlineStr"/>
       <c r="F59" s="16" t="inlineStr"/>
       <c r="G59" s="16" t="inlineStr"/>
+      <c r="H59" s="16" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr"/>
@@ -7367,6 +7606,7 @@
       <c r="E60" s="16" t="inlineStr"/>
       <c r="F60" s="16" t="inlineStr"/>
       <c r="G60" s="16" t="inlineStr"/>
+      <c r="H60" s="16" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr"/>
@@ -7376,6 +7616,149 @@
       <c r="E61" s="16" t="inlineStr"/>
       <c r="F61" s="16" t="inlineStr"/>
       <c r="G61" s="16" t="inlineStr"/>
+      <c r="H61" s="16" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr"/>
+      <c r="B62" s="22" t="inlineStr"/>
+      <c r="C62" s="22" t="inlineStr">
+        <is>
+          <t>WENDY WAGONER interview — Christian Academy of Indiana (IN), 2026-10-02  |  Attendees: Pat Williamson, Megan Van Vlear, Lisa Van Vlear, Erin Eggertsen, Jacob Waller</t>
+        </is>
+      </c>
+      <c r="D62" s="22" t="inlineStr"/>
+      <c r="E62" s="22" t="inlineStr"/>
+      <c r="F62" s="22" t="inlineStr"/>
+      <c r="G62" s="22" t="inlineStr"/>
+      <c r="H62" s="22" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="18" t="inlineStr"/>
+      <c r="B63" s="18" t="inlineStr"/>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>Team member</t>
+        </is>
+      </c>
+      <c r="D63" s="18" t="inlineStr">
+        <is>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — teacher/admin — 2026-09-24</t>
+        </is>
+      </c>
+      <c r="E63" s="18" t="inlineStr">
+        <is>
+          <t>Atlantic Shores Christian School (VA) — current K-5 use — 9/29/26</t>
+        </is>
+      </c>
+      <c r="F63" s="18" t="inlineStr">
+        <is>
+          <t>Will Weaver — Des Moines Christian School (IA) — Head of Spiritual Formation (admin) — 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G63" s="18" t="inlineStr">
+        <is>
+          <t>Horizon Christian Elementary (OR) — current K-5 use — 9/28/26</t>
+        </is>
+      </c>
+      <c r="H63" s="18" t="inlineStr">
+        <is>
+          <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="16" t="inlineStr"/>
+      <c r="B64" s="16" t="inlineStr"/>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Pat Williamson</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr"/>
+      <c r="E64" s="16" t="inlineStr"/>
+      <c r="F64" s="16" t="inlineStr"/>
+      <c r="G64" s="16" t="inlineStr"/>
+      <c r="H64" s="16" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr"/>
+      <c r="B65" s="16" t="inlineStr"/>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>Megan Van Vlear</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr"/>
+      <c r="E65" s="16" t="inlineStr"/>
+      <c r="F65" s="16" t="inlineStr"/>
+      <c r="G65" s="16" t="inlineStr"/>
+      <c r="H65" s="16" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="16" t="inlineStr"/>
+      <c r="B66" s="16" t="inlineStr"/>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>Lisa Van Vlear</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr"/>
+      <c r="E66" s="16" t="inlineStr"/>
+      <c r="F66" s="16" t="inlineStr"/>
+      <c r="G66" s="16" t="inlineStr"/>
+      <c r="H66" s="16" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="16" t="inlineStr"/>
+      <c r="B67" s="16" t="inlineStr"/>
+      <c r="C67" s="16" t="inlineStr">
+        <is>
+          <t>Erin Eggertsen</t>
+        </is>
+      </c>
+      <c r="D67" s="16" t="inlineStr"/>
+      <c r="E67" s="16" t="inlineStr"/>
+      <c r="F67" s="16" t="inlineStr"/>
+      <c r="G67" s="16" t="inlineStr"/>
+      <c r="H67" s="16" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="16" t="inlineStr"/>
+      <c r="B68" s="16" t="inlineStr"/>
+      <c r="C68" s="16" t="inlineStr">
+        <is>
+          <t>Jacob Waller</t>
+        </is>
+      </c>
+      <c r="D68" s="16" t="inlineStr"/>
+      <c r="E68" s="16" t="inlineStr"/>
+      <c r="F68" s="16" t="inlineStr"/>
+      <c r="G68" s="16" t="inlineStr"/>
+      <c r="H68" s="16" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="16" t="inlineStr"/>
+      <c r="B69" s="16" t="inlineStr"/>
+      <c r="C69" s="16" t="inlineStr">
+        <is>
+          <t>Overall / key takeaways for the curriculum</t>
+        </is>
+      </c>
+      <c r="D69" s="16" t="inlineStr"/>
+      <c r="E69" s="16" t="inlineStr"/>
+      <c r="F69" s="16" t="inlineStr"/>
+      <c r="G69" s="16" t="inlineStr"/>
+      <c r="H69" s="16" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="16" t="inlineStr"/>
+      <c r="B70" s="16" t="inlineStr"/>
+      <c r="C70" s="16" t="inlineStr"/>
+      <c r="D70" s="16" t="inlineStr"/>
+      <c r="E70" s="16" t="inlineStr"/>
+      <c r="F70" s="16" t="inlineStr"/>
+      <c r="G70" s="16" t="inlineStr"/>
+      <c r="H70" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Ironbridge (Nicole Burchett + Crystal Thompson) interview
Oct 5 interview with Ironbridge Christian Academy: Nicole Burchett
(Administrator/Director, former DeepRoots teacher) and Crystal Thompson
(5th/6th 'Bridge 56' Bible teacher). DeepRoots attendees: Troy Winkler,
Pat Williamson, Taylor Chartier, Lisa Van Vlear, Will Tuomey.

Added an Ironbridge column on the All Interviews master (burgundy) plus
a dedicated interview tab in the Q&A workbook. She covered 34 of the 39
questions. Not a round-2 outreach recipient, so no tracker row.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -5888,7 +5888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5899,6 +5899,7 @@
     <col width="58" customWidth="1" min="6" max="6"/>
     <col width="58" customWidth="1" min="7" max="7"/>
     <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="58" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5949,6 +5950,11 @@
           <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
         </is>
       </c>
+      <c r="I2" s="15" t="inlineStr">
+        <is>
+          <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -5981,6 +5987,11 @@
           <t>They call it middle school (not junior high) and it is grades 5 through 8, a configuration that is new this year following a new building. Grades 5-6 function as an 'intermediate middle school' block, while grades 7-8 merge to serve as building blocks preparing students to roll into high school.</t>
         </is>
       </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
+          <t>Unconventional structure: 'Bridge 56' covers 5th and 6th graders ('that step out of middle school'), and junior high is 7th and 8th grade. Students are grouped by developmental stage, with 5th graders together and 6th graders together in separate classes rather than all four mixed.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -6013,6 +6024,11 @@
           <t>She framed the key divide as between 5th-6th graders and 7th-8th graders, driven largely by faith development (spiritual and emotional). Elementary students are 'little sponges' with a stable DeepRoots foundation; middle schoolers hit a 'crossroads' of taking personal ownership of their faith, wrestling internally with who they are and with 'wonder questions,' and need relational, safe environments where their questions aren't met with shock. She called question 2 'complex'—'you probably could spend the whole time on that one.'</t>
         </is>
       </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Nicole said the developmental gap is why the grades are separated — there is a 'huge difference between a kindergartener and a fifth grader, but then also a fifth grader and an eighth grader or a sixth grader and an eighth grader,' which drives the Bridge 56 vs. junior-high split. Specific per-grade spiritual/emotional distinctions were not detailed.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -6053,6 +6069,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I5" s="16" t="inlineStr">
+        <is>
+          <t>They are a covenant school, so families should be churched, but public-school transfers often lack depth. Mrs. Thompson and Nicole send home church-event info and family activities, text weekend prayer-request messages, and encourage storybook Bibles and apps at home; Nicole tells parents up front that they no longer teach foundational Bible stories and gives them resources to prep kids. She cited a student who didn't know why Adam and Eve left the garden, which made jumping into Job hard.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -6093,6 +6114,11 @@
           <t>In elementary, homeroom teachers teach DeepRoots directly and she praised it as a reliable, sound-doctrine 'great tool' and framework teachers can trust and make their own. The middle-school side is patched together: 5th grade moved away from DeepRoots to a hands-on apologetics track (The Case for Christ Junior), 6th grade teachers (led by Becky Wy) had to 'morph something to work' for the new 5-6 track, and 7-8 use cobbled-together tracks after being pulled from high school scheduling—largely because 'there just wasn't a lot to use' for middle school.</t>
         </is>
       </c>
+      <c r="I6" s="16" t="inlineStr">
+        <is>
+          <t>They use DeepRoots and love it; Mrs. Thompson especially loves the videos in the 5th/6th grade curriculum. Her main frustration is not the curriculum but time — moving to an 80-minute block every other day makes finishing all the units a challenge, and as a self-described 'big talker' she doesn't want to skip the rich content.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -6125,6 +6151,11 @@
           <t>She favors thematic weekly outlines with flexible starting activities rather than rigid daily scripts: a 'theme for the week' plus ideas for how students can 'start your day with Jesus' (e.g., a song), then the core lesson/content, woven with discussion questions and spiritual-discipline experiences. Resources should let teachers adapt to the students in front of them.</t>
         </is>
       </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -6157,6 +6188,11 @@
           <t>A 'heart for God'—their school's central aim—with students taking personal ownership of their faith, where 'faith becomes sight,' and cultivating a desire to serve and 'spread the love of Jesus' at home, on campus, and worldwide.</t>
         </is>
       </c>
+      <c r="I8" s="16" t="inlineStr">
+        <is>
+          <t>Mrs. Thompson wants students pointed back to 'the Lord's plan for their lives' and, with Nicole, is 'very passionate about apologetics' — kids should believe it, know why they believe it, and be able to defend it when they leave the classroom. She said the false-beliefs sections (which they call the 'isms') and the 'Mars Hill section' are eye-opening and help kids escape the 'Christian school bubble,' leaving knowing 'the Lord has a plan and the Bible is truth.'</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -6197,6 +6233,11 @@
           <t>User-friendly, easy-to-implement resources with sound doctrine that teachers can 'trust and count on' and adapt; specifically discussion questions tied to passages or topics, and 'spiritual discipline toolboxes' with experiences teachers can run. She stressed many capable teachers simply need the tools put 'in their hands' and that ready-made, trustworthy material saves them time.</t>
         </is>
       </c>
+      <c r="I9" s="16" t="inlineStr">
+        <is>
+          <t>Mrs. Thompson loves the added videos — short, to the point, and good at filling gaps. The reflection journal questions (new to her this year) 'got kids thinking,' and her students love acting out lessons; she noted the inductive-study observations and markings in 5th/6th 'take a long time' to balance.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -6229,6 +6270,11 @@
           <t>It depends heavily on the activity. She half-joked she can get kindergarteners to do imaginative prayer for 40 minutes and cited the 'a minute for however old you are' rule of thumb, but said if discussion is challenging, on the 'forefront of what they want to know,' and sparks curiosity, engagement goes well beyond that—and experiential, participatory activities with buy-in can last even longer. Bible classes run 30-40 minutes, typically ~20 minutes high-content teaching and ~20 minutes discussion.</t>
         </is>
       </c>
+      <c r="I10" s="16" t="inlineStr">
+        <is>
+          <t>Class periods are 80 minutes and mostly discussion; Mrs. Thompson estimated roughly 40 minutes for teaching and discussion and about 20 minutes for reading and activities combined.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -6265,6 +6311,11 @@
           <t>Speaking of middle school broadly rather than by grade, she pointed to discussion (especially curiosity-driven, 'wonder question' discussion), experiential and service opportunities, spiritual disciplines, and end-of-year/capstone projects as most powerful and engaging.</t>
         </is>
       </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Sixth graders enjoy the activities, especially the drawing activities (she cited the 'benevolent wisdom' drawing activity); across the board kids love acting out lessons and responded well to the reflection journal questions.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -6305,6 +6356,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>Everything runs on a Vibe smartboard; Mrs. Thompson projects the teacher window (not the student view) as an extended screen so she can highlight text for students to read rather than just listen to her. The school is not heavy on technology — one shared set that everyone uses.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -6337,6 +6393,11 @@
           <t>Taking ownership of their faith and figuring out 'who they are'; 'wonder questions' about God and a world that is 'groaning' and hard; and sensitive personal 'triggers'—family and real-life situations that surface during stories/lessons—that students are wrestling with.</t>
         </is>
       </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Mrs. Thompson said her 5th/6th graders wrestle (as adults do) with how a good and loving God causes or allows suffering — e.g., in Job you can give them the definitions but genuinely understanding it is hard — and with how to follow Christ when the pressures of the world come in.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -6369,6 +6430,11 @@
           <t>Yes. Classes work together to lead chapel through the year, and 5th graders write an apologetics 'defend your faith' essay they share with each other. She described a 'spiritual portfolio' of 'relics' of spiritual fruit collected over time that transitions with students to the next grade/school, letting them 'see their faith development along the way'; such capstone projects give students pride and visible growth.</t>
         </is>
       </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>Not as a group, given her small-class dynamics. Instead they do an individual end-of-year project where each student picks a topic, gets criteria, and leads the class through a Bible lesson with an assessment at the end; she values it because Bible can be an uncomfortable class and it gets kids comfortable speaking about Bible topics and leading prayer.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -6401,6 +6467,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Parent engagement is a weak spot — Nicole said parents aren't very engaged on the at-home portal and the school isn't heavy on tech (one shared set). Kids liked the Treehouse login, but Bible-translation mismatches were a challenge (e.g., KJV verses vs. the NLT used at their old school, and the CSB now used by all Bridge 56 students). They rely on a weekly newsletter, weekend prayer-request messages, and sent-home family activities.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -6433,6 +6504,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>Nicole said they give some homework but are 'big on family' and don't believe kids should be in school all day and then face hours of homework. The load leans toward large-scale work — memory verses, study guides, projects, and preparing to teach their Bible lesson — rather than busywork.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -6465,6 +6541,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Mrs. Thompson shows Superbook and Saddleback Kids videos to build background knowledge before a unit, uses the songs on the DeepRoots website, and sometimes shows clips from 'The Chosen' that fit the lesson; older kids have grown more willing to sing the books of the Bible in front of classmates.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -6505,6 +6586,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>Around three minutes; the in-lesson videos kids watch are about two to three minutes.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -6545,6 +6631,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>Maps and timelines are most effective (they help kids see where in the world and when things happened), and she said kids honestly like the cartoon artwork too — her class loved today's illustration of what Deborah probably looked like. Historical artwork has been the least engaging.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
@@ -6585,6 +6676,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>Printables — the whole school does paper-pencil assessments; Mrs. Thompson did digital assessments back when Nicole was in the classroom but prefers paper-pencil copies, which is what they use.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -6617,6 +6713,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>About 50/50; Mrs. Thompson said the 5th/6th grade curriculum is well balanced, the images are engaging, and she particularly likes the headings and captions.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -6649,6 +6750,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
@@ -6681,6 +6787,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I23" s="16" t="inlineStr">
+        <is>
+          <t>No — they are not limited by the amount of material they're allowed to print.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
@@ -6713,6 +6824,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Per the meeting summary, the school fully funds any necessary classroom supplies, so the school (not the teacher) provides the funds.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -6745,6 +6861,11 @@
           <t>Classes run 30-40 minutes, so with ~20 minutes of core content there is roughly another ~20 minutes for discussion or alternative/experiential activities. She affirmed a 'digging deeper' section for schools with longer periods would be helpful, and noted resources can also be 'sprinkled in other moments' of the day (start-of-day activities, houses/projects) rather than all in one block.</t>
         </is>
       </c>
+      <c r="I25" s="16" t="inlineStr">
+        <is>
+          <t>Mrs. Thompson said she 'usually cover[s] almost everything' and has never used an essentials-only list — she likes to go through nearly all the material. Because of the block schedule she sometimes skips or postpones specific pieces (e.g., historical-art days, or the Elizabeth Elliot biography on day nine), which she wouldn't do if she had Bible every day.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -6777,6 +6898,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Yes — 'I think it'd be great.' She was enthusiastic about a multi-subject timeline with clickable summaries and images on empires, literature, music, arts, people, and scientific inventions.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
@@ -6809,6 +6935,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I27" s="16" t="inlineStr">
+        <is>
+          <t>No set limit — 'the screen's on all the time' since everything runs through the smartboard/TV, but students are never on devices personally.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
@@ -6849,6 +6980,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>Mrs. Thompson pointed to the newsletter that tells parents where the class is headed and to sending home family activities (today's encouraged families to read Matthew 5 together); in the younger grades they encourage families to read the Bible stories together.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -6881,6 +7017,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I29" s="16" t="inlineStr">
+        <is>
+          <t>Mrs. Thompson would probably send it home with families with advance permission, but said she would 'absolutely teach it' — 'there's nothing about the Bible that I wouldn't teach' — and already covers God's view on marriage in class. Nicole would be for having teachers teach it and giving resources to parents who don't know how to broach it, with the two of them deciding implementation as a school.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
@@ -6913,6 +7054,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Yes — Mrs. Thompson was interested in a separate logic course taught through videos and reinforced with worksheets.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -6945,6 +7091,11 @@
           <t>Yes. She confirmed a 'digging deeper'/extra section would be useful and suggested it hold spiritual-discipline 'toolbox' ideas tied to what the story is highlighting, 'start your day / end your day' activities, brain-break style items, and topical 'if this arises' guidance with tidbits and resources for sensitive triggers students bring up.</t>
         </is>
       </c>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Yes — she'd use discussion and further Bible reading, with the hope of eventually getting to journaling (she's working on getting better at journaling herself and building it with her students).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -6977,6 +7128,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -7009,6 +7165,11 @@
           <t>She didn't directly rank the two, but leaned strongly toward relational, discussion-based and group/experiential learning as most powerful for middle school, while also valuing individual contemplative disciplines she teaches (e.g., meditation, 'take a minute' to pause and pray without words) where 'the Lord is going to meet each of you differently.'</t>
         </is>
       </c>
+      <c r="I33" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
@@ -7041,6 +7202,11 @@
           <t>A thematic weekly outline with a flexible start-of-day activity, then focused content (~20 min) and discussion (~20 min within a 30-40 min period), woven with an experiential spiritual-discipline element and good discussion questions, framed so teachers understand 'why we do it,' with room to evolve the lesson and adapt to immediate student needs.</t>
         </is>
       </c>
+      <c r="I34" s="16" t="inlineStr">
+        <is>
+          <t>She described a discussion-heavy 80-minute block (she's a self-described 'big talker') where she goes through the full teacher page, eliminating or simplifying some pieces for time or class size — e.g., reading a passage instead of acting it out — with roughly 40 minutes of teaching/discussion and 20 minutes of reading/activities, inductive study now done in school-provided journaling Bibles, and real-life connections (sermons, podcasts, songs). On a topic she loves, like the 'isms,' she said she's been known to turn a 20-minute lesson into three hours.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
@@ -7081,6 +7247,11 @@
           <t>Success shows up as students taking personal ownership of their faith and growing a 'heart for God'—movement she sees made visible through things like the spiritual portfolio of 'relics' of spiritual fruit that tracks a student's faith development over time, and through genuine worshipful, fruitful response rather than just completing content.</t>
         </is>
       </c>
+      <c r="I35" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -7121,6 +7292,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <t>Historical artwork has been the least engaging visual style for her students; they respond better to cartoon-style artwork, maps, and timelines.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -7153,6 +7329,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I37" s="16" t="inlineStr">
+        <is>
+          <t>The short, point-driven videos that 'fill in some gaps' are what she values most, plus background-knowledge/intro clips before a unit — she named Superbook, Saddleback Kids, and 'The Chosen' clips, along with the songs on the DeepRoots site.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -7189,6 +7370,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="I38" s="16" t="inlineStr">
+        <is>
+          <t>She didn't give a number, but she repeatedly said her students 'love acting out' lessons, suggesting role-play lands well with her classes; in her smallest groups (one class of four, last year's of seven) she sometimes just reads the material instead.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
@@ -7221,6 +7407,11 @@
           <t>She cautioned against faith learning becoming 'just boxes that we're checking' and against overly rigid, minute-by-minute daily scripts, preferring flexible weekly thematic outlines teachers can adapt; she did not otherwise enumerate disliked curriculum elements.</t>
         </is>
       </c>
+      <c r="I39" s="16" t="inlineStr">
+        <is>
+          <t>She didn't single out curriculum elements she dislikes; pressed by Pat for 'the good and the bad,' her main friction was time/the block schedule and that the inductive-study markings and observations 'take a long time' to balance in 5th/6th grade.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
@@ -7253,6 +7444,11 @@
           <t>Challenging discussion on the 'forefront of what they want to know' that inspires curiosity, experiential activities where students have buy-in and participate, service and 'wonder question' conversations met safely and with God's truth, and opportunities to take ownership of their faith.</t>
         </is>
       </c>
+      <c r="I40" s="16" t="inlineStr">
+        <is>
+          <t>Discussion (her classes are discussion-heavy), acting out lessons, the reflection journal questions, drawing activities (e.g., 'benevolent wisdom'), maps and timelines, cartoon artwork, and short point-driven videos all hold her students' attention.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
@@ -7287,6 +7483,11 @@
       <c r="H41" s="16" t="inlineStr">
         <is>
           <t>A reliable, sound-doctrine DeepRoots framework that is user-friendly and 'easy to implement'—flexible weekly thematic outlines rather than rigid scripts, discussion questions, spiritual-discipline 'toolboxes' and experiential opportunities with the 'why' explained so teachers aren't hesitant, a 'digging deeper' section for extra time, and topical 'if this arises' guidance for sensitive triggers—tools teachers can trust and 'make their own' for the students in front of them.</t>
+        </is>
+      </c>
+      <c r="I41" s="16" t="inlineStr">
+        <is>
+          <t>She effectively described DeepRoots as already easy to teach and impactful — she loves it and points to the short videos, the apologetics 'isms'/Mars Hill content, the reflection journals, and the well-balanced pages — with the one real need being adaptability to a block schedule so teachers covering Bible every other day can get through all the units.</t>
         </is>
       </c>
     </row>
@@ -7299,6 +7500,7 @@
       <c r="F42" s="16" t="inlineStr"/>
       <c r="G42" s="16" t="inlineStr"/>
       <c r="H42" s="16" t="inlineStr"/>
+      <c r="I42" s="16" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
@@ -7313,6 +7515,7 @@
       <c r="F43" s="17" t="inlineStr"/>
       <c r="G43" s="17" t="inlineStr"/>
       <c r="H43" s="17" t="inlineStr"/>
+      <c r="I43" s="17" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="22" t="inlineStr"/>
@@ -7327,6 +7530,7 @@
       <c r="F44" s="22" t="inlineStr"/>
       <c r="G44" s="22" t="inlineStr"/>
       <c r="H44" s="22" t="inlineStr"/>
+      <c r="I44" s="22" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="18" t="inlineStr"/>
@@ -7361,6 +7565,11 @@
           <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
         </is>
       </c>
+      <c r="I45" s="18" t="inlineStr">
+        <is>
+          <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="16" t="inlineStr"/>
@@ -7379,6 +7588,7 @@
       <c r="F46" s="16" t="inlineStr"/>
       <c r="G46" s="16" t="inlineStr"/>
       <c r="H46" s="16" t="inlineStr"/>
+      <c r="I46" s="16" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr"/>
@@ -7397,6 +7607,7 @@
       <c r="F47" s="16" t="inlineStr"/>
       <c r="G47" s="16" t="inlineStr"/>
       <c r="H47" s="16" t="inlineStr"/>
+      <c r="I47" s="16" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr"/>
@@ -7415,6 +7626,7 @@
       <c r="F48" s="16" t="inlineStr"/>
       <c r="G48" s="16" t="inlineStr"/>
       <c r="H48" s="16" t="inlineStr"/>
+      <c r="I48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr"/>
@@ -7433,6 +7645,7 @@
       <c r="F49" s="16" t="inlineStr"/>
       <c r="G49" s="16" t="inlineStr"/>
       <c r="H49" s="16" t="inlineStr"/>
+      <c r="I49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr"/>
@@ -7451,6 +7664,7 @@
       <c r="F50" s="16" t="inlineStr"/>
       <c r="G50" s="16" t="inlineStr"/>
       <c r="H50" s="16" t="inlineStr"/>
+      <c r="I50" s="16" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr"/>
@@ -7465,6 +7679,7 @@
       <c r="F51" s="16" t="inlineStr"/>
       <c r="G51" s="16" t="inlineStr"/>
       <c r="H51" s="16" t="inlineStr"/>
+      <c r="I51" s="16" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr"/>
@@ -7475,6 +7690,7 @@
       <c r="F52" s="16" t="inlineStr"/>
       <c r="G52" s="16" t="inlineStr"/>
       <c r="H52" s="16" t="inlineStr"/>
+      <c r="I52" s="16" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="22" t="inlineStr"/>
@@ -7489,6 +7705,7 @@
       <c r="F53" s="22" t="inlineStr"/>
       <c r="G53" s="22" t="inlineStr"/>
       <c r="H53" s="22" t="inlineStr"/>
+      <c r="I53" s="22" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr"/>
@@ -7521,6 +7738,11 @@
       <c r="H54" s="18" t="inlineStr">
         <is>
           <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
+        </is>
+      </c>
+      <c r="I54" s="18" t="inlineStr">
+        <is>
+          <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7537,6 +7759,7 @@
       <c r="F55" s="16" t="inlineStr"/>
       <c r="G55" s="16" t="inlineStr"/>
       <c r="H55" s="16" t="inlineStr"/>
+      <c r="I55" s="16" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr"/>
@@ -7551,6 +7774,7 @@
       <c r="F56" s="16" t="inlineStr"/>
       <c r="G56" s="16" t="inlineStr"/>
       <c r="H56" s="16" t="inlineStr"/>
+      <c r="I56" s="16" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr"/>
@@ -7565,6 +7789,7 @@
       <c r="F57" s="16" t="inlineStr"/>
       <c r="G57" s="16" t="inlineStr"/>
       <c r="H57" s="16" t="inlineStr"/>
+      <c r="I57" s="16" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr"/>
@@ -7579,6 +7804,7 @@
       <c r="F58" s="16" t="inlineStr"/>
       <c r="G58" s="16" t="inlineStr"/>
       <c r="H58" s="16" t="inlineStr"/>
+      <c r="I58" s="16" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr"/>
@@ -7593,6 +7819,7 @@
       <c r="F59" s="16" t="inlineStr"/>
       <c r="G59" s="16" t="inlineStr"/>
       <c r="H59" s="16" t="inlineStr"/>
+      <c r="I59" s="16" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr"/>
@@ -7607,6 +7834,7 @@
       <c r="F60" s="16" t="inlineStr"/>
       <c r="G60" s="16" t="inlineStr"/>
       <c r="H60" s="16" t="inlineStr"/>
+      <c r="I60" s="16" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr"/>
@@ -7617,6 +7845,7 @@
       <c r="F61" s="16" t="inlineStr"/>
       <c r="G61" s="16" t="inlineStr"/>
       <c r="H61" s="16" t="inlineStr"/>
+      <c r="I61" s="16" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="22" t="inlineStr"/>
@@ -7631,6 +7860,7 @@
       <c r="F62" s="22" t="inlineStr"/>
       <c r="G62" s="22" t="inlineStr"/>
       <c r="H62" s="22" t="inlineStr"/>
+      <c r="I62" s="22" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="18" t="inlineStr"/>
@@ -7663,6 +7893,11 @@
       <c r="H63" s="18" t="inlineStr">
         <is>
           <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
+        </is>
+      </c>
+      <c r="I63" s="18" t="inlineStr">
+        <is>
+          <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7679,6 +7914,7 @@
       <c r="F64" s="16" t="inlineStr"/>
       <c r="G64" s="16" t="inlineStr"/>
       <c r="H64" s="16" t="inlineStr"/>
+      <c r="I64" s="16" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr"/>
@@ -7693,6 +7929,7 @@
       <c r="F65" s="16" t="inlineStr"/>
       <c r="G65" s="16" t="inlineStr"/>
       <c r="H65" s="16" t="inlineStr"/>
+      <c r="I65" s="16" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="16" t="inlineStr"/>
@@ -7707,6 +7944,7 @@
       <c r="F66" s="16" t="inlineStr"/>
       <c r="G66" s="16" t="inlineStr"/>
       <c r="H66" s="16" t="inlineStr"/>
+      <c r="I66" s="16" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr"/>
@@ -7721,6 +7959,7 @@
       <c r="F67" s="16" t="inlineStr"/>
       <c r="G67" s="16" t="inlineStr"/>
       <c r="H67" s="16" t="inlineStr"/>
+      <c r="I67" s="16" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr"/>
@@ -7735,6 +7974,7 @@
       <c r="F68" s="16" t="inlineStr"/>
       <c r="G68" s="16" t="inlineStr"/>
       <c r="H68" s="16" t="inlineStr"/>
+      <c r="I68" s="16" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr"/>
@@ -7749,6 +7989,7 @@
       <c r="F69" s="16" t="inlineStr"/>
       <c r="G69" s="16" t="inlineStr"/>
       <c r="H69" s="16" t="inlineStr"/>
+      <c r="I69" s="16" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="16" t="inlineStr"/>
@@ -7759,6 +8000,162 @@
       <c r="F70" s="16" t="inlineStr"/>
       <c r="G70" s="16" t="inlineStr"/>
       <c r="H70" s="16" t="inlineStr"/>
+      <c r="I70" s="16" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="22" t="inlineStr"/>
+      <c r="B71" s="22" t="inlineStr"/>
+      <c r="C71" s="22" t="inlineStr">
+        <is>
+          <t>IRONBRIDGE interview — Ironbridge Christian Academy (Nicole Burchett + Crystal Thompson), 2026-10-05  |  Attendees: Troy Winkler, Pat Williamson, Taylor Chartier, Lisa Van Vlear, Will Tuomey</t>
+        </is>
+      </c>
+      <c r="D71" s="22" t="inlineStr"/>
+      <c r="E71" s="22" t="inlineStr"/>
+      <c r="F71" s="22" t="inlineStr"/>
+      <c r="G71" s="22" t="inlineStr"/>
+      <c r="H71" s="22" t="inlineStr"/>
+      <c r="I71" s="22" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="18" t="inlineStr"/>
+      <c r="B72" s="18" t="inlineStr"/>
+      <c r="C72" s="18" t="inlineStr">
+        <is>
+          <t>Team member</t>
+        </is>
+      </c>
+      <c r="D72" s="18" t="inlineStr">
+        <is>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — teacher/admin — 2026-09-24</t>
+        </is>
+      </c>
+      <c r="E72" s="18" t="inlineStr">
+        <is>
+          <t>Atlantic Shores Christian School (VA) — current K-5 use — 9/29/26</t>
+        </is>
+      </c>
+      <c r="F72" s="18" t="inlineStr">
+        <is>
+          <t>Will Weaver — Des Moines Christian School (IA) — Head of Spiritual Formation (admin) — 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G72" s="18" t="inlineStr">
+        <is>
+          <t>Horizon Christian Elementary (OR) — current K-5 use — 9/28/26</t>
+        </is>
+      </c>
+      <c r="H72" s="18" t="inlineStr">
+        <is>
+          <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
+        </is>
+      </c>
+      <c r="I72" s="18" t="inlineStr">
+        <is>
+          <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="16" t="inlineStr"/>
+      <c r="B73" s="16" t="inlineStr"/>
+      <c r="C73" s="16" t="inlineStr">
+        <is>
+          <t>Troy Winkler</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr"/>
+      <c r="E73" s="16" t="inlineStr"/>
+      <c r="F73" s="16" t="inlineStr"/>
+      <c r="G73" s="16" t="inlineStr"/>
+      <c r="H73" s="16" t="inlineStr"/>
+      <c r="I73" s="16" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="16" t="inlineStr"/>
+      <c r="B74" s="16" t="inlineStr"/>
+      <c r="C74" s="16" t="inlineStr">
+        <is>
+          <t>Pat Williamson</t>
+        </is>
+      </c>
+      <c r="D74" s="16" t="inlineStr"/>
+      <c r="E74" s="16" t="inlineStr"/>
+      <c r="F74" s="16" t="inlineStr"/>
+      <c r="G74" s="16" t="inlineStr"/>
+      <c r="H74" s="16" t="inlineStr"/>
+      <c r="I74" s="16" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="16" t="inlineStr"/>
+      <c r="B75" s="16" t="inlineStr"/>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>Taylor Chartier</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr"/>
+      <c r="E75" s="16" t="inlineStr"/>
+      <c r="F75" s="16" t="inlineStr"/>
+      <c r="G75" s="16" t="inlineStr"/>
+      <c r="H75" s="16" t="inlineStr"/>
+      <c r="I75" s="16" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="16" t="inlineStr"/>
+      <c r="B76" s="16" t="inlineStr"/>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>Lisa Van Vlear</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr"/>
+      <c r="E76" s="16" t="inlineStr"/>
+      <c r="F76" s="16" t="inlineStr"/>
+      <c r="G76" s="16" t="inlineStr"/>
+      <c r="H76" s="16" t="inlineStr"/>
+      <c r="I76" s="16" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="16" t="inlineStr"/>
+      <c r="B77" s="16" t="inlineStr"/>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>Will Tuomey</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr"/>
+      <c r="E77" s="16" t="inlineStr"/>
+      <c r="F77" s="16" t="inlineStr"/>
+      <c r="G77" s="16" t="inlineStr"/>
+      <c r="H77" s="16" t="inlineStr"/>
+      <c r="I77" s="16" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="16" t="inlineStr"/>
+      <c r="B78" s="16" t="inlineStr"/>
+      <c r="C78" s="16" t="inlineStr">
+        <is>
+          <t>Overall / key takeaways for the curriculum</t>
+        </is>
+      </c>
+      <c r="D78" s="16" t="inlineStr"/>
+      <c r="E78" s="16" t="inlineStr"/>
+      <c r="F78" s="16" t="inlineStr"/>
+      <c r="G78" s="16" t="inlineStr"/>
+      <c r="H78" s="16" t="inlineStr"/>
+      <c r="I78" s="16" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="16" t="inlineStr"/>
+      <c r="B79" s="16" t="inlineStr"/>
+      <c r="C79" s="16" t="inlineStr"/>
+      <c r="D79" s="16" t="inlineStr"/>
+      <c r="E79" s="16" t="inlineStr"/>
+      <c r="F79" s="16" t="inlineStr"/>
+      <c r="G79" s="16" t="inlineStr"/>
+      <c r="H79" s="16" t="inlineStr"/>
+      <c r="I79" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Dayspring (Donna Hurley + Angela Adams) interview
Oct 6 interview with Dayspring Christian Academy (Lancaster, PA):
Donna Hurley (Director of Curriculum & Instruction) and Angela Adams
(upper-school Bible dept chair). DeepRoots attendees: Troy Winkler,
Lisa Van Vlear, Nancy Wood.

Added a Dayspring column on the All Interviews master (gold) plus a
dedicated interview tab in the Q&A workbook. Dayspring uses no
purchased Bible curriculum (teachers author everything) - strong
demand signal. Not a round-2 outreach recipient, so no tracker row.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUC7AKNsC5W1a963Yi5JKY
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -5888,7 +5888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5900,6 +5900,7 @@
     <col width="58" customWidth="1" min="7" max="7"/>
     <col width="58" customWidth="1" min="8" max="8"/>
     <col width="58" customWidth="1" min="9" max="9"/>
+    <col width="58" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5955,6 +5956,11 @@
           <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
         </is>
       </c>
+      <c r="J2" s="15" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy (PA) — Donna Hurley + Angela Adams — 2026-10-06</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -5992,6 +5998,11 @@
           <t>Unconventional structure: 'Bridge 56' covers 5th and 6th graders ('that step out of middle school'), and junior high is 7th and 8th grade. Students are grouped by developmental stage, with 5th graders together and 6th graders together in separate classes rather than all four mixed.</t>
         </is>
       </c>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>Middle school is grades 6 through 8; sixth grade is considered the move into middle school (Angela Adams).</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -6029,6 +6040,11 @@
           <t>Nicole said the developmental gap is why the grades are separated — there is a 'huge difference between a kindergartener and a fifth grader, but then also a fifth grader and an eighth grader or a sixth grader and an eighth grader,' which drives the Bridge 56 vs. junior-high split. Specific per-grade spiritual/emotional distinctions were not detailed.</t>
         </is>
       </c>
+      <c r="J4" s="16" t="inlineStr">
+        <is>
+          <t>Sixth graders are largely concrete thinkers still in an 'elementary mentality,' beginning to move toward abstract thought and needing structured building from the concrete; their faith tends to be home-driven and childlike, self-focused, and they often just repeat back what the teacher wants for a good grade. Seventh graders can take on research-based projects and discussion but can be 'squirrely and impulsive,' needing a firm and consistent hand in classroom management, and begin making their faith their own. Eighth graders move further into abstract thinking and are more willing to put real reflection into writing. Across the band students care intensely what peers think and transition from parent-driven faith to deciding whether they believe it for themselves (Angela Adams and Donna Hurley).</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -6074,6 +6090,11 @@
           <t>They are a covenant school, so families should be churched, but public-school transfers often lack depth. Mrs. Thompson and Nicole send home church-event info and family activities, text weekend prayer-request messages, and encourage storybook Bibles and apps at home; Nicole tells parents up front that they no longer teach foundational Bible stories and gives them resources to prep kids. She cited a student who didn't know why Adam and Eve left the garden, which made jumping into Job hard.</t>
         </is>
       </c>
+      <c r="J5" s="16" t="inlineStr">
+        <is>
+          <t>Angela Adams stressed never assuming all students know the Bible stories; some hear them for the first time even in a Christian school. She shared the seventh-grade teacher's approach: keep reading, acting out, or showing a good video of each story so a child who never heard it can follow, while sharing deeper insights from the Bible Recap and Enduring Word commentary to keep churched students engaged, and asking students what they learned about God, not just the story. She recounted a new-believer family who, after their son struggled with an Acts chapter 2 handout, asked to sit down and do it with him at home because they had never read the book of Acts.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -6119,6 +6140,11 @@
           <t>They use DeepRoots and love it; Mrs. Thompson especially loves the videos in the 5th/6th grade curriculum. Her main frustration is not the curriculum but time — moving to an 80-minute block every other day makes finishing all the units a challenge, and as a self-described 'big talker' she doesn't want to skip the rich content.</t>
         </is>
       </c>
+      <c r="J6" s="16" t="inlineStr">
+        <is>
+          <t>The school has no purchased curriculum; teachers write their own, working from internally developed curriculum guides and objectives for each Bible course and building on what prior teachers have done. Angela Adams noted the guides have good outlines, content, and key chapters but little interactive student material, so the seventh-grade teacher had to create note-taking sheets and scripts herself. They agreed it would be nice to have a real curriculum to look at and lean on.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
@@ -6156,6 +6182,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>Apologetics and 'defending scripture' — the veracity of scripture and archaeological evidence (Noah's Ark, the Tower of Babel, messianic prophecies); world-history timelines showing where events fall; vocabulary instruction; geography (Israel, Syria, Lebanon, the Babylonian and Roman empires); applications and takeaways plus reflection on what each story teaches about who God is; and resources pointing students to where they can go to learn more (Angela Adams and Donna Hurley).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
@@ -6193,6 +6224,11 @@
           <t>Mrs. Thompson wants students pointed back to 'the Lord's plan for their lives' and, with Nicole, is 'very passionate about apologetics' — kids should believe it, know why they believe it, and be able to defend it when they leave the classroom. She said the false-beliefs sections (which they call the 'isms') and the 'Mars Hill section' are eye-opening and help kids escape the 'Christian school bubble,' leaving knowing 'the Lord has a plan and the Bible is truth.'</t>
         </is>
       </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>A love for the word of God as living, active, and relevant; knowing the salvation message and gospel; understanding theological terms students often take for granted (salvation, justification, atonement, peace with God) — Dayspring is 'really big in defining words'; the character of God, who he is and what he loves and hates and how we respond (noted by Lisa Van Vlear); and, as Donna Hurley prayed, growing into men and women who honor God with their lives.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
@@ -6238,6 +6274,11 @@
           <t>Mrs. Thompson loves the added videos — short, to the point, and good at filling gaps. The reflection journal questions (new to her this year) 'got kids thinking,' and her students love acting out lessons; she noted the inductive-study observations and markings in 5th/6th 'take a long time' to balance.</t>
         </is>
       </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>After Nancy Wood clarified the question as what they would most want in a curriculum: object lessons that grab attention and stick; hands-on things students can do and move around during the long block; and 'learning supports' offering student choice so one student can take an artistic route while another does drama or a script to reach the same objective. They also value videos, drama and creative activities, note-taking sheets, and slideshow projects, plus fresh ideas for student engagement and pointers to further resources (Angela Adams and Donna Hurley).</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
@@ -6275,6 +6316,11 @@
           <t>Class periods are 80 minutes and mostly discussion; Mrs. Thompson estimated roughly 40 minutes for teaching and discussion and about 20 minutes for reading and activities combined.</t>
         </is>
       </c>
+      <c r="J10" s="16" t="inlineStr">
+        <is>
+          <t>Angela Adams said sixth graders can handle up to 30 minutes of instruction if they are actively engaged in something like note-taking; the seventh-grade teacher agreed on about 30 minutes. Reading is about 15 minutes (up to 15-20), discussion 15-20 minutes, and activities 20-30 minutes (the seventh-grade teacher said up to 40 when students are actively doing something). Donna Hurley's rule of thumb: 20-25 minutes of teaching, then do something with it, then back into another 15-20 minutes, yielding a balanced 40-45 minutes of teaching across the 80-minute block.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -6316,6 +6362,11 @@
           <t>Sixth graders enjoy the activities, especially the drawing activities (she cited the 'benevolent wisdom' drawing activity); across the board kids love acting out lessons and responded well to the reflection journal questions.</t>
         </is>
       </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Skits are the biggest draw — students love acting out stories, and modernizing parables (one group moved a parable to the local McDonald's). Also Acts chapter posters that form a timeline of Paul's final journey, the 'philosophy chair' discussion activity, Post-it sticky-note station rotations, group and partner/table talk, and slideshow creation (a seventh-grade favorite). Above all, middle schoolers 'just need to move' (Angela Adams).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
@@ -6361,6 +6412,11 @@
           <t>Everything runs on a Vibe smartboard; Mrs. Thompson projects the teacher window (not the student view) as an extended screen so she can highlight text for students to read rather than just listen to her. The school is not heavy on technology — one shared set that everyone uses.</t>
         </is>
       </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Teachers use projectors to display images and teaching material, play educational videos occasionally, and run review games like Kahoot, which students love. They also use computers for typing reports or papers, though they still value handwritten work (Angela Adams).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
@@ -6398,6 +6454,11 @@
           <t>Mrs. Thompson said her 5th/6th graders wrestle (as adults do) with how a good and loving God causes or allows suffering — e.g., in Job you can give them the definitions but genuinely understanding it is hard — and with how to follow Christ when the pressures of the world come in.</t>
         </is>
       </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Sixth graders ask every year 'Where did evil come from? Did God create evil?' — and that returns in eighth grade with Job and Satan. Also understanding the gospel, the chronological order of events, and basic theology terms like salvation and atonement (Angela Adams noted atonement lands harder because New Testament precedes Old Testament). The seventh-grade teacher often heard 'Why did the people in the Old Testament act the way they did?' along with questions about cultural differences.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -6435,6 +6496,11 @@
           <t>Not as a group, given her small-class dynamics. Instead they do an individual end-of-year project where each student picks a topic, gets criteria, and leads the class through a Bible lesson with an assessment at the end; she values it because Bible can be an uncomfortable class and it gets kids comfortable speaking about Bible topics and leading prayer.</t>
         </is>
       </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>The seventh-grade teacher said 'maybe'; Angela Adams said she would, depending on what the project was.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
@@ -6472,6 +6538,11 @@
           <t>Parent engagement is a weak spot — Nicole said parents aren't very engaged on the at-home portal and the school isn't heavy on tech (one shared set). Kids liked the Treehouse login, but Bible-translation mismatches were a challenge (e.g., KJV verses vs. the NLT used at their old school, and the CSB now used by all Bridge 56 students). They rely on a weekly newsletter, weekend prayer-request messages, and sent-home family activities.</t>
         </is>
       </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>A monthly memory verse is sent home to the whole family through a weekly newsletter called 'the beacon' (lower school learns the same verse broken into smaller chunks). Donna Hurley also cited schoolwide practices: a principal's 'word of the day' tied to scripture during homeroom, daily homeroom prayer, and gender- and grade-separated prayer groups once every six-day rotation. A parent recently emailed asking whether students learn the vocabulary behind the monthly verses.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
@@ -6509,6 +6580,11 @@
           <t>Nicole said they give some homework but are 'big on family' and don't believe kids should be in school all day and then face hours of homework. The load leans toward large-scale work — memory verses, study guides, projects, and preparing to teach their Bible lesson — rather than busywork.</t>
         </is>
       </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>Homework is minimal for Bible — mainly Bible memory, which is also covered in class so students memorize it with the teacher as well as reviewing it at home (Angela Adams).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -6546,6 +6622,11 @@
           <t>Mrs. Thompson shows Superbook and Saddleback Kids videos to build background knowledge before a unit, uses the songs on the DeepRoots website, and sometimes shows clips from 'The Chosen' that fit the lesson; older kids have grown more willing to sing the books of the Bible in front of classmates.</t>
         </is>
       </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Angela Adams uses a 'Heroes of the Faith' video on Judas Maccabeus for the intertestamental period, Eric Ludy's gospel video on YouTube, Got Questions for some theology, snippets of The Chosen, and the Bible Project to introduce books of the Bible. The seventh-grade teacher uses Revelation Media's iBible videos for Genesis, Got Questions, Ark in the Darkness, Prince of Egypt (Moses, the plagues, Passover), a Ten Commandments peg-memorization system with songs, Gideon Films YouTube videos, the Bible Project, House of David snippets, Sight and Sound, and Piercing Word.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
@@ -6591,6 +6672,11 @@
           <t>Around three minutes; the in-lesson videos kids watch are about two to three minutes.</t>
         </is>
       </c>
+      <c r="J18" s="16" t="inlineStr">
+        <is>
+          <t>Three minutes or more for a video, unless showing a full-length movie.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
@@ -6636,6 +6722,11 @@
           <t>Maps and timelines are most effective (they help kids see where in the world and when things happened), and she said kids honestly like the cartoon artwork too — her class loved today's illustration of what Deborah probably looked like. Historical artwork has been the least engaging.</t>
         </is>
       </c>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>They liked all the visual options offered and couldn't pick a favorite; 'visuals are great,' and a mix of text and visuals is nice.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
@@ -6681,6 +6772,11 @@
           <t>Printables — the whole school does paper-pencil assessments; Mrs. Thompson did digital assessments back when Nicole was in the classroom but prefers paper-pencil copies, which is what they use.</t>
         </is>
       </c>
+      <c r="J20" s="16" t="inlineStr">
+        <is>
+          <t>Both wrote printables, though digital is occasionally fine — for example a teacher's slideshow presentation (Angela Adams and Donna Hurley).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
@@ -6718,6 +6814,11 @@
           <t>About 50/50; Mrs. Thompson said the 5th/6th grade curriculum is well balanced, the images are engaging, and she particularly likes the headings and captions.</t>
         </is>
       </c>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>A mix of text and visuals is nice.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -6755,6 +6856,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>Not framed around the curriculum artifact itself, but Donna Hurley said the goal is for Bible class to be 'enjoyable... engaging... welcoming and not dull,' citing Jesus as the master teacher who drew people in; both prized object lessons that grab attention and stick, drama, and movement to keep students engaged.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
@@ -6792,6 +6898,11 @@
           <t>No — they are not limited by the amount of material they're allowed to print.</t>
         </is>
       </c>
+      <c r="J23" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
@@ -6829,6 +6940,11 @@
           <t>Per the meeting summary, the school fully funds any necessary classroom supplies, so the school (not the teacher) provides the funds.</t>
         </is>
       </c>
+      <c r="J24" s="16" t="inlineStr">
+        <is>
+          <t>The school has a budget that covers supplies as long as requests are submitted a year ahead; they also have 'very giving' parents who are kind and helpful, though they try not to ask too much of them (Angela Adams).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
@@ -6866,6 +6982,11 @@
           <t>Mrs. Thompson said she 'usually cover[s] almost everything' and has never used an essentials-only list — she likes to go through nearly all the material. Because of the block schedule she sometimes skips or postpones specific pieces (e.g., historical-art days, or the Elizabeth Elliot biography on day nine), which she wouldn't do if she had Bible every day.</t>
         </is>
       </c>
+      <c r="J25" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="inlineStr">
@@ -6903,6 +7024,11 @@
           <t>Yes — 'I think it'd be great.' She was enthusiastic about a multi-subject timeline with clickable summaries and images on empires, literature, music, arts, people, and scientific inventions.</t>
         </is>
       </c>
+      <c r="J26" s="16" t="inlineStr">
+        <is>
+          <t>Strong interest. Both wanted world-history timelines so students see where biblical events fall; Donna Hurley said 'the timeline is such a big deal,' that her own timeline helps her place things and gives the big-picture continuity, and that comparing scripture with world history conveys 'this actually happened.' Angela Adams tied it to seventh-grade ancient-history study and wanted geography woven in (the clickable-media specifics were not asked verbatim).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="inlineStr">
@@ -6940,6 +7066,11 @@
           <t>No set limit — 'the screen's on all the time' since everything runs through the smartboard/TV, but students are never on devices personally.</t>
         </is>
       </c>
+      <c r="J27" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="16" t="inlineStr">
@@ -6985,6 +7116,11 @@
           <t>Mrs. Thompson pointed to the newsletter that tells parents where the class is headed and to sending home family activities (today's encouraged families to read Matthew 5 together); in the younger grades they encourage families to read the Bible stories together.</t>
         </is>
       </c>
+      <c r="J28" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="16" t="inlineStr">
@@ -7022,6 +7158,11 @@
           <t>Mrs. Thompson would probably send it home with families with advance permission, but said she would 'absolutely teach it' — 'there's nothing about the Bible that I wouldn't teach' — and already covers God's view on marriage in class. Nicole would be for having teachers teach it and giving resources to parents who don't know how to broach it, with the two of them deciding implementation as a school.</t>
         </is>
       </c>
+      <c r="J29" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
@@ -7059,6 +7200,11 @@
           <t>Yes — Mrs. Thompson was interested in a separate logic course taught through videos and reinforced with worksheets.</t>
         </is>
       </c>
+      <c r="J30" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="16" t="inlineStr">
@@ -7096,6 +7242,11 @@
           <t>Yes — she'd use discussion and further Bible reading, with the hope of eventually getting to journaling (she's working on getting better at journaling herself and building it with her students).</t>
         </is>
       </c>
+      <c r="J31" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="16" t="inlineStr">
@@ -7133,6 +7284,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="J32" s="16" t="inlineStr">
+        <is>
+          <t>They prefer printables but would welcome a textbook-style reference; Donna Hurley specifically wished for a resource that points students to where they can go to learn more — information 'at the fingertips' — without relying on phones or QR codes.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="16" t="inlineStr">
@@ -7170,6 +7326,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="J33" s="16" t="inlineStr">
+        <is>
+          <t>Both value group and discussion work — students love partner and table talk, group skits, and philosophy-chair debate — while also building an individual written-reflection component in personal notebooks where students record their own takeaways; Donna Hurley added that privacy matters, since ungraded reflection lets students respond honestly (Donna Hurley and Angela Adams).</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
@@ -7207,6 +7368,11 @@
           <t>She described a discussion-heavy 80-minute block (she's a self-described 'big talker') where she goes through the full teacher page, eliminating or simplifying some pieces for time or class size — e.g., reading a passage instead of acting it out — with roughly 40 minutes of teaching/discussion and 20 minutes of reading/activities, inductive study now done in school-provided journaling Bibles, and real-life connections (sermons, podcasts, songs). On a topic she loves, like the 'isms,' she said she's been known to turn a 20-minute lesson into three hours.</t>
         </is>
       </c>
+      <c r="J34" s="16" t="inlineStr">
+        <is>
+          <t>Angela Adams typically opens with Bible memory through a game on the monthly verse (about 15-20 minutes), then teaches with movement and changing activities, ending with students reflecting on and recording their learning. Donna Hurley described 20-25 minutes of teaching, then doing something with it, then returning to teaching, balanced with learning supports — enjoyable and engaging, 'not all fun and games' but never dull. Students bring and use their Bibles in every class.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="16" t="inlineStr">
@@ -7252,6 +7418,11 @@
           <t>Not directly addressed in this interview.</t>
         </is>
       </c>
+      <c r="J35" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="16" t="inlineStr">
@@ -7297,6 +7468,11 @@
           <t>Historical artwork has been the least engaging visual style for her students; they respond better to cartoon-style artwork, maps, and timelines.</t>
         </is>
       </c>
+      <c r="J36" s="16" t="inlineStr">
+        <is>
+          <t>Not directly addressed in this interview.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="16" t="inlineStr">
@@ -7334,6 +7510,11 @@
           <t>The short, point-driven videos that 'fill in some gaps' are what she values most, plus background-knowledge/intro clips before a unit — she named Superbook, Saddleback Kids, and 'The Chosen' clips, along with the songs on the DeepRoots site.</t>
         </is>
       </c>
+      <c r="J37" s="16" t="inlineStr">
+        <is>
+          <t>They would value more vetted apologetics and archaeological-evidence videos (the former Old Testament teacher said it 'would be awesome to have more resources in place' for topics like Noah's Ark and the Tower of Babel) and short clips that introduce books of the Bible, such as the Bible Project, that follow scripture closely (Angela Adams).</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="16" t="inlineStr">
@@ -7375,6 +7556,11 @@
           <t>She didn't give a number, but she repeatedly said her students 'love acting out' lessons, suggesting role-play lands well with her classes; in her smallest groups (one class of four, last year's of seven) she sometimes just reads the material instead.</t>
         </is>
       </c>
+      <c r="J38" s="16" t="inlineStr">
+        <is>
+          <t>No 1-10 rating was given, but skits and acting out stories are among students' most-loved engagements; Angela Adams said her students light up when told they will act something out and don't even need a script.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="16" t="inlineStr">
@@ -7412,6 +7598,11 @@
           <t>She didn't single out curriculum elements she dislikes; pressed by Pat for 'the good and the bad,' her main friction was time/the block schedule and that the inductive-study markings and observations 'take a long time' to balance in 5th/6th grade.</t>
         </is>
       </c>
+      <c r="J39" s="16" t="inlineStr">
+        <is>
+          <t>They are wary of dull material and of mindless busywork — Angela Adams said they are 'careful about the word activity' because they don't want it to be a mindless activity, and Donna Hurley stressed Bible class should be engaging and 'not dull.'</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="16" t="inlineStr">
@@ -7449,6 +7640,11 @@
           <t>Discussion (her classes are discussion-heavy), acting out lessons, the reflection journal questions, drawing activities (e.g., 'benevolent wisdom'), maps and timelines, cartoon artwork, and short point-driven videos all hold her students' attention.</t>
         </is>
       </c>
+      <c r="J40" s="16" t="inlineStr">
+        <is>
+          <t>Skits and drama, object lessons, the philosophy chair, Post-it station rotations, review games like Kahoot, video clips, partner and table discussion, and anything that lets them move; the aim is an enjoyable, engaging, welcoming class that is never dull (Angela Adams and Donna Hurley).</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="16" t="inlineStr">
@@ -7488,6 +7684,11 @@
       <c r="I41" s="16" t="inlineStr">
         <is>
           <t>She effectively described DeepRoots as already easy to teach and impactful — she loves it and points to the short videos, the apologetics 'isms'/Mars Hill content, the reflection journals, and the well-balanced pages — with the one real need being adaptability to a block schedule so teachers covering Bible every other day can get through all the units.</t>
+        </is>
+      </c>
+      <c r="J41" s="16" t="inlineStr">
+        <is>
+          <t>Something they currently build entirely themselves, made ready-made. Internally they teach New Testament survey (6th, starting with the 400-year intertestamental period), Old Testament survey (7th), and wisdom books (8th), and they want a curriculum that adds apologetics and archaeological evidence, world-history timelines, vocabulary, geography, and strong application and reflection, plus engagement 'learning supports' with student choice, object lessons, and resource pointers. It should suit 80-minute blocks with movement, favor printables with occasional digital, use videos of three-plus minutes, and be enjoyable and engaging rather than dull — and requests must be budgeted early, before December, since the state budget does not cover Christian materials like Bible.</t>
         </is>
       </c>
     </row>
@@ -7501,6 +7702,7 @@
       <c r="G42" s="16" t="inlineStr"/>
       <c r="H42" s="16" t="inlineStr"/>
       <c r="I42" s="16" t="inlineStr"/>
+      <c r="J42" s="16" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
@@ -7516,6 +7718,7 @@
       <c r="G43" s="17" t="inlineStr"/>
       <c r="H43" s="17" t="inlineStr"/>
       <c r="I43" s="17" t="inlineStr"/>
+      <c r="J43" s="17" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="22" t="inlineStr"/>
@@ -7531,6 +7734,7 @@
       <c r="G44" s="22" t="inlineStr"/>
       <c r="H44" s="22" t="inlineStr"/>
       <c r="I44" s="22" t="inlineStr"/>
+      <c r="J44" s="22" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="18" t="inlineStr"/>
@@ -7568,6 +7772,11 @@
       <c r="I45" s="18" t="inlineStr">
         <is>
           <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
+        </is>
+      </c>
+      <c r="J45" s="18" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy (PA) — Donna Hurley + Angela Adams — 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -7589,6 +7798,7 @@
       <c r="G46" s="16" t="inlineStr"/>
       <c r="H46" s="16" t="inlineStr"/>
       <c r="I46" s="16" t="inlineStr"/>
+      <c r="J46" s="16" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="16" t="inlineStr"/>
@@ -7608,6 +7818,7 @@
       <c r="G47" s="16" t="inlineStr"/>
       <c r="H47" s="16" t="inlineStr"/>
       <c r="I47" s="16" t="inlineStr"/>
+      <c r="J47" s="16" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="16" t="inlineStr"/>
@@ -7627,6 +7838,7 @@
       <c r="G48" s="16" t="inlineStr"/>
       <c r="H48" s="16" t="inlineStr"/>
       <c r="I48" s="16" t="inlineStr"/>
+      <c r="J48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="16" t="inlineStr"/>
@@ -7646,6 +7858,7 @@
       <c r="G49" s="16" t="inlineStr"/>
       <c r="H49" s="16" t="inlineStr"/>
       <c r="I49" s="16" t="inlineStr"/>
+      <c r="J49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="16" t="inlineStr"/>
@@ -7665,6 +7878,7 @@
       <c r="G50" s="16" t="inlineStr"/>
       <c r="H50" s="16" t="inlineStr"/>
       <c r="I50" s="16" t="inlineStr"/>
+      <c r="J50" s="16" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="16" t="inlineStr"/>
@@ -7680,6 +7894,7 @@
       <c r="G51" s="16" t="inlineStr"/>
       <c r="H51" s="16" t="inlineStr"/>
       <c r="I51" s="16" t="inlineStr"/>
+      <c r="J51" s="16" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="16" t="inlineStr"/>
@@ -7691,6 +7906,7 @@
       <c r="G52" s="16" t="inlineStr"/>
       <c r="H52" s="16" t="inlineStr"/>
       <c r="I52" s="16" t="inlineStr"/>
+      <c r="J52" s="16" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="22" t="inlineStr"/>
@@ -7706,6 +7922,7 @@
       <c r="G53" s="22" t="inlineStr"/>
       <c r="H53" s="22" t="inlineStr"/>
       <c r="I53" s="22" t="inlineStr"/>
+      <c r="J53" s="22" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr"/>
@@ -7743,6 +7960,11 @@
       <c r="I54" s="18" t="inlineStr">
         <is>
           <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
+        </is>
+      </c>
+      <c r="J54" s="18" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy (PA) — Donna Hurley + Angela Adams — 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -7760,6 +7982,7 @@
       <c r="G55" s="16" t="inlineStr"/>
       <c r="H55" s="16" t="inlineStr"/>
       <c r="I55" s="16" t="inlineStr"/>
+      <c r="J55" s="16" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="16" t="inlineStr"/>
@@ -7775,6 +7998,7 @@
       <c r="G56" s="16" t="inlineStr"/>
       <c r="H56" s="16" t="inlineStr"/>
       <c r="I56" s="16" t="inlineStr"/>
+      <c r="J56" s="16" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="16" t="inlineStr"/>
@@ -7790,6 +8014,7 @@
       <c r="G57" s="16" t="inlineStr"/>
       <c r="H57" s="16" t="inlineStr"/>
       <c r="I57" s="16" t="inlineStr"/>
+      <c r="J57" s="16" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="16" t="inlineStr"/>
@@ -7805,6 +8030,7 @@
       <c r="G58" s="16" t="inlineStr"/>
       <c r="H58" s="16" t="inlineStr"/>
       <c r="I58" s="16" t="inlineStr"/>
+      <c r="J58" s="16" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="16" t="inlineStr"/>
@@ -7820,6 +8046,7 @@
       <c r="G59" s="16" t="inlineStr"/>
       <c r="H59" s="16" t="inlineStr"/>
       <c r="I59" s="16" t="inlineStr"/>
+      <c r="J59" s="16" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="16" t="inlineStr"/>
@@ -7835,6 +8062,7 @@
       <c r="G60" s="16" t="inlineStr"/>
       <c r="H60" s="16" t="inlineStr"/>
       <c r="I60" s="16" t="inlineStr"/>
+      <c r="J60" s="16" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="16" t="inlineStr"/>
@@ -7846,6 +8074,7 @@
       <c r="G61" s="16" t="inlineStr"/>
       <c r="H61" s="16" t="inlineStr"/>
       <c r="I61" s="16" t="inlineStr"/>
+      <c r="J61" s="16" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="22" t="inlineStr"/>
@@ -7861,6 +8090,7 @@
       <c r="G62" s="22" t="inlineStr"/>
       <c r="H62" s="22" t="inlineStr"/>
       <c r="I62" s="22" t="inlineStr"/>
+      <c r="J62" s="22" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="18" t="inlineStr"/>
@@ -7898,6 +8128,11 @@
       <c r="I63" s="18" t="inlineStr">
         <is>
           <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
+        </is>
+      </c>
+      <c r="J63" s="18" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy (PA) — Donna Hurley + Angela Adams — 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -7915,6 +8150,7 @@
       <c r="G64" s="16" t="inlineStr"/>
       <c r="H64" s="16" t="inlineStr"/>
       <c r="I64" s="16" t="inlineStr"/>
+      <c r="J64" s="16" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="16" t="inlineStr"/>
@@ -7930,6 +8166,7 @@
       <c r="G65" s="16" t="inlineStr"/>
       <c r="H65" s="16" t="inlineStr"/>
       <c r="I65" s="16" t="inlineStr"/>
+      <c r="J65" s="16" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="16" t="inlineStr"/>
@@ -7945,6 +8182,7 @@
       <c r="G66" s="16" t="inlineStr"/>
       <c r="H66" s="16" t="inlineStr"/>
       <c r="I66" s="16" t="inlineStr"/>
+      <c r="J66" s="16" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="16" t="inlineStr"/>
@@ -7960,6 +8198,7 @@
       <c r="G67" s="16" t="inlineStr"/>
       <c r="H67" s="16" t="inlineStr"/>
       <c r="I67" s="16" t="inlineStr"/>
+      <c r="J67" s="16" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="16" t="inlineStr"/>
@@ -7975,6 +8214,7 @@
       <c r="G68" s="16" t="inlineStr"/>
       <c r="H68" s="16" t="inlineStr"/>
       <c r="I68" s="16" t="inlineStr"/>
+      <c r="J68" s="16" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="16" t="inlineStr"/>
@@ -7990,6 +8230,7 @@
       <c r="G69" s="16" t="inlineStr"/>
       <c r="H69" s="16" t="inlineStr"/>
       <c r="I69" s="16" t="inlineStr"/>
+      <c r="J69" s="16" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="16" t="inlineStr"/>
@@ -8001,6 +8242,7 @@
       <c r="G70" s="16" t="inlineStr"/>
       <c r="H70" s="16" t="inlineStr"/>
       <c r="I70" s="16" t="inlineStr"/>
+      <c r="J70" s="16" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="22" t="inlineStr"/>
@@ -8016,6 +8258,7 @@
       <c r="G71" s="22" t="inlineStr"/>
       <c r="H71" s="22" t="inlineStr"/>
       <c r="I71" s="22" t="inlineStr"/>
+      <c r="J71" s="22" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="18" t="inlineStr"/>
@@ -8053,6 +8296,11 @@
       <c r="I72" s="18" t="inlineStr">
         <is>
           <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
+        </is>
+      </c>
+      <c r="J72" s="18" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy (PA) — Donna Hurley + Angela Adams — 2026-10-06</t>
         </is>
       </c>
     </row>
@@ -8070,6 +8318,7 @@
       <c r="G73" s="16" t="inlineStr"/>
       <c r="H73" s="16" t="inlineStr"/>
       <c r="I73" s="16" t="inlineStr"/>
+      <c r="J73" s="16" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="16" t="inlineStr"/>
@@ -8085,6 +8334,7 @@
       <c r="G74" s="16" t="inlineStr"/>
       <c r="H74" s="16" t="inlineStr"/>
       <c r="I74" s="16" t="inlineStr"/>
+      <c r="J74" s="16" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="16" t="inlineStr"/>
@@ -8100,6 +8350,7 @@
       <c r="G75" s="16" t="inlineStr"/>
       <c r="H75" s="16" t="inlineStr"/>
       <c r="I75" s="16" t="inlineStr"/>
+      <c r="J75" s="16" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="16" t="inlineStr"/>
@@ -8115,6 +8366,7 @@
       <c r="G76" s="16" t="inlineStr"/>
       <c r="H76" s="16" t="inlineStr"/>
       <c r="I76" s="16" t="inlineStr"/>
+      <c r="J76" s="16" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="16" t="inlineStr"/>
@@ -8130,6 +8382,7 @@
       <c r="G77" s="16" t="inlineStr"/>
       <c r="H77" s="16" t="inlineStr"/>
       <c r="I77" s="16" t="inlineStr"/>
+      <c r="J77" s="16" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="16" t="inlineStr"/>
@@ -8145,6 +8398,7 @@
       <c r="G78" s="16" t="inlineStr"/>
       <c r="H78" s="16" t="inlineStr"/>
       <c r="I78" s="16" t="inlineStr"/>
+      <c r="J78" s="16" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="16" t="inlineStr"/>
@@ -8156,6 +8410,143 @@
       <c r="G79" s="16" t="inlineStr"/>
       <c r="H79" s="16" t="inlineStr"/>
       <c r="I79" s="16" t="inlineStr"/>
+      <c r="J79" s="16" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="22" t="inlineStr"/>
+      <c r="B80" s="22" t="inlineStr"/>
+      <c r="C80" s="22" t="inlineStr">
+        <is>
+          <t>DAYSPRING interview — Dayspring Christian Academy (Donna Hurley + Angela Adams), 2026-10-06  |  Attendees: Troy Winkler, Lisa Van Vlear, Nancy Wood</t>
+        </is>
+      </c>
+      <c r="D80" s="22" t="inlineStr"/>
+      <c r="E80" s="22" t="inlineStr"/>
+      <c r="F80" s="22" t="inlineStr"/>
+      <c r="G80" s="22" t="inlineStr"/>
+      <c r="H80" s="22" t="inlineStr"/>
+      <c r="I80" s="22" t="inlineStr"/>
+      <c r="J80" s="22" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="18" t="inlineStr"/>
+      <c r="B81" s="18" t="inlineStr"/>
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>Team member</t>
+        </is>
+      </c>
+      <c r="D81" s="18" t="inlineStr">
+        <is>
+          <t>Meredith Arldt — Aliso Viejo Christian School (CA) — teacher/admin — 2026-09-24</t>
+        </is>
+      </c>
+      <c r="E81" s="18" t="inlineStr">
+        <is>
+          <t>Atlantic Shores Christian School (VA) — current K-5 use — 9/29/26</t>
+        </is>
+      </c>
+      <c r="F81" s="18" t="inlineStr">
+        <is>
+          <t>Will Weaver — Des Moines Christian School (IA) — Head of Spiritual Formation (admin) — 2026-09-30</t>
+        </is>
+      </c>
+      <c r="G81" s="18" t="inlineStr">
+        <is>
+          <t>Horizon Christian Elementary (OR) — current K-5 use — 9/28/26</t>
+        </is>
+      </c>
+      <c r="H81" s="18" t="inlineStr">
+        <is>
+          <t>Wendy Wagoner — Christian Academy of Indiana (IN) — Spiritual Life Coordinator — 2026-10-02</t>
+        </is>
+      </c>
+      <c r="I81" s="18" t="inlineStr">
+        <is>
+          <t>Ironbridge Christian Academy — Nicole Burchett + Crystal Thompson — 2026-10-05</t>
+        </is>
+      </c>
+      <c r="J81" s="18" t="inlineStr">
+        <is>
+          <t>Dayspring Christian Academy (PA) — Donna Hurley + Angela Adams — 2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="16" t="inlineStr"/>
+      <c r="B82" s="16" t="inlineStr"/>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>Troy Winkler</t>
+        </is>
+      </c>
+      <c r="D82" s="16" t="inlineStr"/>
+      <c r="E82" s="16" t="inlineStr"/>
+      <c r="F82" s="16" t="inlineStr"/>
+      <c r="G82" s="16" t="inlineStr"/>
+      <c r="H82" s="16" t="inlineStr"/>
+      <c r="I82" s="16" t="inlineStr"/>
+      <c r="J82" s="16" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="16" t="inlineStr"/>
+      <c r="B83" s="16" t="inlineStr"/>
+      <c r="C83" s="16" t="inlineStr">
+        <is>
+          <t>Lisa Van Vlear</t>
+        </is>
+      </c>
+      <c r="D83" s="16" t="inlineStr"/>
+      <c r="E83" s="16" t="inlineStr"/>
+      <c r="F83" s="16" t="inlineStr"/>
+      <c r="G83" s="16" t="inlineStr"/>
+      <c r="H83" s="16" t="inlineStr"/>
+      <c r="I83" s="16" t="inlineStr"/>
+      <c r="J83" s="16" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="16" t="inlineStr"/>
+      <c r="B84" s="16" t="inlineStr"/>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>Nancy Wood</t>
+        </is>
+      </c>
+      <c r="D84" s="16" t="inlineStr"/>
+      <c r="E84" s="16" t="inlineStr"/>
+      <c r="F84" s="16" t="inlineStr"/>
+      <c r="G84" s="16" t="inlineStr"/>
+      <c r="H84" s="16" t="inlineStr"/>
+      <c r="I84" s="16" t="inlineStr"/>
+      <c r="J84" s="16" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="16" t="inlineStr"/>
+      <c r="B85" s="16" t="inlineStr"/>
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>Overall / key takeaways for the curriculum</t>
+        </is>
+      </c>
+      <c r="D85" s="16" t="inlineStr"/>
+      <c r="E85" s="16" t="inlineStr"/>
+      <c r="F85" s="16" t="inlineStr"/>
+      <c r="G85" s="16" t="inlineStr"/>
+      <c r="H85" s="16" t="inlineStr"/>
+      <c r="I85" s="16" t="inlineStr"/>
+      <c r="J85" s="16" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="16" t="inlineStr"/>
+      <c r="B86" s="16" t="inlineStr"/>
+      <c r="C86" s="16" t="inlineStr"/>
+      <c r="D86" s="16" t="inlineStr"/>
+      <c r="E86" s="16" t="inlineStr"/>
+      <c r="F86" s="16" t="inlineStr"/>
+      <c r="G86" s="16" t="inlineStr"/>
+      <c r="H86" s="16" t="inlineStr"/>
+      <c r="I86" s="16" t="inlineStr"/>
+      <c r="J86" s="16" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Daily reply check 2026-10-12: Dayspring (Hurley) follow-ups, Wagoner written answers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X6pQ6fTNqhxfMHwzmkABoJ
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -5182,12 +5182,12 @@
       <c r="K136" s="5" t="n"/>
       <c r="L136" s="5" t="inlineStr">
         <is>
-          <t>BOOKED: Tue Oct 6 2026, 3:20 PM ET (30 min) - Google Meet invite sent; Angela Adams (Bible dept chair, aadams@dayspringchristian.com) joining - Donna asked Troy to send Angela her own invite (Troy said he would, 2026-09-30)</t>
+          <t>COMPLETED interview Tue Oct 6 2026, 3:20 PM ET (Donna Hurley + Angela Adams). Gr 6-8 curriculum guides received 2026-10-07.</t>
         </is>
       </c>
       <c r="M136" s="5" t="inlineStr">
         <is>
-          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up. | 2026-09-19: out of school recently; will check with Angela and follow up with times. | 2026-09-21: Donna replied "When would you like to schedule the call?" Troy proposed Thu Sep 24 3PM ET. Title confirmed: Director of Curriculum and Instruction, Dayspring. Awaiting confirm. | 2026-09-21: Sep 24 re-check reminder cancelled (Donna already scheduling). | 2026-09-29: Donna proposed Tue Oct 6 3:20 PM ET (Angela can join); Troy confirmed. Donna did not receive first invite; resent. | 2026-09-30: Donna found invite and responded; asked Troy to send Angela a separate invite - Troy replied he'd do so. Verify Angela's invite went out. Questions-preview email not yet sent.</t>
+          <t>Referred by Dee Henry (Dayspring). Troy engaged 2026-09-14. | Scheduling nudge sent 2026-09-17 (asked for times, offered to send questions ahead). | Replied 2026-09-19: apologized for delay (out of school more than usual), will check with Angela on whether she wants to take part, will respond soon. No times proposed yet. FLAG: send questions-preview email once she confirms/asks; no action needed until she follows up. | 2026-09-19: out of school recently; will check with Angela and follow up with times. | 2026-09-21: Donna replied "When would you like to schedule the call?" Troy proposed Thu Sep 24 3PM ET. Title confirmed: Director of Curriculum and Instruction, Dayspring. Awaiting confirm. | 2026-09-21: Sep 24 re-check reminder cancelled (Donna already scheduling). | 2026-09-29: Donna proposed Tue Oct 6 3:20 PM ET (Angela can join); Troy confirmed. Donna did not receive first invite; resent. | 2026-09-30: Donna found invite and responded; asked Troy to send Angela a separate invite - Troy replied he'd do so. Verify Angela's invite went out. Questions-preview email not yet sent. | 2026-10-06: Interview held (Donna + Angela Adams). Donna emailed same day: thanked Troy/team, praised Angela, and added that Dayspring is a Principle Approach school (students build handwritten notebooks of learning rather than disposable workbooks/fill-in-blank/multiple choice) - useful for curriculum design. Offered to send grades 6-8 Bible curriculum guides. | 2026-10-06: Troy sent thank-you. 2026-10-07: Troy accepted the guides; Donna sent Gr6 NT Survey, Gr7 OT Survey, Gr8 Wisdom Books curriculum guides (attached). No action needed unless team wants follow-up.</t>
         </is>
       </c>
     </row>
@@ -5312,12 +5312,12 @@
       </c>
       <c r="L138" s="5" t="inlineStr">
         <is>
-          <t>COMPLETED interview Fri Oct 2 2026, 3:00 PM ET (Pat Williamson ran it; Gemini notes + transcript). Answers: Interview Doc + Q&amp;A Sheet (Wendy Wagoner tab/column).</t>
+          <t>COMPLETED interview Fri Oct 2 2026, 3:00 PM ET (Pat Williamson ran it; Gemini notes + transcript). Answers: Interview Doc + Q&amp;A Sheet (Wendy Wagoner tab/column). Written answers received 2026-10-10 (Google Doc).</t>
         </is>
       </c>
       <c r="M138" s="5" t="inlineStr">
         <is>
-          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-21: drafted second nudge proposing a specific slot: Fri Sep 25 3:00 PM ET (her local, New Albany IN = Eastern). Grade level unconfirmed. Awaiting confirmation. | 2026-09-21: Troy handled live in Gmail. Wendy: received questions, cannot this week, might do next week. Troy: 3PM ET any day next week. Awaiting Wendy to name a day. | 2026-09-28: Wendy proposed Fri 3PM; Troy confirmed (cc Pat). 2026-09-29: Wendy confirmed she received the questions and is preparing for Friday. No action needed except confirm Pat's invite went out.</t>
+          <t>Round 1 contact; agreed 2026-09-16, questions sent 2026-09-16. | Scheduling nudge sent 2026-09-17 (asked for times). | 2026-09-21: drafted second nudge proposing a specific slot: Fri Sep 25 3:00 PM ET (her local, New Albany IN = Eastern). Grade level unconfirmed. Awaiting confirmation. | 2026-09-21: Troy handled live in Gmail. Wendy: received questions, cannot this week, might do next week. Troy: 3PM ET any day next week. Awaiting Wendy to name a day. | 2026-09-28: Wendy proposed Fri 3PM; Troy confirmed (cc Pat). 2026-09-29: Wendy confirmed she received the questions and is preparing for Friday. No action needed except confirm Pat's invite went out. | 2026-10-10: Wendy replied with written answers to the remaining questions (Google Doc 'Middle School Answers', brief notes in blue): https://docs.google.com/document/d/1xEJ1jUJ2mKhAdkitU5rbd84cMPQpYDU34sC7AF4EILc/edit - offered to clarify; cc Pat. Add to Interview Doc/Q&amp;A sheet. (Questions-preview email already sent; interview done.)</t>
         </is>
       </c>
       <c r="N138" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Daily reply check 2026-10-20: Studt (Concord), Kronberger, Morris, Thompson replies
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KdhZmMzf5FrmbdLkFq5bML
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -2879,6 +2879,36 @@
           <t>jstudt@concordchristianschool.org</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>NO for himself — redirected; Jen Studt (elementary) accepted Thu Oct 22 11:00 AM ET call, then on 2026-10-20 said she does not work with middle school and referred us to MS principal Steven Madonna (smadonna@concordcs.org) and MS asst. principal Danielle Turner (dturner@concordcs.org)</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Thu Oct 22 2026, 11:00 AM ET Meet jtv-sgjc-jsa (booked via check-in thread) — Jen says it would waste our time; likely cancel</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>2026-10-19: Replied to Oct 19 "How is your first quarter going?" check-in: happy to give feedback, loves DeepRoots; offered Thursday morning; Troy booked Thu Oct 22 11AM ET + sent questions doc. 2026-10-20: Jen says questions are MS-specific, she would waste our time; refers us to Steven Madonna (MS principal) and Danielle Turner (MS asst. principal) and will tell them to expect outreach. FLAG: decide whether to cancel Thu invite and email Madonna/Turner with the questions-preview email.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2997,6 +3027,26 @@
       <c r="F70" t="inlineStr">
         <is>
           <t>ckronberger@crosshillchristian.com</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>UNCLEAR — brief reply "Good here! Thanks, Troy!" (no response to interview ask; elementary principal)</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>2026-10-19: Replied to "How is your first quarter going?" check-in: "Good here! Thanks, Troy!" — no times or interest in interview. No action unless you want to follow up.</t>
         </is>
       </c>
     </row>
@@ -3762,6 +3812,26 @@
           <t>tmm@elkhartchristian.org</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>NO — no longer in role; redirected</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>2026-10-19: Tara Morris now Athletic Assistant; refers us to Kara Burch, new Elementary Assistant (KEB@elkhartchristian.org). FLAG: consider contacting Kara Burch.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -4225,6 +4295,26 @@
       <c r="F106" t="inlineStr">
         <is>
           <t>lthompson@foothillchristian.org</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>NO — uses own middle school materials; suggests other schools</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>2026-10-19: Linda Thompson (VP Curriculum &amp; Instruction): everything going well; Foothill uses own MS materials, other schools better for MS DeepRoots conversations. Declined politely.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: Concord MS principal (Madonna) declined
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011EYQ3sxQnYzCSY8twaYmq6
</commit_message>
<xml_diff>
--- a/outreach/DeepRoots_Round2_Response_Tracker.xlsx
+++ b/outreach/DeepRoots_Round2_Response_Tracker.xlsx
@@ -2891,7 +2891,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>NO for himself — redirected; Jen Studt (elementary) accepted Thu Oct 22 11:00 AM ET call, then on 2026-10-20 said she does not work with middle school and referred us to MS principal Steven Madonna (smadonna@concordcs.org) and MS asst. principal Danielle Turner (dturner@concordcs.org)</t>
+          <t>NO for himself — redirected; Jen Studt (elementary) accepted Thu Oct 22 11:00 AM ET call, then on 2026-10-20 said she does not work with middle school and referred us to MS principal Steven Madonna (smadonna@concordcs.org) and MS asst. principal Danielle Turner (dturner@concordcs.org) | Referral Steven Madonna (MS) declined 2026-10-21</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>2026-10-19: Replied to Oct 19 "How is your first quarter going?" check-in: happy to give feedback, loves DeepRoots; offered Thursday morning; Troy booked Thu Oct 22 11AM ET + sent questions doc. 2026-10-20: Jen says questions are MS-specific, she would waste our time; refers us to Steven Madonna (MS principal) and Danielle Turner (MS asst. principal) and will tell them to expect outreach. FLAG: decide whether to cancel Thu invite and email Madonna/Turner with the questions-preview email.</t>
+          <t>2026-10-19: Replied to Oct 19 "How is your first quarter going?" check-in: happy to give feedback, loves DeepRoots; offered Thursday morning; Troy booked Thu Oct 22 11AM ET + sent questions doc. 2026-10-20: Jen says questions are MS-specific, she would waste our time; refers us to Steven Madonna (MS principal) and Danielle Turner (MS asst. principal) and will tell them to expect outreach. FLAG: decide whether to cancel Thu invite and email Madonna/Turner with the questions-preview email. | 2026-10-21: Steven Madonna (MS principal, smadonna@concordchristianschool.org; cc Turner, P. Williamson) replied to the intro: DECLINED — "okay for this school year and next with the Bible curriculum." No interview; no questions-preview email needed. Dead end for Concord.</t>
         </is>
       </c>
     </row>

</xml_diff>